<commit_message>
Update both itinerary workbooks for 14:00 Jammu arrival on Day 1
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A4yYiJq592wzPacq5vAVkN
</commit_message>
<xml_diff>
--- a/docs/itineraries/vaishno-devi-helicopter-4d-plan.xlsx
+++ b/docs/itineraries/vaishno-devi-helicopter-4d-plan.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="693" uniqueCount="440">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="693" uniqueCount="441">
   <si>
     <t xml:space="preserve">Vaishno Devi Helicopter Yatra – Overview</t>
   </si>
@@ -100,7 +100,7 @@
     <t xml:space="preserve">Other transport: 2 helicopter flights (5–8 min each), Bhairon ropeway, ~5.5 km on the mountain track (2.5 km Day 2, ~3 km Day 3).</t>
   </si>
   <si>
-    <t xml:space="preserve">Assumptions: arrival at Jammu by 13:00 on Day 1; helicopter slots 10:30 (Day 2) and 11:00 (Day 3); one vehicle convoy for the group.</t>
+    <t xml:space="preserve">Assumptions: arrival at Jammu by 14:00 on Day 1; helicopter slots 10:30 (Day 2) and 11:00 (Day 3); one vehicle convoy for the group.</t>
   </si>
   <si>
     <t xml:space="preserve">4 Days Vaishno Devi Helicopter Package – Minute-to-Minute Plan</t>
@@ -139,7 +139,7 @@
     <t xml:space="preserve">On own – at home / origin airport / in flight</t>
   </si>
   <si>
-    <t xml:space="preserve">Breakfast on own before or during travel to Jammu (not included)</t>
+    <t xml:space="preserve">Breakfast on own before or during travel to Jammu (not included); carry a light snack, lunch is at 15:15</t>
   </si>
   <si>
     <t xml:space="preserve">Arrival</t>
@@ -181,7 +181,7 @@
     <t xml:space="preserve">Hotel restaurant, Jammu</t>
   </si>
   <si>
-    <t xml:space="preserve">Lunch – at the hotel, pre-ordered pure-veg thali so we leave on time; group pays</t>
+    <t xml:space="preserve">Late lunch – at the hotel, pre-ordered pure-veg thali served on arrival; group pays</t>
   </si>
   <si>
     <t xml:space="preserve">Raghunath Temple</t>
@@ -475,7 +475,7 @@
     <t xml:space="preserve">Not included</t>
   </si>
   <si>
-    <t xml:space="preserve">14:20–15:00</t>
+    <t xml:space="preserve">15:15–15:50</t>
   </si>
   <si>
     <t xml:space="preserve">Hotel, pre-ordered thali</t>
@@ -484,45 +484,48 @@
     <t xml:space="preserve">Group pays</t>
   </si>
   <si>
+    <t xml:space="preserve">20:15–21:15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hotel, pre-ordered menu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06:30–07:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hotel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Complimentary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12:15–13:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bhojanalaya, Bhawan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shrine Board (SMVDSB)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pay at counter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:30–20:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">07:00–07:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hotel restaurant, Katra (or pure-veg restaurant, Main Bazaar)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hotel / restaurant</t>
+  </si>
+  <si>
     <t xml:space="preserve">20:00–21:00</t>
   </si>
   <si>
-    <t xml:space="preserve">Hotel, pre-ordered menu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">06:30–07:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hotel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Complimentary</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12:15–13:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bhojanalaya, Bhawan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shrine Board (SMVDSB)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pay at counter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19:30–20:30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">07:00–07:30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hotel restaurant, Katra (or pure-veg restaurant, Main Bazaar)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hotel / restaurant</t>
-  </si>
-  <si>
     <t xml:space="preserve">07:00–07:40</t>
   </si>
   <si>
@@ -559,7 +562,7 @@
     <t xml:space="preserve">Uses arrival day well; five temples in 32 km</t>
   </si>
   <si>
-    <t xml:space="preserve">Afternoon-only window after a 13:00 arrival; little slack if flights are late</t>
+    <t xml:space="preserve">Afternoon-only window after a 14:00 arrival; little slack if flights are late</t>
   </si>
   <si>
     <t xml:space="preserve">Bhairon by ropeway</t>
@@ -886,7 +889,7 @@
     <t xml:space="preserve">T−45 days</t>
   </si>
   <si>
-    <t xml:space="preserve">Book flights / trains: arrival by 13:00 on Day 1; departure after 11:00 Day 4</t>
+    <t xml:space="preserve">Book flights / trains: arrival by 14:00 on Day 1; departure after 11:00 Day 4</t>
   </si>
   <si>
     <t xml:space="preserve">Travel desk</t>
@@ -1327,7 +1330,7 @@
     <t xml:space="preserve">Point to confirm</t>
   </si>
   <si>
-    <t xml:space="preserve">Every yatri's arrival in Jammu by 13:00 on Day 1, and departure flight / train times on Day 4</t>
+    <t xml:space="preserve">Every yatri's arrival in Jammu by 14:00 on Day 1, and departure flight / train times on Day 4</t>
   </si>
   <si>
     <t xml:space="preserve">Helicopter slots booked for Day 2 and Day 3 + reporting time</t>
@@ -2018,7 +2021,7 @@
       </c>
       <c r="G5" s="9" t="n">
         <f aca="false">_xlfn.MAXIFS('Minute-by-Minute'!$D$5:$D$60,'Minute-by-Minute'!$A$5:$A$60,A5)</f>
-        <v>0.875</v>
+        <v>0.885416666666667</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2149,121 +2152,121 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
     </row>
   </sheetData>
@@ -2293,74 +2296,74 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="C2" s="23"/>
       <c r="D2" s="23"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C3" s="23"/>
       <c r="D3" s="23"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="C4" s="23"/>
       <c r="D4" s="23"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="C5" s="23"/>
       <c r="D5" s="23"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="C6" s="23"/>
       <c r="D6" s="23"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="C7" s="23"/>
       <c r="D7" s="23"/>
@@ -2383,7 +2386,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B10" s="14"/>
       <c r="C10" s="23"/>
@@ -2391,7 +2394,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B11" s="14"/>
       <c r="C11" s="23"/>
@@ -2399,7 +2402,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="B12" s="14"/>
       <c r="C12" s="23"/>
@@ -2407,14 +2410,14 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="C13" s="14"/>
       <c r="D13" s="14" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
     </row>
   </sheetData>
@@ -2444,187 +2447,187 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D5" s="24"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="D6" s="24"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
+        <v>409</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>410</v>
+      </c>
+      <c r="C7" s="7" t="s">
         <v>408</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>409</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>407</v>
       </c>
       <c r="D7" s="24"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="D8" s="24"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="D9" s="24"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="D10" s="24"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="D11" s="24"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="D12" s="24"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="D13" s="24"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
+        <v>420</v>
+      </c>
+      <c r="B14" s="7" t="s">
         <v>419</v>
       </c>
-      <c r="B14" s="7" t="s">
-        <v>418</v>
-      </c>
       <c r="C14" s="7" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="D14" s="24"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="D15" s="24"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="D16" s="24"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="D17" s="24"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="D18" s="25" t="n">
         <f aca="false">SUMIF(C5:C17,"Yes",D5:D17)</f>
@@ -2633,10 +2636,10 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="D19" s="26" t="n">
         <v>0.05</v>
@@ -2644,7 +2647,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="D20" s="25" t="n">
         <f aca="false">D18*(1+D19)</f>
@@ -2653,7 +2656,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
     </row>
   </sheetData>
@@ -2681,69 +2684,69 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="B2" s="14"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="B3" s="14"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="B4" s="14"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B5" s="14"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="B6" s="14"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="B7" s="14"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="B8" s="14"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B9" s="14"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="B10" s="14"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="B11" s="14"/>
     </row>
@@ -2863,10 +2866,10 @@
         <v>46459</v>
       </c>
       <c r="C6" s="16" t="n">
-        <v>0.541666666666667</v>
+        <v>0.583333333333333</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>0.5625</v>
+        <v>0.604166666666667</v>
       </c>
       <c r="E6" s="14" t="n">
         <f aca="false">ROUND((D6-C6)*1440,0)</f>
@@ -2896,10 +2899,10 @@
         <v>46459</v>
       </c>
       <c r="C7" s="16" t="n">
-        <v>0.5625</v>
+        <v>0.604166666666667</v>
       </c>
       <c r="D7" s="16" t="n">
-        <v>0.576388888888889</v>
+        <v>0.618055555555556</v>
       </c>
       <c r="E7" s="14" t="n">
         <f aca="false">ROUND((D7-C7)*1440,0)</f>
@@ -2933,14 +2936,14 @@
         <v>46459</v>
       </c>
       <c r="C8" s="16" t="n">
-        <v>0.576388888888889</v>
+        <v>0.618055555555556</v>
       </c>
       <c r="D8" s="16" t="n">
-        <v>0.597222222222222</v>
+        <v>0.635416666666667</v>
       </c>
       <c r="E8" s="14" t="n">
         <f aca="false">ROUND((D8-C8)*1440,0)</f>
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F8" s="14" t="s">
         <v>43</v>
@@ -2966,14 +2969,14 @@
         <v>46459</v>
       </c>
       <c r="C9" s="13" t="n">
-        <v>0.597222222222222</v>
+        <v>0.635416666666667</v>
       </c>
       <c r="D9" s="13" t="n">
-        <v>0.625</v>
+        <v>0.659722222222222</v>
       </c>
       <c r="E9" s="11" t="n">
         <f aca="false">ROUND((D9-C9)*1440,0)</f>
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="F9" s="11" t="s">
         <v>46</v>
@@ -2999,10 +3002,10 @@
         <v>46459</v>
       </c>
       <c r="C10" s="16" t="n">
-        <v>0.625</v>
+        <v>0.659722222222222</v>
       </c>
       <c r="D10" s="16" t="n">
-        <v>0.635416666666667</v>
+        <v>0.670138888888889</v>
       </c>
       <c r="E10" s="14" t="n">
         <f aca="false">ROUND((D10-C10)*1440,0)</f>
@@ -3036,14 +3039,14 @@
         <v>46459</v>
       </c>
       <c r="C11" s="16" t="n">
-        <v>0.635416666666667</v>
+        <v>0.670138888888889</v>
       </c>
       <c r="D11" s="16" t="n">
-        <v>0.666666666666667</v>
+        <v>0.697916666666667</v>
       </c>
       <c r="E11" s="14" t="n">
         <f aca="false">ROUND((D11-C11)*1440,0)</f>
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="F11" s="14" t="s">
         <v>51</v>
@@ -3069,10 +3072,10 @@
         <v>46459</v>
       </c>
       <c r="C12" s="16" t="n">
-        <v>0.666666666666667</v>
+        <v>0.697916666666667</v>
       </c>
       <c r="D12" s="16" t="n">
-        <v>0.673611111111111</v>
+        <v>0.704861111111111</v>
       </c>
       <c r="E12" s="14" t="n">
         <f aca="false">ROUND((D12-C12)*1440,0)</f>
@@ -3106,14 +3109,14 @@
         <v>46459</v>
       </c>
       <c r="C13" s="16" t="n">
-        <v>0.673611111111111</v>
+        <v>0.704861111111111</v>
       </c>
       <c r="D13" s="16" t="n">
-        <v>0.694444444444444</v>
+        <v>0.722222222222222</v>
       </c>
       <c r="E13" s="14" t="n">
         <f aca="false">ROUND((D13-C13)*1440,0)</f>
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F13" s="14" t="s">
         <v>51</v>
@@ -3139,10 +3142,10 @@
         <v>46459</v>
       </c>
       <c r="C14" s="16" t="n">
-        <v>0.694444444444444</v>
+        <v>0.722222222222222</v>
       </c>
       <c r="D14" s="16" t="n">
-        <v>0.708333333333333</v>
+        <v>0.736111111111111</v>
       </c>
       <c r="E14" s="14" t="n">
         <f aca="false">ROUND((D14-C14)*1440,0)</f>
@@ -3176,14 +3179,14 @@
         <v>46459</v>
       </c>
       <c r="C15" s="16" t="n">
-        <v>0.708333333333333</v>
+        <v>0.736111111111111</v>
       </c>
       <c r="D15" s="16" t="n">
-        <v>0.75</v>
+        <v>0.770833333333333</v>
       </c>
       <c r="E15" s="14" t="n">
         <f aca="false">ROUND((D15-C15)*1440,0)</f>
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="F15" s="14" t="s">
         <v>51</v>
@@ -3209,10 +3212,10 @@
         <v>46459</v>
       </c>
       <c r="C16" s="16" t="n">
-        <v>0.75</v>
+        <v>0.770833333333333</v>
       </c>
       <c r="D16" s="16" t="n">
-        <v>0.767361111111111</v>
+        <v>0.788194444444444</v>
       </c>
       <c r="E16" s="14" t="n">
         <f aca="false">ROUND((D16-C16)*1440,0)</f>
@@ -3246,10 +3249,10 @@
         <v>46459</v>
       </c>
       <c r="C17" s="16" t="n">
-        <v>0.767361111111111</v>
+        <v>0.788194444444444</v>
       </c>
       <c r="D17" s="16" t="n">
-        <v>0.791666666666667</v>
+        <v>0.8125</v>
       </c>
       <c r="E17" s="14" t="n">
         <f aca="false">ROUND((D17-C17)*1440,0)</f>
@@ -3279,10 +3282,10 @@
         <v>46459</v>
       </c>
       <c r="C18" s="16" t="n">
-        <v>0.791666666666667</v>
+        <v>0.8125</v>
       </c>
       <c r="D18" s="16" t="n">
-        <v>0.805555555555556</v>
+        <v>0.826388888888889</v>
       </c>
       <c r="E18" s="14" t="n">
         <f aca="false">ROUND((D18-C18)*1440,0)</f>
@@ -3316,14 +3319,14 @@
         <v>46459</v>
       </c>
       <c r="C19" s="16" t="n">
-        <v>0.805555555555556</v>
+        <v>0.826388888888889</v>
       </c>
       <c r="D19" s="16" t="n">
-        <v>0.833333333333333</v>
+        <v>0.84375</v>
       </c>
       <c r="E19" s="14" t="n">
         <f aca="false">ROUND((D19-C19)*1440,0)</f>
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="F19" s="14" t="s">
         <v>43</v>
@@ -3349,10 +3352,10 @@
         <v>46459</v>
       </c>
       <c r="C20" s="13" t="n">
-        <v>0.833333333333333</v>
+        <v>0.84375</v>
       </c>
       <c r="D20" s="13" t="n">
-        <v>0.875</v>
+        <v>0.885416666666667</v>
       </c>
       <c r="E20" s="11" t="n">
         <f aca="false">ROUND((D20-C20)*1440,0)</f>
@@ -5021,7 +5024,7 @@
         <v>66</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
       <c r="D12" s="14" t="s">
         <v>127</v>
@@ -5041,7 +5044,7 @@
         <v>32</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D13" s="14" t="s">
         <v>127</v>
@@ -5064,7 +5067,7 @@
         <v>18</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E14" s="14" t="s">
         <v>152</v>
@@ -5098,13 +5101,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5112,76 +5115,76 @@
         <v>79</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
   </sheetData>
@@ -5211,184 +5214,184 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
   </sheetData>
@@ -5416,202 +5419,202 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="14" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="14" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="14" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="14" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="14" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="14" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="14" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B25" s="14" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
   </sheetData>
@@ -5641,188 +5644,188 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D4" s="23"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B5" s="14" t="s">
+        <v>278</v>
+      </c>
+      <c r="C5" s="14" t="s">
         <v>277</v>
-      </c>
-      <c r="C5" s="14" t="s">
-        <v>276</v>
       </c>
       <c r="D5" s="23"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D6" s="23"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D7" s="23"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D8" s="23"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D9" s="23"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B10" s="14" t="s">
+        <v>286</v>
+      </c>
+      <c r="C10" s="14" t="s">
         <v>285</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>284</v>
       </c>
       <c r="D10" s="23"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D11" s="23"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D12" s="23"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D13" s="23"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D14" s="23"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D15" s="23"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D16" s="23"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D17" s="23"/>
     </row>
@@ -5851,146 +5854,146 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
     </row>
   </sheetData>
@@ -6018,34 +6021,34 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6053,55 +6056,55 @@
         <v>79</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add registration and booking deadlines
Registrations close 25 Dec 2026, yatri data to the travel agent on
30 Dec 2026, helicopter tickets booked on 1 Jan 2027. Added to both
workbooks' checklists and overview, and the closing date to the
brochures and posters.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A4yYiJq592wzPacq5vAVkN
</commit_message>
<xml_diff>
--- a/docs/itineraries/vaishno-devi-helicopter-4d-plan.xlsx
+++ b/docs/itineraries/vaishno-devi-helicopter-4d-plan.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="693" uniqueCount="441">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="703" uniqueCount="453">
   <si>
     <t xml:space="preserve">Vaishno Devi Helicopter Yatra – Overview</t>
   </si>
@@ -49,6 +49,9 @@
     <t xml:space="preserve">← change this date and every day / row date updates</t>
   </si>
   <si>
+    <t xml:space="preserve">Key dates</t>
+  </si>
+  <si>
     <t xml:space="preserve">Day</t>
   </si>
   <si>
@@ -70,18 +73,27 @@
     <t xml:space="preserve">Last end</t>
   </si>
   <si>
+    <t xml:space="preserve">Registrations close</t>
+  </si>
+  <si>
     <t xml:space="preserve">Jammu arrival, Jammu temples</t>
   </si>
   <si>
     <t xml:space="preserve">Jammu</t>
   </si>
   <si>
+    <t xml:space="preserve">Yatri data to travel agent</t>
+  </si>
+  <si>
     <t xml:space="preserve">Jammu → Katra → Sanjichhat (helicopter) → Bhawan</t>
   </si>
   <si>
     <t xml:space="preserve">Bhawan</t>
   </si>
   <si>
+    <t xml:space="preserve">Helicopter tickets booked</t>
+  </si>
+  <si>
     <t xml:space="preserve">Bhawan → Bhairon → Sanjichhat (helicopter) → Katra</t>
   </si>
   <si>
@@ -859,6 +871,9 @@
     <t xml:space="preserve">Owner</t>
   </si>
   <si>
+    <t xml:space="preserve">Notes</t>
+  </si>
+  <si>
     <t xml:space="preserve">Status (fill in)</t>
   </si>
   <si>
@@ -871,15 +886,36 @@
     <t xml:space="preserve">Yatra coordinator</t>
   </si>
   <si>
-    <t xml:space="preserve">Collect yatri names, photo ID, age, phone, emergency contact, medical notes</t>
+    <t xml:space="preserve">By 25 Dec 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Registrations close: collect yatri names, photo ID (Aadhaar / passport), age, weight, phone, emergency contact, medical notes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Last date 25 Dec 2026; name exactly as on ID; weight needed for the helicopter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30 Dec 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Send complete yatri data to the travel agent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Names as on ID, ID numbers, ages, weights, phone numbers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Jan 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Book helicopter Day 2 &amp; Day 3 on SMVDSB portal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Travel agent with yatra coordinator</t>
   </si>
   <si>
     <t xml:space="preserve">Booking opening day</t>
   </si>
   <si>
-    <t xml:space="preserve">Book helicopter Day 2 &amp; Day 3 on SMVDSB portal</t>
-  </si>
-  <si>
     <t xml:space="preserve">Book Bhawan accommodation Day 2 night</t>
   </si>
   <si>
@@ -1333,7 +1369,7 @@
     <t xml:space="preserve">Every yatri's arrival in Jammu by 14:00 on Day 1, and departure flight / train times on Day 4</t>
   </si>
   <si>
-    <t xml:space="preserve">Helicopter slots booked for Day 2 and Day 3 + reporting time</t>
+    <t xml:space="preserve">Helicopter slots booked on 1 Jan 2027 for Day 2 and Day 3 + reporting time</t>
   </si>
   <si>
     <t xml:space="preserve">Helicopter baggage limit per yatri; where main luggage waits</t>
@@ -1942,7 +1978,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -1951,6 +1987,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="17"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1973,28 +2011,37 @@
       <c r="C3" s="5" t="s">
         <v>3</v>
       </c>
+      <c r="I3" s="3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="J4" s="8" t="n">
+        <v>46381</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2006,14 +2053,14 @@
         <v>46459</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D5" s="7" t="n">
         <f aca="false">SUMIF('Minute-by-Minute'!$A$5:$A$60,A5,'Minute-by-Minute'!$I$5:$I$60)</f>
         <v>32</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F5" s="9" t="n">
         <f aca="false">_xlfn.MINIFS('Minute-by-Minute'!$C$5:$C$60,'Minute-by-Minute'!$A$5:$A$60,A5)</f>
@@ -2023,6 +2070,12 @@
         <f aca="false">_xlfn.MAXIFS('Minute-by-Minute'!$D$5:$D$60,'Minute-by-Minute'!$A$5:$A$60,A5)</f>
         <v>0.885416666666667</v>
       </c>
+      <c r="I5" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="J5" s="8" t="n">
+        <v>46386</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="n">
@@ -2033,14 +2086,14 @@
         <v>46460</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D6" s="7" t="n">
         <f aca="false">SUMIF('Minute-by-Minute'!$A$5:$A$60,A6,'Minute-by-Minute'!$I$5:$I$60)</f>
         <v>52</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F6" s="9" t="n">
         <f aca="false">_xlfn.MINIFS('Minute-by-Minute'!$C$5:$C$60,'Minute-by-Minute'!$A$5:$A$60,A6)</f>
@@ -2050,6 +2103,12 @@
         <f aca="false">_xlfn.MAXIFS('Minute-by-Minute'!$D$5:$D$60,'Minute-by-Minute'!$A$5:$A$60,A6)</f>
         <v>0.854166666666667</v>
       </c>
+      <c r="I6" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="J6" s="8" t="n">
+        <v>46388</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="n">
@@ -2060,14 +2119,14 @@
         <v>46461</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D7" s="7" t="n">
         <f aca="false">SUMIF('Minute-by-Minute'!$A$5:$A$60,A7,'Minute-by-Minute'!$I$5:$I$60)</f>
         <v>9</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="F7" s="9" t="n">
         <f aca="false">_xlfn.MINIFS('Minute-by-Minute'!$C$5:$C$60,'Minute-by-Minute'!$A$5:$A$60,A7)</f>
@@ -2087,14 +2146,14 @@
         <v>46462</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="D8" s="7" t="n">
         <f aca="false">SUMIF('Minute-by-Minute'!$A$5:$A$60,A8,'Minute-by-Minute'!$I$5:$I$60)</f>
         <v>50</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F8" s="9" t="n">
         <f aca="false">_xlfn.MINIFS('Minute-by-Minute'!$C$5:$C$60,'Minute-by-Minute'!$A$5:$A$60,A8)</f>
@@ -2107,7 +2166,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="D9" s="3" t="n">
         <f aca="false">SUM(D5:D8)</f>
@@ -2116,12 +2175,12 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -2152,121 +2211,121 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>347</v>
+        <v>359</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>348</v>
+        <v>360</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>349</v>
+        <v>361</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>350</v>
+        <v>362</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>351</v>
+        <v>363</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>352</v>
+        <v>364</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>353</v>
+        <v>365</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>354</v>
+        <v>366</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>355</v>
+        <v>367</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>356</v>
+        <v>368</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>357</v>
+        <v>369</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>358</v>
+        <v>370</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>359</v>
+        <v>371</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>360</v>
+        <v>372</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>361</v>
+        <v>373</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>362</v>
+        <v>374</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>363</v>
+        <v>375</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>364</v>
+        <v>376</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>365</v>
+        <v>377</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>366</v>
+        <v>378</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>367</v>
+        <v>379</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>368</v>
+        <v>380</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>369</v>
+        <v>381</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>324</v>
+        <v>336</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>370</v>
+        <v>382</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>371</v>
+        <v>383</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>355</v>
+        <v>367</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>318</v>
+        <v>330</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>372</v>
+        <v>384</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>373</v>
+        <v>385</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>374</v>
+        <v>386</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>375</v>
+        <v>387</v>
       </c>
     </row>
   </sheetData>
@@ -2296,81 +2355,81 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>377</v>
+        <v>389</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>378</v>
+        <v>390</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>379</v>
+        <v>391</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>291</v>
+        <v>303</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>380</v>
+        <v>392</v>
       </c>
       <c r="C2" s="23"/>
       <c r="D2" s="23"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>381</v>
+        <v>393</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>382</v>
+        <v>394</v>
       </c>
       <c r="C3" s="23"/>
       <c r="D3" s="23"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>383</v>
+        <v>395</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>384</v>
+        <v>396</v>
       </c>
       <c r="C4" s="23"/>
       <c r="D4" s="23"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>385</v>
+        <v>397</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>386</v>
+        <v>398</v>
       </c>
       <c r="C5" s="23"/>
       <c r="D5" s="23"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>387</v>
+        <v>399</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>388</v>
+        <v>400</v>
       </c>
       <c r="C6" s="23"/>
       <c r="D6" s="23"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>389</v>
+        <v>401</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>390</v>
+        <v>402</v>
       </c>
       <c r="C7" s="23"/>
       <c r="D7" s="23"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B8" s="14"/>
       <c r="C8" s="23"/>
@@ -2378,7 +2437,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="B9" s="14"/>
       <c r="C9" s="23"/>
@@ -2386,7 +2445,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>391</v>
+        <v>403</v>
       </c>
       <c r="B10" s="14"/>
       <c r="C10" s="23"/>
@@ -2394,7 +2453,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>392</v>
+        <v>404</v>
       </c>
       <c r="B11" s="14"/>
       <c r="C11" s="23"/>
@@ -2402,7 +2461,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>393</v>
+        <v>405</v>
       </c>
       <c r="B12" s="14"/>
       <c r="C12" s="23"/>
@@ -2410,14 +2469,14 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>394</v>
+        <v>406</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>395</v>
+        <v>407</v>
       </c>
       <c r="C13" s="14"/>
       <c r="D13" s="14" t="s">
-        <v>396</v>
+        <v>408</v>
       </c>
     </row>
   </sheetData>
@@ -2447,187 +2506,187 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>397</v>
+        <v>409</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>398</v>
+        <v>410</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>399</v>
+        <v>411</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>400</v>
+        <v>412</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>401</v>
+        <v>413</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>402</v>
+        <v>414</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>403</v>
+        <v>415</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>404</v>
+        <v>416</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>405</v>
+        <v>417</v>
       </c>
       <c r="D5" s="24"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>406</v>
+        <v>418</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>407</v>
+        <v>419</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>408</v>
+        <v>420</v>
       </c>
       <c r="D6" s="24"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>409</v>
+        <v>421</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>410</v>
+        <v>422</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>408</v>
+        <v>420</v>
       </c>
       <c r="D7" s="24"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>411</v>
+        <v>423</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>407</v>
+        <v>419</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>408</v>
+        <v>420</v>
       </c>
       <c r="D8" s="24"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>412</v>
+        <v>424</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>413</v>
+        <v>425</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>408</v>
+        <v>420</v>
       </c>
       <c r="D9" s="24"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>414</v>
+        <v>426</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>404</v>
+        <v>416</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>408</v>
+        <v>420</v>
       </c>
       <c r="D10" s="24"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>415</v>
+        <v>427</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>404</v>
+        <v>416</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>408</v>
+        <v>420</v>
       </c>
       <c r="D11" s="24"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>416</v>
+        <v>428</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>417</v>
+        <v>429</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>408</v>
+        <v>420</v>
       </c>
       <c r="D12" s="24"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>418</v>
+        <v>430</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>419</v>
+        <v>431</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>408</v>
+        <v>420</v>
       </c>
       <c r="D13" s="24"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
+        <v>432</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>431</v>
+      </c>
+      <c r="C14" s="7" t="s">
         <v>420</v>
-      </c>
-      <c r="B14" s="7" t="s">
-        <v>419</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>408</v>
       </c>
       <c r="D14" s="24"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>421</v>
+        <v>433</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>419</v>
+        <v>431</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>408</v>
+        <v>420</v>
       </c>
       <c r="D15" s="24"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>422</v>
+        <v>434</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>404</v>
+        <v>416</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>408</v>
+        <v>420</v>
       </c>
       <c r="D16" s="24"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>423</v>
+        <v>435</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>424</v>
+        <v>436</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>408</v>
+        <v>420</v>
       </c>
       <c r="D17" s="24"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>425</v>
+        <v>437</v>
       </c>
       <c r="D18" s="25" t="n">
         <f aca="false">SUMIF(C5:C17,"Yes",D5:D17)</f>
@@ -2636,10 +2695,10 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>426</v>
+        <v>438</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>427</v>
+        <v>439</v>
       </c>
       <c r="D19" s="26" t="n">
         <v>0.05</v>
@@ -2647,7 +2706,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>428</v>
+        <v>440</v>
       </c>
       <c r="D20" s="25" t="n">
         <f aca="false">D18*(1+D19)</f>
@@ -2656,7 +2715,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>429</v>
+        <v>441</v>
       </c>
     </row>
   </sheetData>
@@ -2684,69 +2743,69 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>430</v>
+        <v>442</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>431</v>
+        <v>443</v>
       </c>
       <c r="B2" s="14"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>432</v>
+        <v>444</v>
       </c>
       <c r="B3" s="14"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>433</v>
+        <v>445</v>
       </c>
       <c r="B4" s="14"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>434</v>
+        <v>446</v>
       </c>
       <c r="B5" s="14"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>435</v>
+        <v>447</v>
       </c>
       <c r="B6" s="14"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>436</v>
+        <v>448</v>
       </c>
       <c r="B7" s="14"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>437</v>
+        <v>449</v>
       </c>
       <c r="B8" s="14"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>438</v>
+        <v>450</v>
       </c>
       <c r="B9" s="14"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>439</v>
+        <v>451</v>
       </c>
       <c r="B10" s="14"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>440</v>
+        <v>452</v>
       </c>
       <c r="B11" s="14"/>
     </row>
@@ -2783,47 +2842,47 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J4" s="10" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="K4" s="10" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2845,15 +2904,15 @@
         <v>30</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="G5" s="11" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H5" s="11"/>
       <c r="I5" s="11"/>
       <c r="J5" s="11" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="K5" s="11"/>
     </row>
@@ -2876,18 +2935,18 @@
         <v>30</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="G6" s="14" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="H6" s="14"/>
       <c r="I6" s="14"/>
       <c r="J6" s="14" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="K6" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2909,22 +2968,22 @@
         <v>20</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="H7" s="14" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="I7" s="14" t="n">
         <v>7</v>
       </c>
       <c r="J7" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="K7" s="17" t="s">
         <v>42</v>
-      </c>
-      <c r="K7" s="17" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2946,18 +3005,18 @@
         <v>25</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="G8" s="14" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="H8" s="14"/>
       <c r="I8" s="14"/>
       <c r="J8" s="14" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="K8" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2979,18 +3038,18 @@
         <v>35</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="G9" s="11" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="H9" s="11"/>
       <c r="I9" s="11"/>
       <c r="J9" s="11" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="K9" s="18" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3012,22 +3071,22 @@
         <v>15</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="G10" s="14" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="H10" s="14" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="I10" s="14" t="n">
         <v>5</v>
       </c>
       <c r="J10" s="14" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="K10" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3049,18 +3108,18 @@
         <v>40</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="G11" s="14" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="H11" s="14"/>
       <c r="I11" s="14"/>
       <c r="J11" s="14" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="K11" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3082,22 +3141,22 @@
         <v>10</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="G12" s="14" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="H12" s="14" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="I12" s="14" t="n">
         <v>1</v>
       </c>
       <c r="J12" s="14" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="K12" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3119,18 +3178,18 @@
         <v>25</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="G13" s="14" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="H13" s="14"/>
       <c r="I13" s="14"/>
       <c r="J13" s="14" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="K13" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3152,22 +3211,22 @@
         <v>20</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="G14" s="14" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="H14" s="14" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="I14" s="14" t="n">
         <v>6</v>
       </c>
       <c r="J14" s="14" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="K14" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3189,18 +3248,18 @@
         <v>50</v>
       </c>
       <c r="F15" s="14" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="G15" s="14" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="H15" s="14"/>
       <c r="I15" s="14"/>
       <c r="J15" s="14" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="K15" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3222,22 +3281,22 @@
         <v>25</v>
       </c>
       <c r="F16" s="14" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="G16" s="14" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="H16" s="14" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="I16" s="14" t="n">
         <v>7</v>
       </c>
       <c r="J16" s="14" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="K16" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3259,18 +3318,18 @@
         <v>35</v>
       </c>
       <c r="F17" s="14" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="G17" s="14" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="H17" s="14"/>
       <c r="I17" s="14"/>
       <c r="J17" s="14" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="K17" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3292,22 +3351,22 @@
         <v>20</v>
       </c>
       <c r="F18" s="14" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="G18" s="14" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="H18" s="14" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="I18" s="14" t="n">
         <v>6</v>
       </c>
       <c r="J18" s="14" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="K18" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3329,18 +3388,18 @@
         <v>25</v>
       </c>
       <c r="F19" s="14" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="G19" s="14" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="H19" s="14"/>
       <c r="I19" s="14"/>
       <c r="J19" s="14" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="K19" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3362,18 +3421,18 @@
         <v>60</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="G20" s="11" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="H20" s="11"/>
       <c r="I20" s="11"/>
       <c r="J20" s="11" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="K20" s="18" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3395,18 +3454,18 @@
         <v>30</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="G21" s="11" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="H21" s="11"/>
       <c r="I21" s="11"/>
       <c r="J21" s="11" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="K21" s="18" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3428,18 +3487,18 @@
         <v>15</v>
       </c>
       <c r="F22" s="14" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="G22" s="14" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="H22" s="14"/>
       <c r="I22" s="14"/>
       <c r="J22" s="14" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="K22" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3461,22 +3520,22 @@
         <v>90</v>
       </c>
       <c r="F23" s="14" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="G23" s="14" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="H23" s="14" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="I23" s="14" t="n">
         <v>50</v>
       </c>
       <c r="J23" s="14" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="K23" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3498,18 +3557,18 @@
         <v>30</v>
       </c>
       <c r="F24" s="14" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="G24" s="14" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="H24" s="14"/>
       <c r="I24" s="14"/>
       <c r="J24" s="14" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="K24" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3531,22 +3590,22 @@
         <v>10</v>
       </c>
       <c r="F25" s="14" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="G25" s="14" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="H25" s="14" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="I25" s="14" t="n">
         <v>2</v>
       </c>
       <c r="J25" s="14" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="K25" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3568,18 +3627,18 @@
         <v>65</v>
       </c>
       <c r="F26" s="14" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="G26" s="14" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="H26" s="14"/>
       <c r="I26" s="14"/>
       <c r="J26" s="14" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="K26" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3601,20 +3660,20 @@
         <v>10</v>
       </c>
       <c r="F27" s="19" t="s">
+        <v>83</v>
+      </c>
+      <c r="G27" s="19" t="s">
         <v>79</v>
       </c>
-      <c r="G27" s="19" t="s">
-        <v>75</v>
-      </c>
       <c r="H27" s="19" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="I27" s="19"/>
       <c r="J27" s="19" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="K27" s="22" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3636,20 +3695,20 @@
         <v>65</v>
       </c>
       <c r="F28" s="14" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="G28" s="14" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="H28" s="14" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="I28" s="14"/>
       <c r="J28" s="14" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="K28" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3671,18 +3730,18 @@
         <v>30</v>
       </c>
       <c r="F29" s="14" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="G29" s="14" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="H29" s="14"/>
       <c r="I29" s="14"/>
       <c r="J29" s="14" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="K29" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3704,18 +3763,18 @@
         <v>45</v>
       </c>
       <c r="F30" s="11" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="G30" s="11" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="H30" s="11"/>
       <c r="I30" s="11"/>
       <c r="J30" s="11" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="K30" s="18" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3737,18 +3796,18 @@
         <v>210</v>
       </c>
       <c r="F31" s="14" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="G31" s="14" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="H31" s="14"/>
       <c r="I31" s="14"/>
       <c r="J31" s="14" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="K31" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3770,18 +3829,18 @@
         <v>90</v>
       </c>
       <c r="F32" s="14" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="G32" s="14" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="H32" s="14"/>
       <c r="I32" s="14"/>
       <c r="J32" s="14" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="K32" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3803,18 +3862,18 @@
         <v>90</v>
       </c>
       <c r="F33" s="14" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="G33" s="14" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="H33" s="14"/>
       <c r="I33" s="14"/>
       <c r="J33" s="14" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="K33" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3836,18 +3895,18 @@
         <v>60</v>
       </c>
       <c r="F34" s="11" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="G34" s="11" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="H34" s="11"/>
       <c r="I34" s="11"/>
       <c r="J34" s="11" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="K34" s="18" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3869,18 +3928,18 @@
         <v>60</v>
       </c>
       <c r="F35" s="14" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="G35" s="14" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="H35" s="14"/>
       <c r="I35" s="14"/>
       <c r="J35" s="14" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="K35" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3902,18 +3961,18 @@
         <v>90</v>
       </c>
       <c r="F36" s="14" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="G36" s="14" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="H36" s="14"/>
       <c r="I36" s="14"/>
       <c r="J36" s="14" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="K36" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3935,18 +3994,18 @@
         <v>30</v>
       </c>
       <c r="F37" s="11" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="G37" s="11" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="H37" s="11"/>
       <c r="I37" s="11"/>
       <c r="J37" s="11" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="K37" s="18" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3968,18 +4027,18 @@
         <v>15</v>
       </c>
       <c r="F38" s="14" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="G38" s="14" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="H38" s="14"/>
       <c r="I38" s="14"/>
       <c r="J38" s="14" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="K38" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4001,20 +4060,20 @@
         <v>15</v>
       </c>
       <c r="F39" s="14" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="G39" s="14" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="H39" s="14" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="I39" s="14"/>
       <c r="J39" s="14" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="K39" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4036,20 +4095,20 @@
         <v>20</v>
       </c>
       <c r="F40" s="19" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="G40" s="19" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="H40" s="19" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="I40" s="19"/>
       <c r="J40" s="19" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="K40" s="22" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4071,18 +4130,18 @@
         <v>40</v>
       </c>
       <c r="F41" s="14" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="G41" s="14" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="H41" s="14"/>
       <c r="I41" s="14"/>
       <c r="J41" s="14" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="K41" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4104,20 +4163,20 @@
         <v>60</v>
       </c>
       <c r="F42" s="14" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="G42" s="14" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="H42" s="14" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="I42" s="14"/>
       <c r="J42" s="14" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="K42" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4139,18 +4198,18 @@
         <v>60</v>
       </c>
       <c r="F43" s="14" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="G43" s="14" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="H43" s="14"/>
       <c r="I43" s="14"/>
       <c r="J43" s="14" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="K43" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4172,20 +4231,20 @@
         <v>10</v>
       </c>
       <c r="F44" s="19" t="s">
+        <v>83</v>
+      </c>
+      <c r="G44" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="H44" s="19" t="s">
         <v>79</v>
-      </c>
-      <c r="G44" s="19" t="s">
-        <v>80</v>
-      </c>
-      <c r="H44" s="19" t="s">
-        <v>75</v>
       </c>
       <c r="I44" s="19"/>
       <c r="J44" s="19" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="K44" s="22" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4207,22 +4266,22 @@
         <v>15</v>
       </c>
       <c r="F45" s="14" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="G45" s="14" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="H45" s="14" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="I45" s="14" t="n">
         <v>2</v>
       </c>
       <c r="J45" s="14" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="K45" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4244,18 +4303,18 @@
         <v>50</v>
       </c>
       <c r="F46" s="14" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="G46" s="14" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="H46" s="14"/>
       <c r="I46" s="14"/>
       <c r="J46" s="14" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="K46" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4277,18 +4336,18 @@
         <v>45</v>
       </c>
       <c r="F47" s="11" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="G47" s="11" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="H47" s="11"/>
       <c r="I47" s="11"/>
       <c r="J47" s="11" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="K47" s="18" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4310,18 +4369,18 @@
         <v>180</v>
       </c>
       <c r="F48" s="14" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="G48" s="14" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="H48" s="14"/>
       <c r="I48" s="14"/>
       <c r="J48" s="14" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="K48" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4343,22 +4402,22 @@
         <v>15</v>
       </c>
       <c r="F49" s="14" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="G49" s="14" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="H49" s="14" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="I49" s="14" t="n">
         <v>3</v>
       </c>
       <c r="J49" s="14" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="K49" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4380,18 +4439,18 @@
         <v>45</v>
       </c>
       <c r="F50" s="14" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="G50" s="14" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="H50" s="14"/>
       <c r="I50" s="14"/>
       <c r="J50" s="14" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="K50" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4413,22 +4472,22 @@
         <v>10</v>
       </c>
       <c r="F51" s="14" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="G51" s="14" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="H51" s="14" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="I51" s="14" t="n">
         <v>1</v>
       </c>
       <c r="J51" s="14" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="K51" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4450,18 +4509,18 @@
         <v>30</v>
       </c>
       <c r="F52" s="14" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="G52" s="14" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="H52" s="14"/>
       <c r="I52" s="14"/>
       <c r="J52" s="14" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="K52" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4483,22 +4542,22 @@
         <v>15</v>
       </c>
       <c r="F53" s="14" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="G53" s="14" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="H53" s="14" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="I53" s="14" t="n">
         <v>2</v>
       </c>
       <c r="J53" s="14" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="K53" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4520,18 +4579,18 @@
         <v>95</v>
       </c>
       <c r="F54" s="14" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="G54" s="14" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="H54" s="14"/>
       <c r="I54" s="14"/>
       <c r="J54" s="14" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="K54" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4553,22 +4612,22 @@
         <v>15</v>
       </c>
       <c r="F55" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="G55" s="14" t="s">
         <v>125</v>
       </c>
-      <c r="G55" s="14" t="s">
-        <v>121</v>
-      </c>
       <c r="H55" s="14" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="I55" s="14" t="n">
         <v>1</v>
       </c>
       <c r="J55" s="14" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="K55" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4590,18 +4649,18 @@
         <v>60</v>
       </c>
       <c r="F56" s="11" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="G56" s="11" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="H56" s="11"/>
       <c r="I56" s="11"/>
       <c r="J56" s="11" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="K56" s="18" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4623,18 +4682,18 @@
         <v>40</v>
       </c>
       <c r="F57" s="11" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="G57" s="11" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="H57" s="11"/>
       <c r="I57" s="11"/>
       <c r="J57" s="11" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="K57" s="18" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4656,18 +4715,18 @@
         <v>20</v>
       </c>
       <c r="F58" s="14" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="G58" s="14" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="H58" s="14"/>
       <c r="I58" s="14"/>
       <c r="J58" s="14" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="K58" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4689,22 +4748,22 @@
         <v>90</v>
       </c>
       <c r="F59" s="14" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="G59" s="14" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="H59" s="14" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="I59" s="14" t="n">
         <v>50</v>
       </c>
       <c r="J59" s="14" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="K59" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4726,23 +4785,23 @@
         <v>30</v>
       </c>
       <c r="F60" s="14" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="G60" s="14" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="H60" s="14"/>
       <c r="I60" s="14"/>
       <c r="J60" s="14" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="K60" s="17" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="5" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
     </row>
   </sheetData>
@@ -4833,27 +4892,27 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4861,19 +4920,19 @@
         <v>1</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4881,19 +4940,19 @@
         <v>1</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4901,19 +4960,19 @@
         <v>1</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4921,19 +4980,19 @@
         <v>2</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4941,19 +5000,19 @@
         <v>2</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4961,19 +5020,19 @@
         <v>2</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4981,19 +5040,19 @@
         <v>3</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C10" s="14" t="s">
+        <v>163</v>
+      </c>
+      <c r="D10" s="14" t="s">
         <v>159</v>
       </c>
-      <c r="D10" s="14" t="s">
-        <v>155</v>
-      </c>
       <c r="E10" s="14" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5001,19 +5060,19 @@
         <v>3</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5021,19 +5080,19 @@
         <v>3</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5041,19 +5100,19 @@
         <v>4</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5061,19 +5120,19 @@
         <v>4</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="E14" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="F14" s="14" t="s">
         <v>152</v>
-      </c>
-      <c r="F14" s="14" t="s">
-        <v>148</v>
       </c>
     </row>
   </sheetData>
@@ -5101,90 +5160,90 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
     </row>
   </sheetData>
@@ -5214,184 +5273,184 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
     </row>
   </sheetData>
@@ -5419,202 +5478,202 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="14" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="14" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="14" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="14" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="14" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="14" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="14" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="B25" s="14" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
     </row>
   </sheetData>
@@ -5633,201 +5692,236 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="70"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>274</v>
+        <v>278</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>279</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>277</v>
-      </c>
-      <c r="D4" s="23"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>282</v>
+      </c>
+      <c r="D4" s="14"/>
+      <c r="E4" s="23"/>
+    </row>
+    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>275</v>
+        <v>283</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>278</v>
+        <v>284</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>277</v>
-      </c>
-      <c r="D5" s="23"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>282</v>
+      </c>
+      <c r="D5" s="14" t="s">
+        <v>285</v>
+      </c>
+      <c r="E5" s="23"/>
+    </row>
+    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>280</v>
+        <v>287</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>277</v>
-      </c>
-      <c r="D6" s="23"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>282</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>288</v>
+      </c>
+      <c r="E6" s="23"/>
+    </row>
+    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>279</v>
+        <v>289</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>281</v>
+        <v>290</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>277</v>
-      </c>
-      <c r="D7" s="23"/>
+        <v>291</v>
+      </c>
+      <c r="D7" s="14"/>
+      <c r="E7" s="23"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>279</v>
+        <v>292</v>
       </c>
       <c r="B8" s="14" t="s">
+        <v>293</v>
+      </c>
+      <c r="C8" s="14" t="s">
         <v>282</v>
       </c>
-      <c r="C8" s="14" t="s">
-        <v>277</v>
-      </c>
-      <c r="D8" s="23"/>
+      <c r="D8" s="14"/>
+      <c r="E8" s="23"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>283</v>
+        <v>292</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>284</v>
+        <v>294</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>285</v>
-      </c>
-      <c r="D9" s="23"/>
+        <v>282</v>
+      </c>
+      <c r="D9" s="14"/>
+      <c r="E9" s="23"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>283</v>
+        <v>295</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>286</v>
+        <v>296</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>285</v>
-      </c>
-      <c r="D10" s="23"/>
+        <v>297</v>
+      </c>
+      <c r="D10" s="14"/>
+      <c r="E10" s="23"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>287</v>
+        <v>295</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>288</v>
+        <v>298</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>285</v>
-      </c>
-      <c r="D11" s="23"/>
+        <v>297</v>
+      </c>
+      <c r="D11" s="14"/>
+      <c r="E11" s="23"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>289</v>
+        <v>299</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>291</v>
-      </c>
-      <c r="D12" s="23"/>
+        <v>297</v>
+      </c>
+      <c r="D12" s="14"/>
+      <c r="E12" s="23"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>289</v>
+        <v>301</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>292</v>
+        <v>302</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>285</v>
-      </c>
-      <c r="D13" s="23"/>
+        <v>303</v>
+      </c>
+      <c r="D13" s="14"/>
+      <c r="E13" s="23"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>294</v>
+        <v>304</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>291</v>
-      </c>
-      <c r="D14" s="23"/>
+        <v>297</v>
+      </c>
+      <c r="D14" s="14"/>
+      <c r="E14" s="23"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
-        <v>295</v>
+        <v>305</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>296</v>
+        <v>306</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>291</v>
-      </c>
-      <c r="D15" s="23"/>
+        <v>303</v>
+      </c>
+      <c r="D15" s="14"/>
+      <c r="E15" s="23"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>297</v>
+        <v>307</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>298</v>
+        <v>308</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>291</v>
-      </c>
-      <c r="D16" s="23"/>
+        <v>303</v>
+      </c>
+      <c r="D16" s="14"/>
+      <c r="E16" s="23"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
-        <v>299</v>
+        <v>309</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>300</v>
+        <v>310</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>291</v>
-      </c>
-      <c r="D17" s="23"/>
+        <v>303</v>
+      </c>
+      <c r="D17" s="14"/>
+      <c r="E17" s="23"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="14" t="s">
+        <v>311</v>
+      </c>
+      <c r="B18" s="14" t="s">
+        <v>312</v>
+      </c>
+      <c r="C18" s="14" t="s">
+        <v>303</v>
+      </c>
+      <c r="D18" s="14"/>
+      <c r="E18" s="23"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -5854,146 +5948,146 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>301</v>
+        <v>313</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>302</v>
+        <v>314</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>303</v>
+        <v>315</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>304</v>
+        <v>316</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>303</v>
+        <v>315</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>305</v>
+        <v>317</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>303</v>
+        <v>315</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>306</v>
+        <v>318</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>303</v>
+        <v>315</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>307</v>
+        <v>319</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>303</v>
+        <v>315</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>308</v>
+        <v>320</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>303</v>
+        <v>315</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>309</v>
+        <v>321</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>303</v>
+        <v>315</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>310</v>
+        <v>322</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>311</v>
+        <v>323</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>312</v>
+        <v>324</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>311</v>
+        <v>323</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>313</v>
+        <v>325</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>311</v>
+        <v>323</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>314</v>
+        <v>326</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>311</v>
+        <v>323</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>315</v>
+        <v>327</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>311</v>
+        <v>323</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>316</v>
+        <v>328</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>311</v>
+        <v>323</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>317</v>
+        <v>329</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
-        <v>318</v>
+        <v>330</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>319</v>
+        <v>331</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>320</v>
+        <v>332</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>321</v>
+        <v>333</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
-        <v>322</v>
+        <v>334</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>323</v>
+        <v>335</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>324</v>
+        <v>336</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>325</v>
+        <v>337</v>
       </c>
     </row>
   </sheetData>
@@ -6021,90 +6115,90 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>326</v>
+        <v>338</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>327</v>
+        <v>339</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>328</v>
+        <v>340</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>329</v>
+        <v>341</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>330</v>
+        <v>342</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>331</v>
+        <v>343</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>332</v>
+        <v>344</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>333</v>
+        <v>345</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>334</v>
+        <v>346</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>335</v>
+        <v>347</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>336</v>
+        <v>348</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>337</v>
+        <v>349</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>338</v>
+        <v>350</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>339</v>
+        <v>351</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>340</v>
+        <v>352</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>341</v>
+        <v>353</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>342</v>
+        <v>354</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>343</v>
+        <v>355</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>344</v>
+        <v>356</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>345</v>
+        <v>357</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>346</v>
+        <v>358</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Re-time both itineraries: breakfast 07:30-08:30, depart hotel 09:00 daily
Helicopter slots move to 12:15 on Days 2 and 3; Jammu-Srinagar flight
to about 12:00; 4-day return travel after 12:30; 8-day departure from
Srinagar after 18:45. Workbooks and brochures rebuilt from the new
schedule.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A4yYiJq592wzPacq5vAVkN
</commit_message>
<xml_diff>
--- a/docs/itineraries/vaishno-devi-helicopter-4d-plan.xlsx
+++ b/docs/itineraries/vaishno-devi-helicopter-4d-plan.xlsx
@@ -23,7 +23,7 @@
     <sheet name="Open Points" sheetId="13" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Minute-by-Minute'!$A$4:$K$60</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Minute-by-Minute'!$A$4:$K$61</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="703" uniqueCount="453">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="707" uniqueCount="452">
   <si>
     <t xml:space="preserve">Vaishno Devi Helicopter Yatra – Overview</t>
   </si>
@@ -112,7 +112,7 @@
     <t xml:space="preserve">Other transport: 2 helicopter flights (5–8 min each), Bhairon ropeway, ~5.5 km on the mountain track (2.5 km Day 2, ~3 km Day 3).</t>
   </si>
   <si>
-    <t xml:space="preserve">Assumptions: arrival at Jammu by 14:00 on Day 1; helicopter slots 10:30 (Day 2) and 11:00 (Day 3); one vehicle convoy for the group.</t>
+    <t xml:space="preserve">Assumptions: arrival at Jammu by 14:00 on Day 1; breakfast 07:30–08:30 and departure from the hotel at 09:00 every day; helicopter slots 12:15 (Day 2) and 12:15 (Day 3); one vehicle convoy for the group.</t>
   </si>
   <si>
     <t xml:space="preserve">4 Days Vaishno Devi Helicopter Package – Minute-to-Minute Plan</t>
@@ -253,7 +253,7 @@
     <t xml:space="preserve">Dinner – at the hotel, pre-ordered pure-veg menu; group pays (not in room rate)</t>
   </si>
   <si>
-    <t xml:space="preserve">Breakfast – complimentary with the hotel stay (request 06:30 opening)</t>
+    <t xml:space="preserve">Breakfast – complimentary with the hotel stay</t>
   </si>
   <si>
     <t xml:space="preserve">Check-out, load luggage</t>
@@ -334,7 +334,10 @@
     <t xml:space="preserve">Wake-up, bath, get ready</t>
   </si>
   <si>
-    <t xml:space="preserve">Morning Aarti at the Holy Cave</t>
+    <t xml:space="preserve">Morning Aarti at the Holy Cave (fixed temple timing)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rest, pack small bag</t>
   </si>
   <si>
     <t xml:space="preserve">Breakfast – Shrine Board Bhojanalaya; pay at counter (Bhawan rooms do not include meals)</t>
@@ -436,10 +439,7 @@
     <t xml:space="preserve">Dinner – at the hotel, pre-ordered pure-veg menu; group pays; Day 4 briefing</t>
   </si>
   <si>
-    <t xml:space="preserve">Breakfast – complimentary with the hotel stay</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Check-out, load luggage; collect packed lunch if departure is after 13:00</t>
+    <t xml:space="preserve">Check-out, load luggage; collect packed lunch for the journey</t>
   </si>
   <si>
     <t xml:space="preserve">Drive to Jammu (Jammu Tawi station ~48 km; SMVD Katra station only 2 km)</t>
@@ -451,7 +451,7 @@
     <t xml:space="preserve">Jammu Airport / Jammu Tawi Rly Stn</t>
   </si>
   <si>
-    <t xml:space="preserve">Drop-off, farewell, Jai Mata Di!</t>
+    <t xml:space="preserve">Drop-off, farewell, Jai Mata Di! (book return flights / trains after 12:30)</t>
   </si>
   <si>
     <t xml:space="preserve">Legend: yellow rows = meals, blue rows = helicopter / ropeway.</t>
@@ -502,7 +502,7 @@
     <t xml:space="preserve">Hotel, pre-ordered menu</t>
   </si>
   <si>
-    <t xml:space="preserve">06:30–07:00</t>
+    <t xml:space="preserve">07:30–08:30</t>
   </si>
   <si>
     <t xml:space="preserve">Hotel</t>
@@ -511,7 +511,7 @@
     <t xml:space="preserve">Complimentary</t>
   </si>
   <si>
-    <t xml:space="preserve">12:15–13:00</t>
+    <t xml:space="preserve">14:00–14:45</t>
   </si>
   <si>
     <t xml:space="preserve">Bhojanalaya, Bhawan</t>
@@ -526,7 +526,7 @@
     <t xml:space="preserve">19:30–20:30</t>
   </si>
   <si>
-    <t xml:space="preserve">07:00–07:30</t>
+    <t xml:space="preserve">13:15–14:00</t>
   </si>
   <si>
     <t xml:space="preserve">Hotel restaurant, Katra (or pure-veg restaurant, Main Bazaar)</t>
@@ -538,10 +538,7 @@
     <t xml:space="preserve">20:00–21:00</t>
   </si>
   <si>
-    <t xml:space="preserve">07:00–07:40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Packed from Katra hotel, only if departure after 13:00</t>
+    <t xml:space="preserve">Packed from Katra hotel for onward travel after 12:30</t>
   </si>
   <si>
     <t xml:space="preserve">Aspect</t>
@@ -682,7 +679,7 @@
     <t xml:space="preserve">Avoid peak dates; darshan right after lunch</t>
   </si>
   <si>
-    <t xml:space="preserve">Darshan Day 3 early morning, keep the 11:00 flight</t>
+    <t xml:space="preserve">Darshan Day 3 early morning, keep the 12:15 flight</t>
   </si>
   <si>
     <t xml:space="preserve">Aarti passes not available</t>
@@ -925,7 +922,7 @@
     <t xml:space="preserve">T−45 days</t>
   </si>
   <si>
-    <t xml:space="preserve">Book flights / trains: arrival by 14:00 on Day 1; departure after 11:00 Day 4</t>
+    <t xml:space="preserve">Book flights / trains: arrival by 14:00 on Day 1; departure after 12:30 Day 4</t>
   </si>
   <si>
     <t xml:space="preserve">Travel desk</t>
@@ -2056,18 +2053,18 @@
         <v>13</v>
       </c>
       <c r="D5" s="7" t="n">
-        <f aca="false">SUMIF('Minute-by-Minute'!$A$5:$A$60,A5,'Minute-by-Minute'!$I$5:$I$60)</f>
+        <f aca="false">SUMIF('Minute-by-Minute'!$A$5:$A$61,A5,'Minute-by-Minute'!$I$5:$I$61)</f>
         <v>32</v>
       </c>
       <c r="E5" s="7" t="s">
         <v>14</v>
       </c>
       <c r="F5" s="9" t="n">
-        <f aca="false">_xlfn.MINIFS('Minute-by-Minute'!$C$5:$C$60,'Minute-by-Minute'!$A$5:$A$60,A5)</f>
+        <f aca="false">_xlfn.MINIFS('Minute-by-Minute'!$C$5:$C$61,'Minute-by-Minute'!$A$5:$A$61,A5)</f>
         <v>0.333333333333333</v>
       </c>
       <c r="G5" s="9" t="n">
-        <f aca="false">_xlfn.MAXIFS('Minute-by-Minute'!$D$5:$D$60,'Minute-by-Minute'!$A$5:$A$60,A5)</f>
+        <f aca="false">_xlfn.MAXIFS('Minute-by-Minute'!$D$5:$D$61,'Minute-by-Minute'!$A$5:$A$61,A5)</f>
         <v>0.885416666666667</v>
       </c>
       <c r="I5" s="7" t="s">
@@ -2089,18 +2086,18 @@
         <v>16</v>
       </c>
       <c r="D6" s="7" t="n">
-        <f aca="false">SUMIF('Minute-by-Minute'!$A$5:$A$60,A6,'Minute-by-Minute'!$I$5:$I$60)</f>
+        <f aca="false">SUMIF('Minute-by-Minute'!$A$5:$A$61,A6,'Minute-by-Minute'!$I$5:$I$61)</f>
         <v>52</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>17</v>
       </c>
       <c r="F6" s="9" t="n">
-        <f aca="false">_xlfn.MINIFS('Minute-by-Minute'!$C$5:$C$60,'Minute-by-Minute'!$A$5:$A$60,A6)</f>
-        <v>0.270833333333333</v>
+        <f aca="false">_xlfn.MINIFS('Minute-by-Minute'!$C$5:$C$61,'Minute-by-Minute'!$A$5:$A$61,A6)</f>
+        <v>0.3125</v>
       </c>
       <c r="G6" s="9" t="n">
-        <f aca="false">_xlfn.MAXIFS('Minute-by-Minute'!$D$5:$D$60,'Minute-by-Minute'!$A$5:$A$60,A6)</f>
+        <f aca="false">_xlfn.MAXIFS('Minute-by-Minute'!$D$5:$D$61,'Minute-by-Minute'!$A$5:$A$61,A6)</f>
         <v>0.854166666666667</v>
       </c>
       <c r="I6" s="7" t="s">
@@ -2122,18 +2119,18 @@
         <v>19</v>
       </c>
       <c r="D7" s="7" t="n">
-        <f aca="false">SUMIF('Minute-by-Minute'!$A$5:$A$60,A7,'Minute-by-Minute'!$I$5:$I$60)</f>
+        <f aca="false">SUMIF('Minute-by-Minute'!$A$5:$A$61,A7,'Minute-by-Minute'!$I$5:$I$61)</f>
         <v>9</v>
       </c>
       <c r="E7" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F7" s="9" t="n">
-        <f aca="false">_xlfn.MINIFS('Minute-by-Minute'!$C$5:$C$60,'Minute-by-Minute'!$A$5:$A$60,A7)</f>
+        <f aca="false">_xlfn.MINIFS('Minute-by-Minute'!$C$5:$C$61,'Minute-by-Minute'!$A$5:$A$61,A7)</f>
         <v>0.1875</v>
       </c>
       <c r="G7" s="9" t="n">
-        <f aca="false">_xlfn.MAXIFS('Minute-by-Minute'!$D$5:$D$60,'Minute-by-Minute'!$A$5:$A$60,A7)</f>
+        <f aca="false">_xlfn.MAXIFS('Minute-by-Minute'!$D$5:$D$61,'Minute-by-Minute'!$A$5:$A$61,A7)</f>
         <v>0.875</v>
       </c>
     </row>
@@ -2149,19 +2146,19 @@
         <v>21</v>
       </c>
       <c r="D8" s="7" t="n">
-        <f aca="false">SUMIF('Minute-by-Minute'!$A$5:$A$60,A8,'Minute-by-Minute'!$I$5:$I$60)</f>
+        <f aca="false">SUMIF('Minute-by-Minute'!$A$5:$A$61,A8,'Minute-by-Minute'!$I$5:$I$61)</f>
         <v>50</v>
       </c>
       <c r="E8" s="7" t="s">
         <v>22</v>
       </c>
       <c r="F8" s="9" t="n">
-        <f aca="false">_xlfn.MINIFS('Minute-by-Minute'!$C$5:$C$60,'Minute-by-Minute'!$A$5:$A$60,A8)</f>
-        <v>0.291666666666667</v>
+        <f aca="false">_xlfn.MINIFS('Minute-by-Minute'!$C$5:$C$61,'Minute-by-Minute'!$A$5:$A$61,A8)</f>
+        <v>0.3125</v>
       </c>
       <c r="G8" s="9" t="n">
-        <f aca="false">_xlfn.MAXIFS('Minute-by-Minute'!$D$5:$D$60,'Minute-by-Minute'!$A$5:$A$60,A8)</f>
-        <v>0.416666666666667</v>
+        <f aca="false">_xlfn.MAXIFS('Minute-by-Minute'!$D$5:$D$61,'Minute-by-Minute'!$A$5:$A$61,A8)</f>
+        <v>0.458333333333333</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2211,121 +2208,121 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
+        <v>358</v>
+      </c>
+      <c r="B1" s="10" t="s">
         <v>359</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="C1" s="10" t="s">
         <v>360</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="D1" s="10" t="s">
         <v>361</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="E1" s="10" t="s">
         <v>362</v>
-      </c>
-      <c r="E1" s="10" t="s">
-        <v>363</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
+        <v>363</v>
+      </c>
+      <c r="B2" s="14" t="s">
         <v>364</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="C2" s="14" t="s">
         <v>365</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="D2" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="E2" s="14" t="s">
         <v>366</v>
-      </c>
-      <c r="D2" s="14" t="s">
-        <v>170</v>
-      </c>
-      <c r="E2" s="14" t="s">
-        <v>367</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
+        <v>367</v>
+      </c>
+      <c r="B3" s="14" t="s">
         <v>368</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="C3" s="14" t="s">
         <v>369</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="D3" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="E3" s="14" t="s">
         <v>370</v>
-      </c>
-      <c r="D3" s="14" t="s">
-        <v>170</v>
-      </c>
-      <c r="E3" s="14" t="s">
-        <v>371</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
+        <v>371</v>
+      </c>
+      <c r="B4" s="14" t="s">
         <v>372</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="C4" s="14" t="s">
         <v>373</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="D4" s="14" t="s">
         <v>374</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="E4" s="14" t="s">
         <v>375</v>
-      </c>
-      <c r="E4" s="14" t="s">
-        <v>376</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
+        <v>376</v>
+      </c>
+      <c r="B5" s="14" t="s">
         <v>377</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="C5" s="14" t="s">
         <v>378</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="D5" s="14" t="s">
         <v>379</v>
       </c>
-      <c r="D5" s="14" t="s">
+      <c r="E5" s="14" t="s">
         <v>380</v>
-      </c>
-      <c r="E5" s="14" t="s">
-        <v>381</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="B6" s="14" t="s">
+        <v>381</v>
+      </c>
+      <c r="C6" s="14" t="s">
         <v>382</v>
       </c>
-      <c r="C6" s="14" t="s">
-        <v>383</v>
-      </c>
       <c r="D6" s="14" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="B7" s="14" t="s">
+        <v>383</v>
+      </c>
+      <c r="C7" s="14" t="s">
         <v>384</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="D7" s="14" t="s">
         <v>385</v>
       </c>
-      <c r="D7" s="14" t="s">
+      <c r="E7" s="14" t="s">
         <v>386</v>
-      </c>
-      <c r="E7" s="14" t="s">
-        <v>387</v>
       </c>
     </row>
   </sheetData>
@@ -2355,74 +2352,74 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
+        <v>387</v>
+      </c>
+      <c r="B1" s="10" t="s">
         <v>388</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="C1" s="10" t="s">
         <v>389</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="D1" s="10" t="s">
         <v>390</v>
-      </c>
-      <c r="D1" s="10" t="s">
-        <v>391</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="C2" s="23"/>
       <c r="D2" s="23"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
+        <v>392</v>
+      </c>
+      <c r="B3" s="14" t="s">
         <v>393</v>
-      </c>
-      <c r="B3" s="14" t="s">
-        <v>394</v>
       </c>
       <c r="C3" s="23"/>
       <c r="D3" s="23"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
+        <v>394</v>
+      </c>
+      <c r="B4" s="14" t="s">
         <v>395</v>
-      </c>
-      <c r="B4" s="14" t="s">
-        <v>396</v>
       </c>
       <c r="C4" s="23"/>
       <c r="D4" s="23"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
+        <v>396</v>
+      </c>
+      <c r="B5" s="14" t="s">
         <v>397</v>
-      </c>
-      <c r="B5" s="14" t="s">
-        <v>398</v>
       </c>
       <c r="C5" s="23"/>
       <c r="D5" s="23"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
+        <v>398</v>
+      </c>
+      <c r="B6" s="14" t="s">
         <v>399</v>
-      </c>
-      <c r="B6" s="14" t="s">
-        <v>400</v>
       </c>
       <c r="C6" s="23"/>
       <c r="D6" s="23"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
+        <v>400</v>
+      </c>
+      <c r="B7" s="14" t="s">
         <v>401</v>
-      </c>
-      <c r="B7" s="14" t="s">
-        <v>402</v>
       </c>
       <c r="C7" s="23"/>
       <c r="D7" s="23"/>
@@ -2437,7 +2434,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B9" s="14"/>
       <c r="C9" s="23"/>
@@ -2445,7 +2442,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="B10" s="14"/>
       <c r="C10" s="23"/>
@@ -2453,7 +2450,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="B11" s="14"/>
       <c r="C11" s="23"/>
@@ -2461,7 +2458,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B12" s="14"/>
       <c r="C12" s="23"/>
@@ -2469,14 +2466,14 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
+        <v>405</v>
+      </c>
+      <c r="B13" s="14" t="s">
         <v>406</v>
-      </c>
-      <c r="B13" s="14" t="s">
-        <v>407</v>
       </c>
       <c r="C13" s="14"/>
       <c r="D13" s="14" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
   </sheetData>
@@ -2506,187 +2503,187 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
+        <v>410</v>
+      </c>
+      <c r="B4" s="6" t="s">
         <v>411</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="C4" s="6" t="s">
         <v>412</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="D4" s="6" t="s">
         <v>413</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>414</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
+        <v>414</v>
+      </c>
+      <c r="B5" s="7" t="s">
         <v>415</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="C5" s="7" t="s">
         <v>416</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>417</v>
       </c>
       <c r="D5" s="24"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
+        <v>417</v>
+      </c>
+      <c r="B6" s="7" t="s">
         <v>418</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="C6" s="7" t="s">
         <v>419</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>420</v>
       </c>
       <c r="D6" s="24"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
+        <v>420</v>
+      </c>
+      <c r="B7" s="7" t="s">
         <v>421</v>
       </c>
-      <c r="B7" s="7" t="s">
-        <v>422</v>
-      </c>
       <c r="C7" s="7" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="D7" s="24"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="B8" s="7" t="s">
+        <v>418</v>
+      </c>
+      <c r="C8" s="7" t="s">
         <v>419</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>420</v>
       </c>
       <c r="D8" s="24"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
+        <v>423</v>
+      </c>
+      <c r="B9" s="7" t="s">
         <v>424</v>
       </c>
-      <c r="B9" s="7" t="s">
-        <v>425</v>
-      </c>
       <c r="C9" s="7" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="D9" s="24"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="D10" s="24"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="D11" s="24"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
+        <v>427</v>
+      </c>
+      <c r="B12" s="7" t="s">
         <v>428</v>
       </c>
-      <c r="B12" s="7" t="s">
-        <v>429</v>
-      </c>
       <c r="C12" s="7" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="D12" s="24"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
+        <v>429</v>
+      </c>
+      <c r="B13" s="7" t="s">
         <v>430</v>
       </c>
-      <c r="B13" s="7" t="s">
-        <v>431</v>
-      </c>
       <c r="C13" s="7" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="D13" s="24"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="D14" s="24"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="D15" s="24"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="D16" s="24"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
+        <v>434</v>
+      </c>
+      <c r="B17" s="7" t="s">
         <v>435</v>
       </c>
-      <c r="B17" s="7" t="s">
-        <v>436</v>
-      </c>
       <c r="C17" s="7" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="D17" s="24"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="D18" s="25" t="n">
         <f aca="false">SUMIF(C5:C17,"Yes",D5:D17)</f>
@@ -2695,10 +2692,10 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>438</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>439</v>
       </c>
       <c r="D19" s="26" t="n">
         <v>0.05</v>
@@ -2706,7 +2703,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="D20" s="25" t="n">
         <f aca="false">D18*(1+D19)</f>
@@ -2715,7 +2712,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
   </sheetData>
@@ -2743,69 +2740,69 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="B2" s="14"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B3" s="14"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B4" s="14"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="B5" s="14"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="B6" s="14"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="B7" s="14"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="B8" s="14"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="B9" s="14"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="B10" s="14"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="B11" s="14"/>
     </row>
@@ -2825,7 +2822,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K62"/>
+  <dimension ref="A1:K63"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -3444,14 +3441,14 @@
         <v>46460</v>
       </c>
       <c r="C21" s="13" t="n">
-        <v>0.270833333333333</v>
+        <v>0.3125</v>
       </c>
       <c r="D21" s="13" t="n">
-        <v>0.291666666666667</v>
+        <v>0.354166666666667</v>
       </c>
       <c r="E21" s="11" t="n">
         <f aca="false">ROUND((D21-C21)*1440,0)</f>
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="F21" s="11" t="s">
         <v>36</v>
@@ -3477,14 +3474,14 @@
         <v>46460</v>
       </c>
       <c r="C22" s="16" t="n">
-        <v>0.291666666666667</v>
+        <v>0.354166666666667</v>
       </c>
       <c r="D22" s="16" t="n">
-        <v>0.302083333333333</v>
+        <v>0.375</v>
       </c>
       <c r="E22" s="14" t="n">
         <f aca="false">ROUND((D22-C22)*1440,0)</f>
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F22" s="14" t="s">
         <v>47</v>
@@ -3510,10 +3507,10 @@
         <v>46460</v>
       </c>
       <c r="C23" s="16" t="n">
-        <v>0.302083333333333</v>
+        <v>0.375</v>
       </c>
       <c r="D23" s="16" t="n">
-        <v>0.364583333333333</v>
+        <v>0.4375</v>
       </c>
       <c r="E23" s="14" t="n">
         <f aca="false">ROUND((D23-C23)*1440,0)</f>
@@ -3547,10 +3544,10 @@
         <v>46460</v>
       </c>
       <c r="C24" s="16" t="n">
-        <v>0.364583333333333</v>
+        <v>0.4375</v>
       </c>
       <c r="D24" s="16" t="n">
-        <v>0.385416666666667</v>
+        <v>0.458333333333333</v>
       </c>
       <c r="E24" s="14" t="n">
         <f aca="false">ROUND((D24-C24)*1440,0)</f>
@@ -3580,10 +3577,10 @@
         <v>46460</v>
       </c>
       <c r="C25" s="16" t="n">
-        <v>0.385416666666667</v>
+        <v>0.458333333333333</v>
       </c>
       <c r="D25" s="16" t="n">
-        <v>0.392361111111111</v>
+        <v>0.465277777777778</v>
       </c>
       <c r="E25" s="14" t="n">
         <f aca="false">ROUND((D25-C25)*1440,0)</f>
@@ -3617,10 +3614,10 @@
         <v>46460</v>
       </c>
       <c r="C26" s="16" t="n">
-        <v>0.392361111111111</v>
+        <v>0.465277777777778</v>
       </c>
       <c r="D26" s="16" t="n">
-        <v>0.4375</v>
+        <v>0.510416666666667</v>
       </c>
       <c r="E26" s="14" t="n">
         <f aca="false">ROUND((D26-C26)*1440,0)</f>
@@ -3650,10 +3647,10 @@
         <v>46460</v>
       </c>
       <c r="C27" s="21" t="n">
-        <v>0.4375</v>
+        <v>0.510416666666667</v>
       </c>
       <c r="D27" s="21" t="n">
-        <v>0.444444444444444</v>
+        <v>0.517361111111111</v>
       </c>
       <c r="E27" s="19" t="n">
         <f aca="false">ROUND((D27-C27)*1440,0)</f>
@@ -3685,10 +3682,10 @@
         <v>46460</v>
       </c>
       <c r="C28" s="16" t="n">
-        <v>0.444444444444444</v>
+        <v>0.517361111111111</v>
       </c>
       <c r="D28" s="16" t="n">
-        <v>0.489583333333333</v>
+        <v>0.5625</v>
       </c>
       <c r="E28" s="14" t="n">
         <f aca="false">ROUND((D28-C28)*1440,0)</f>
@@ -3720,10 +3717,10 @@
         <v>46460</v>
       </c>
       <c r="C29" s="16" t="n">
-        <v>0.489583333333333</v>
+        <v>0.5625</v>
       </c>
       <c r="D29" s="16" t="n">
-        <v>0.510416666666667</v>
+        <v>0.583333333333333</v>
       </c>
       <c r="E29" s="14" t="n">
         <f aca="false">ROUND((D29-C29)*1440,0)</f>
@@ -3753,10 +3750,10 @@
         <v>46460</v>
       </c>
       <c r="C30" s="13" t="n">
-        <v>0.510416666666667</v>
+        <v>0.583333333333333</v>
       </c>
       <c r="D30" s="13" t="n">
-        <v>0.541666666666667</v>
+        <v>0.614583333333333</v>
       </c>
       <c r="E30" s="11" t="n">
         <f aca="false">ROUND((D30-C30)*1440,0)</f>
@@ -3786,14 +3783,14 @@
         <v>46460</v>
       </c>
       <c r="C31" s="16" t="n">
-        <v>0.541666666666667</v>
+        <v>0.614583333333333</v>
       </c>
       <c r="D31" s="16" t="n">
         <v>0.6875</v>
       </c>
       <c r="E31" s="14" t="n">
         <f aca="false">ROUND((D31-C31)*1440,0)</f>
-        <v>210</v>
+        <v>105</v>
       </c>
       <c r="F31" s="14" t="s">
         <v>91</v>
@@ -3975,69 +3972,69 @@
         <v>42</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="11" t="n">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="B37" s="12" t="n">
+      <c r="B37" s="15" t="n">
         <f aca="false">Overview!$B$3+A37-1</f>
         <v>46461</v>
       </c>
-      <c r="C37" s="13" t="n">
+      <c r="C37" s="16" t="n">
         <v>0.291666666666667</v>
       </c>
-      <c r="D37" s="13" t="n">
+      <c r="D37" s="16" t="n">
         <v>0.3125</v>
       </c>
-      <c r="E37" s="11" t="n">
+      <c r="E37" s="14" t="n">
         <f aca="false">ROUND((D37-C37)*1440,0)</f>
         <v>30</v>
       </c>
-      <c r="F37" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="G37" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="H37" s="11"/>
-      <c r="I37" s="11"/>
-      <c r="J37" s="11" t="s">
+      <c r="F37" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="G37" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="H37" s="14"/>
+      <c r="I37" s="14"/>
+      <c r="J37" s="14" t="s">
         <v>100</v>
       </c>
-      <c r="K37" s="18" t="s">
+      <c r="K37" s="17" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="14" t="n">
+    <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="B38" s="15" t="n">
+      <c r="B38" s="12" t="n">
         <f aca="false">Overview!$B$3+A38-1</f>
         <v>46461</v>
       </c>
-      <c r="C38" s="16" t="n">
+      <c r="C38" s="13" t="n">
         <v>0.3125</v>
       </c>
-      <c r="D38" s="16" t="n">
-        <v>0.322916666666667</v>
-      </c>
-      <c r="E38" s="14" t="n">
+      <c r="D38" s="13" t="n">
+        <v>0.354166666666667</v>
+      </c>
+      <c r="E38" s="11" t="n">
         <f aca="false">ROUND((D38-C38)*1440,0)</f>
-        <v>15</v>
-      </c>
-      <c r="F38" s="14" t="s">
-        <v>47</v>
-      </c>
-      <c r="G38" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="H38" s="14"/>
-      <c r="I38" s="14"/>
-      <c r="J38" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="F38" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="G38" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="H38" s="11"/>
+      <c r="I38" s="11"/>
+      <c r="J38" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="K38" s="17" t="s">
+      <c r="K38" s="18" t="s">
         <v>42</v>
       </c>
     </row>
@@ -4050,97 +4047,97 @@
         <v>46461</v>
       </c>
       <c r="C39" s="16" t="n">
-        <v>0.322916666666667</v>
+        <v>0.354166666666667</v>
       </c>
       <c r="D39" s="16" t="n">
-        <v>0.333333333333333</v>
+        <v>0.375</v>
       </c>
       <c r="E39" s="14" t="n">
         <f aca="false">ROUND((D39-C39)*1440,0)</f>
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F39" s="14" t="s">
-        <v>102</v>
+        <v>47</v>
       </c>
       <c r="G39" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="H39" s="14" t="s">
-        <v>103</v>
-      </c>
+      <c r="H39" s="14"/>
       <c r="I39" s="14"/>
       <c r="J39" s="14" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="K39" s="17" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="19" t="n">
+      <c r="A40" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="B40" s="20" t="n">
+      <c r="B40" s="15" t="n">
         <f aca="false">Overview!$B$3+A40-1</f>
         <v>46461</v>
       </c>
-      <c r="C40" s="21" t="n">
-        <v>0.333333333333333</v>
-      </c>
-      <c r="D40" s="21" t="n">
-        <v>0.347222222222222</v>
-      </c>
-      <c r="E40" s="19" t="n">
+      <c r="C40" s="16" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="D40" s="16" t="n">
+        <v>0.385416666666667</v>
+      </c>
+      <c r="E40" s="14" t="n">
         <f aca="false">ROUND((D40-C40)*1440,0)</f>
-        <v>20</v>
-      </c>
-      <c r="F40" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="F40" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="G40" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="H40" s="14" t="s">
+        <v>104</v>
+      </c>
+      <c r="I40" s="14"/>
+      <c r="J40" s="14" t="s">
         <v>105</v>
       </c>
-      <c r="G40" s="19" t="s">
-        <v>103</v>
-      </c>
-      <c r="H40" s="19" t="s">
-        <v>106</v>
-      </c>
-      <c r="I40" s="19"/>
-      <c r="J40" s="19" t="s">
-        <v>107</v>
-      </c>
-      <c r="K40" s="22" t="s">
+      <c r="K40" s="17" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="14" t="n">
+      <c r="A41" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="B41" s="15" t="n">
+      <c r="B41" s="20" t="n">
         <f aca="false">Overview!$B$3+A41-1</f>
         <v>46461</v>
       </c>
-      <c r="C41" s="16" t="n">
-        <v>0.347222222222222</v>
-      </c>
-      <c r="D41" s="16" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="E41" s="14" t="n">
+      <c r="C41" s="21" t="n">
+        <v>0.385416666666667</v>
+      </c>
+      <c r="D41" s="21" t="n">
+        <v>0.399305555555556</v>
+      </c>
+      <c r="E41" s="19" t="n">
         <f aca="false">ROUND((D41-C41)*1440,0)</f>
-        <v>40</v>
-      </c>
-      <c r="F41" s="14" t="s">
-        <v>55</v>
-      </c>
-      <c r="G41" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="F41" s="19" t="s">
+        <v>106</v>
+      </c>
+      <c r="G41" s="19" t="s">
+        <v>104</v>
+      </c>
+      <c r="H41" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="I41" s="19"/>
+      <c r="J41" s="19" t="s">
         <v>108</v>
       </c>
-      <c r="H41" s="14"/>
-      <c r="I41" s="14"/>
-      <c r="J41" s="14" t="s">
-        <v>109</v>
-      </c>
-      <c r="K41" s="17" t="s">
+      <c r="K41" s="22" t="s">
         <v>42</v>
       </c>
     </row>
@@ -4153,27 +4150,25 @@
         <v>46461</v>
       </c>
       <c r="C42" s="16" t="n">
-        <v>0.375</v>
+        <v>0.399305555555556</v>
       </c>
       <c r="D42" s="16" t="n">
-        <v>0.416666666666667</v>
+        <v>0.427083333333333</v>
       </c>
       <c r="E42" s="14" t="n">
         <f aca="false">ROUND((D42-C42)*1440,0)</f>
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="F42" s="14" t="s">
-        <v>110</v>
+        <v>55</v>
       </c>
       <c r="G42" s="14" t="s">
-        <v>111</v>
-      </c>
-      <c r="H42" s="14" t="s">
-        <v>84</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="H42" s="14"/>
       <c r="I42" s="14"/>
       <c r="J42" s="14" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="K42" s="17" t="s">
         <v>42</v>
@@ -4188,22 +4183,24 @@
         <v>46461</v>
       </c>
       <c r="C43" s="16" t="n">
-        <v>0.416666666666667</v>
+        <v>0.427083333333333</v>
       </c>
       <c r="D43" s="16" t="n">
-        <v>0.458333333333333</v>
+        <v>0.46875</v>
       </c>
       <c r="E43" s="14" t="n">
         <f aca="false">ROUND((D43-C43)*1440,0)</f>
         <v>60</v>
       </c>
       <c r="F43" s="14" t="s">
-        <v>81</v>
+        <v>111</v>
       </c>
       <c r="G43" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="H43" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="H43" s="14"/>
       <c r="I43" s="14"/>
       <c r="J43" s="14" t="s">
         <v>113</v>
@@ -4213,74 +4210,70 @@
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="19" t="n">
+      <c r="A44" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="B44" s="20" t="n">
+      <c r="B44" s="15" t="n">
         <f aca="false">Overview!$B$3+A44-1</f>
         <v>46461</v>
       </c>
-      <c r="C44" s="21" t="n">
-        <v>0.458333333333333</v>
-      </c>
-      <c r="D44" s="21" t="n">
-        <v>0.465277777777778</v>
-      </c>
-      <c r="E44" s="19" t="n">
+      <c r="C44" s="16" t="n">
+        <v>0.46875</v>
+      </c>
+      <c r="D44" s="16" t="n">
+        <v>0.510416666666667</v>
+      </c>
+      <c r="E44" s="14" t="n">
         <f aca="false">ROUND((D44-C44)*1440,0)</f>
-        <v>10</v>
-      </c>
-      <c r="F44" s="19" t="s">
-        <v>83</v>
-      </c>
-      <c r="G44" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="F44" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="G44" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="H44" s="19" t="s">
-        <v>79</v>
-      </c>
-      <c r="I44" s="19"/>
-      <c r="J44" s="19" t="s">
+      <c r="H44" s="14"/>
+      <c r="I44" s="14"/>
+      <c r="J44" s="14" t="s">
         <v>114</v>
       </c>
-      <c r="K44" s="22" t="s">
+      <c r="K44" s="17" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="14" t="n">
+      <c r="A45" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="B45" s="15" t="n">
+      <c r="B45" s="20" t="n">
         <f aca="false">Overview!$B$3+A45-1</f>
         <v>46461</v>
       </c>
-      <c r="C45" s="16" t="n">
-        <v>0.465277777777778</v>
-      </c>
-      <c r="D45" s="16" t="n">
-        <v>0.475694444444444</v>
-      </c>
-      <c r="E45" s="14" t="n">
+      <c r="C45" s="21" t="n">
+        <v>0.510416666666667</v>
+      </c>
+      <c r="D45" s="21" t="n">
+        <v>0.517361111111111</v>
+      </c>
+      <c r="E45" s="19" t="n">
         <f aca="false">ROUND((D45-C45)*1440,0)</f>
-        <v>15</v>
-      </c>
-      <c r="F45" s="14" t="s">
-        <v>43</v>
-      </c>
-      <c r="G45" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F45" s="19" t="s">
+        <v>83</v>
+      </c>
+      <c r="G45" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="H45" s="19" t="s">
         <v>79</v>
       </c>
-      <c r="H45" s="14" t="s">
+      <c r="I45" s="19"/>
+      <c r="J45" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="I45" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="J45" s="14" t="s">
-        <v>116</v>
-      </c>
-      <c r="K45" s="17" t="s">
+      <c r="K45" s="22" t="s">
         <v>42</v>
       </c>
     </row>
@@ -4293,93 +4286,97 @@
         <v>46461</v>
       </c>
       <c r="C46" s="16" t="n">
-        <v>0.475694444444444</v>
+        <v>0.517361111111111</v>
       </c>
       <c r="D46" s="16" t="n">
-        <v>0.510416666666667</v>
+        <v>0.527777777777778</v>
       </c>
       <c r="E46" s="14" t="n">
         <f aca="false">ROUND((D46-C46)*1440,0)</f>
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="F46" s="14" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="G46" s="14" t="s">
-        <v>115</v>
-      </c>
-      <c r="H46" s="14"/>
-      <c r="I46" s="14"/>
+        <v>79</v>
+      </c>
+      <c r="H46" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="I46" s="14" t="n">
+        <v>2</v>
+      </c>
       <c r="J46" s="14" t="s">
-        <v>49</v>
+        <v>117</v>
       </c>
       <c r="K46" s="17" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="11" t="n">
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="B47" s="12" t="n">
+      <c r="B47" s="15" t="n">
         <f aca="false">Overview!$B$3+A47-1</f>
         <v>46461</v>
       </c>
-      <c r="C47" s="13" t="n">
-        <v>0.510416666666667</v>
-      </c>
-      <c r="D47" s="13" t="n">
-        <v>0.541666666666667</v>
-      </c>
-      <c r="E47" s="11" t="n">
+      <c r="C47" s="16" t="n">
+        <v>0.527777777777778</v>
+      </c>
+      <c r="D47" s="16" t="n">
+        <v>0.552083333333333</v>
+      </c>
+      <c r="E47" s="14" t="n">
         <f aca="false">ROUND((D47-C47)*1440,0)</f>
-        <v>45</v>
-      </c>
-      <c r="F47" s="11" t="s">
-        <v>50</v>
-      </c>
-      <c r="G47" s="11" t="s">
-        <v>117</v>
-      </c>
-      <c r="H47" s="11"/>
-      <c r="I47" s="11"/>
-      <c r="J47" s="11" t="s">
-        <v>118</v>
-      </c>
-      <c r="K47" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="F47" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="G47" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="H47" s="14"/>
+      <c r="I47" s="14"/>
+      <c r="J47" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="K47" s="17" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="14" t="n">
+    <row r="48" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="B48" s="15" t="n">
+      <c r="B48" s="12" t="n">
         <f aca="false">Overview!$B$3+A48-1</f>
         <v>46461</v>
       </c>
-      <c r="C48" s="16" t="n">
-        <v>0.541666666666667</v>
-      </c>
-      <c r="D48" s="16" t="n">
-        <v>0.666666666666667</v>
-      </c>
-      <c r="E48" s="14" t="n">
+      <c r="C48" s="13" t="n">
+        <v>0.552083333333333</v>
+      </c>
+      <c r="D48" s="13" t="n">
+        <v>0.583333333333333</v>
+      </c>
+      <c r="E48" s="11" t="n">
         <f aca="false">ROUND((D48-C48)*1440,0)</f>
-        <v>180</v>
-      </c>
-      <c r="F48" s="14" t="s">
-        <v>91</v>
-      </c>
-      <c r="G48" s="14" t="s">
-        <v>115</v>
-      </c>
-      <c r="H48" s="14"/>
-      <c r="I48" s="14"/>
-      <c r="J48" s="14" t="s">
-        <v>91</v>
-      </c>
-      <c r="K48" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="F48" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="G48" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="H48" s="11"/>
+      <c r="I48" s="11"/>
+      <c r="J48" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="K48" s="18" t="s">
         <v>42</v>
       </c>
     </row>
@@ -4392,35 +4389,31 @@
         <v>46461</v>
       </c>
       <c r="C49" s="16" t="n">
+        <v>0.583333333333333</v>
+      </c>
+      <c r="D49" s="16" t="n">
         <v>0.666666666666667</v>
-      </c>
-      <c r="D49" s="16" t="n">
-        <v>0.677083333333333</v>
       </c>
       <c r="E49" s="14" t="n">
         <f aca="false">ROUND((D49-C49)*1440,0)</f>
-        <v>15</v>
+        <v>120</v>
       </c>
       <c r="F49" s="14" t="s">
-        <v>43</v>
+        <v>91</v>
       </c>
       <c r="G49" s="14" t="s">
-        <v>115</v>
-      </c>
-      <c r="H49" s="14" t="s">
-        <v>119</v>
-      </c>
-      <c r="I49" s="14" t="n">
-        <v>3</v>
-      </c>
+        <v>116</v>
+      </c>
+      <c r="H49" s="14"/>
+      <c r="I49" s="14"/>
       <c r="J49" s="14" t="s">
-        <v>120</v>
+        <v>91</v>
       </c>
       <c r="K49" s="17" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="14" t="n">
         <v>3</v>
       </c>
@@ -4429,23 +4422,27 @@
         <v>46461</v>
       </c>
       <c r="C50" s="16" t="n">
+        <v>0.666666666666667</v>
+      </c>
+      <c r="D50" s="16" t="n">
         <v>0.677083333333333</v>
-      </c>
-      <c r="D50" s="16" t="n">
-        <v>0.708333333333333</v>
       </c>
       <c r="E50" s="14" t="n">
         <f aca="false">ROUND((D50-C50)*1440,0)</f>
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="F50" s="14" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="G50" s="14" t="s">
-        <v>119</v>
-      </c>
-      <c r="H50" s="14"/>
-      <c r="I50" s="14"/>
+        <v>116</v>
+      </c>
+      <c r="H50" s="14" t="s">
+        <v>120</v>
+      </c>
+      <c r="I50" s="14" t="n">
+        <v>3</v>
+      </c>
       <c r="J50" s="14" t="s">
         <v>121</v>
       </c>
@@ -4453,7 +4450,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="14" t="n">
         <v>3</v>
       </c>
@@ -4462,29 +4459,25 @@
         <v>46461</v>
       </c>
       <c r="C51" s="16" t="n">
+        <v>0.677083333333333</v>
+      </c>
+      <c r="D51" s="16" t="n">
         <v>0.708333333333333</v>
-      </c>
-      <c r="D51" s="16" t="n">
-        <v>0.715277777777778</v>
       </c>
       <c r="E51" s="14" t="n">
         <f aca="false">ROUND((D51-C51)*1440,0)</f>
-        <v>10</v>
+        <v>45</v>
       </c>
       <c r="F51" s="14" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="G51" s="14" t="s">
-        <v>119</v>
-      </c>
-      <c r="H51" s="14" t="s">
+        <v>120</v>
+      </c>
+      <c r="H51" s="14"/>
+      <c r="I51" s="14"/>
+      <c r="J51" s="14" t="s">
         <v>122</v>
-      </c>
-      <c r="I51" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="J51" s="14" t="s">
-        <v>123</v>
       </c>
       <c r="K51" s="17" t="s">
         <v>42</v>
@@ -4499,23 +4492,27 @@
         <v>46461</v>
       </c>
       <c r="C52" s="16" t="n">
+        <v>0.708333333333333</v>
+      </c>
+      <c r="D52" s="16" t="n">
         <v>0.715277777777778</v>
-      </c>
-      <c r="D52" s="16" t="n">
-        <v>0.736111111111111</v>
       </c>
       <c r="E52" s="14" t="n">
         <f aca="false">ROUND((D52-C52)*1440,0)</f>
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="F52" s="14" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="G52" s="14" t="s">
-        <v>122</v>
-      </c>
-      <c r="H52" s="14"/>
-      <c r="I52" s="14"/>
+        <v>120</v>
+      </c>
+      <c r="H52" s="14" t="s">
+        <v>123</v>
+      </c>
+      <c r="I52" s="14" t="n">
+        <v>1</v>
+      </c>
       <c r="J52" s="14" t="s">
         <v>124</v>
       </c>
@@ -4532,29 +4529,25 @@
         <v>46461</v>
       </c>
       <c r="C53" s="16" t="n">
+        <v>0.715277777777778</v>
+      </c>
+      <c r="D53" s="16" t="n">
         <v>0.736111111111111</v>
-      </c>
-      <c r="D53" s="16" t="n">
-        <v>0.746527777777778</v>
       </c>
       <c r="E53" s="14" t="n">
         <f aca="false">ROUND((D53-C53)*1440,0)</f>
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F53" s="14" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="G53" s="14" t="s">
-        <v>122</v>
-      </c>
-      <c r="H53" s="14" t="s">
+        <v>123</v>
+      </c>
+      <c r="H53" s="14"/>
+      <c r="I53" s="14"/>
+      <c r="J53" s="14" t="s">
         <v>125</v>
-      </c>
-      <c r="I53" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="J53" s="14" t="s">
-        <v>126</v>
       </c>
       <c r="K53" s="17" t="s">
         <v>42</v>
@@ -4569,25 +4562,29 @@
         <v>46461</v>
       </c>
       <c r="C54" s="16" t="n">
+        <v>0.736111111111111</v>
+      </c>
+      <c r="D54" s="16" t="n">
         <v>0.746527777777778</v>
-      </c>
-      <c r="D54" s="16" t="n">
-        <v>0.8125</v>
       </c>
       <c r="E54" s="14" t="n">
         <f aca="false">ROUND((D54-C54)*1440,0)</f>
-        <v>95</v>
+        <v>15</v>
       </c>
       <c r="F54" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="G54" s="14" t="s">
+        <v>123</v>
+      </c>
+      <c r="H54" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="I54" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="J54" s="14" t="s">
         <v>127</v>
-      </c>
-      <c r="G54" s="14" t="s">
-        <v>125</v>
-      </c>
-      <c r="H54" s="14"/>
-      <c r="I54" s="14"/>
-      <c r="J54" s="14" t="s">
-        <v>128</v>
       </c>
       <c r="K54" s="17" t="s">
         <v>42</v>
@@ -4602,90 +4599,90 @@
         <v>46461</v>
       </c>
       <c r="C55" s="16" t="n">
+        <v>0.746527777777778</v>
+      </c>
+      <c r="D55" s="16" t="n">
         <v>0.8125</v>
-      </c>
-      <c r="D55" s="16" t="n">
-        <v>0.822916666666667</v>
       </c>
       <c r="E55" s="14" t="n">
         <f aca="false">ROUND((D55-C55)*1440,0)</f>
-        <v>15</v>
+        <v>95</v>
       </c>
       <c r="F55" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="G55" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="H55" s="14"/>
+      <c r="I55" s="14"/>
+      <c r="J55" s="14" t="s">
         <v>129</v>
-      </c>
-      <c r="G55" s="14" t="s">
-        <v>125</v>
-      </c>
-      <c r="H55" s="14" t="s">
-        <v>115</v>
-      </c>
-      <c r="I55" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="J55" s="14" t="s">
-        <v>130</v>
       </c>
       <c r="K55" s="17" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="11" t="n">
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="B56" s="12" t="n">
+      <c r="B56" s="15" t="n">
         <f aca="false">Overview!$B$3+A56-1</f>
         <v>46461</v>
       </c>
-      <c r="C56" s="13" t="n">
-        <v>0.833333333333333</v>
-      </c>
-      <c r="D56" s="13" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="E56" s="11" t="n">
+      <c r="C56" s="16" t="n">
+        <v>0.8125</v>
+      </c>
+      <c r="D56" s="16" t="n">
+        <v>0.822916666666667</v>
+      </c>
+      <c r="E56" s="14" t="n">
         <f aca="false">ROUND((D56-C56)*1440,0)</f>
-        <v>60</v>
-      </c>
-      <c r="F56" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="G56" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="F56" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="G56" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="H56" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="I56" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J56" s="14" t="s">
         <v>131</v>
       </c>
-      <c r="H56" s="11"/>
-      <c r="I56" s="11"/>
-      <c r="J56" s="11" t="s">
-        <v>132</v>
-      </c>
-      <c r="K56" s="18" t="s">
+      <c r="K56" s="17" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B57" s="12" t="n">
         <f aca="false">Overview!$B$3+A57-1</f>
-        <v>46462</v>
+        <v>46461</v>
       </c>
       <c r="C57" s="13" t="n">
-        <v>0.291666666666667</v>
+        <v>0.833333333333333</v>
       </c>
       <c r="D57" s="13" t="n">
-        <v>0.319444444444444</v>
+        <v>0.875</v>
       </c>
       <c r="E57" s="11" t="n">
         <f aca="false">ROUND((D57-C57)*1440,0)</f>
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="F57" s="11" t="s">
-        <v>36</v>
+        <v>70</v>
       </c>
       <c r="G57" s="11" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H57" s="11"/>
       <c r="I57" s="11"/>
@@ -4697,39 +4694,39 @@
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="14" t="n">
+      <c r="A58" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="B58" s="15" t="n">
+      <c r="B58" s="12" t="n">
         <f aca="false">Overview!$B$3+A58-1</f>
         <v>46462</v>
       </c>
-      <c r="C58" s="16" t="n">
-        <v>0.319444444444444</v>
-      </c>
-      <c r="D58" s="16" t="n">
-        <v>0.333333333333333</v>
-      </c>
-      <c r="E58" s="14" t="n">
+      <c r="C58" s="13" t="n">
+        <v>0.3125</v>
+      </c>
+      <c r="D58" s="13" t="n">
+        <v>0.354166666666667</v>
+      </c>
+      <c r="E58" s="11" t="n">
         <f aca="false">ROUND((D58-C58)*1440,0)</f>
-        <v>20</v>
-      </c>
-      <c r="F58" s="14" t="s">
-        <v>47</v>
-      </c>
-      <c r="G58" s="14" t="s">
-        <v>115</v>
-      </c>
-      <c r="H58" s="14"/>
-      <c r="I58" s="14"/>
-      <c r="J58" s="14" t="s">
-        <v>134</v>
-      </c>
-      <c r="K58" s="17" t="s">
+        <v>60</v>
+      </c>
+      <c r="F58" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="G58" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="H58" s="11"/>
+      <c r="I58" s="11"/>
+      <c r="J58" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="K58" s="18" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="14" t="n">
         <v>4</v>
       </c>
@@ -4738,35 +4735,31 @@
         <v>46462</v>
       </c>
       <c r="C59" s="16" t="n">
-        <v>0.333333333333333</v>
+        <v>0.354166666666667</v>
       </c>
       <c r="D59" s="16" t="n">
-        <v>0.395833333333333</v>
+        <v>0.375</v>
       </c>
       <c r="E59" s="14" t="n">
         <f aca="false">ROUND((D59-C59)*1440,0)</f>
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="F59" s="14" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="G59" s="14" t="s">
-        <v>115</v>
-      </c>
-      <c r="H59" s="14" t="s">
-        <v>44</v>
-      </c>
-      <c r="I59" s="14" t="n">
-        <v>50</v>
-      </c>
+        <v>116</v>
+      </c>
+      <c r="H59" s="14"/>
+      <c r="I59" s="14"/>
       <c r="J59" s="14" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="K59" s="17" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="14" t="n">
         <v>4</v>
       </c>
@@ -4775,37 +4768,74 @@
         <v>46462</v>
       </c>
       <c r="C60" s="16" t="n">
-        <v>0.395833333333333</v>
+        <v>0.375</v>
       </c>
       <c r="D60" s="16" t="n">
-        <v>0.416666666666667</v>
+        <v>0.4375</v>
       </c>
       <c r="E60" s="14" t="n">
         <f aca="false">ROUND((D60-C60)*1440,0)</f>
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="F60" s="14" t="s">
-        <v>136</v>
+        <v>43</v>
       </c>
       <c r="G60" s="14" t="s">
-        <v>137</v>
-      </c>
-      <c r="H60" s="14"/>
-      <c r="I60" s="14"/>
+        <v>116</v>
+      </c>
+      <c r="H60" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="I60" s="14" t="n">
+        <v>50</v>
+      </c>
       <c r="J60" s="14" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="K60" s="17" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="5" t="s">
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="B61" s="15" t="n">
+        <f aca="false">Overview!$B$3+A61-1</f>
+        <v>46462</v>
+      </c>
+      <c r="C61" s="16" t="n">
+        <v>0.4375</v>
+      </c>
+      <c r="D61" s="16" t="n">
+        <v>0.458333333333333</v>
+      </c>
+      <c r="E61" s="14" t="n">
+        <f aca="false">ROUND((D61-C61)*1440,0)</f>
+        <v>30</v>
+      </c>
+      <c r="F61" s="14" t="s">
+        <v>136</v>
+      </c>
+      <c r="G61" s="14" t="s">
+        <v>137</v>
+      </c>
+      <c r="H61" s="14"/>
+      <c r="I61" s="14"/>
+      <c r="J61" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="K61" s="17" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="5" t="s">
         <v>139</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:K60"/>
+  <autoFilter ref="A4:K61"/>
   <hyperlinks>
     <hyperlink ref="K6" r:id="rId1" display="Open map"/>
     <hyperlink ref="K7" r:id="rId2" display="Open map"/>
@@ -4862,6 +4892,7 @@
     <hyperlink ref="K58" r:id="rId53" display="Open map"/>
     <hyperlink ref="K59" r:id="rId54" display="Open map"/>
     <hyperlink ref="K60" r:id="rId55" display="Open map"/>
+    <hyperlink ref="K61" r:id="rId56" display="Open map"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -4870,7 +4901,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId56"/>
+  <drawing r:id="rId57"/>
 </worksheet>
 </file>
 
@@ -5043,7 +5074,7 @@
         <v>36</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="D10" s="14" t="s">
         <v>159</v>
@@ -5063,7 +5094,7 @@
         <v>50</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="D11" s="14" t="s">
         <v>164</v>
@@ -5086,7 +5117,7 @@
         <v>166</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E12" s="14" t="s">
         <v>154</v>
@@ -5103,10 +5134,10 @@
         <v>36</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>167</v>
+        <v>155</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E13" s="14" t="s">
         <v>156</v>
@@ -5126,7 +5157,7 @@
         <v>22</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E14" s="14" t="s">
         <v>156</v>
@@ -5160,13 +5191,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
+        <v>168</v>
+      </c>
+      <c r="B1" s="10" t="s">
         <v>169</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="C1" s="10" t="s">
         <v>170</v>
-      </c>
-      <c r="C1" s="10" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5174,76 +5205,76 @@
         <v>83</v>
       </c>
       <c r="B2" s="14" t="s">
+        <v>171</v>
+      </c>
+      <c r="C2" s="14" t="s">
         <v>172</v>
-      </c>
-      <c r="C2" s="14" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
+        <v>173</v>
+      </c>
+      <c r="B3" s="14" t="s">
         <v>174</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="C3" s="14" t="s">
         <v>175</v>
-      </c>
-      <c r="C3" s="14" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="B4" s="14" t="s">
         <v>177</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="C4" s="14" t="s">
         <v>178</v>
-      </c>
-      <c r="C4" s="14" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
+        <v>179</v>
+      </c>
+      <c r="B5" s="14" t="s">
         <v>180</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="C5" s="14" t="s">
         <v>181</v>
-      </c>
-      <c r="C5" s="14" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
+        <v>182</v>
+      </c>
+      <c r="B6" s="14" t="s">
         <v>183</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="C6" s="14" t="s">
         <v>184</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
+        <v>185</v>
+      </c>
+      <c r="B7" s="14" t="s">
         <v>186</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="C7" s="14" t="s">
         <v>187</v>
-      </c>
-      <c r="C7" s="14" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
+        <v>188</v>
+      </c>
+      <c r="B8" s="14" t="s">
         <v>189</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="C8" s="14" t="s">
         <v>190</v>
-      </c>
-      <c r="C8" s="14" t="s">
-        <v>191</v>
       </c>
     </row>
   </sheetData>
@@ -5273,184 +5304,184 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
+        <v>191</v>
+      </c>
+      <c r="B1" s="10" t="s">
         <v>192</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="C1" s="10" t="s">
         <v>193</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="D1" s="10" t="s">
         <v>194</v>
-      </c>
-      <c r="D1" s="10" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="B2" s="14" t="s">
         <v>196</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="C2" s="14" t="s">
         <v>197</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="D2" s="14" t="s">
         <v>198</v>
-      </c>
-      <c r="D2" s="14" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
+        <v>199</v>
+      </c>
+      <c r="B3" s="14" t="s">
         <v>200</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="C3" s="14" t="s">
         <v>201</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="D3" s="14" t="s">
         <v>202</v>
-      </c>
-      <c r="D3" s="14" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
+        <v>203</v>
+      </c>
+      <c r="B4" s="14" t="s">
         <v>204</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="C4" s="14" t="s">
         <v>205</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="D4" s="14" t="s">
         <v>206</v>
-      </c>
-      <c r="D4" s="14" t="s">
-        <v>207</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
+        <v>207</v>
+      </c>
+      <c r="B5" s="14" t="s">
         <v>208</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="C5" s="14" t="s">
         <v>209</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="D5" s="14" t="s">
         <v>210</v>
-      </c>
-      <c r="D5" s="14" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
+        <v>211</v>
+      </c>
+      <c r="B6" s="14" t="s">
         <v>212</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="C6" s="14" t="s">
         <v>213</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="D6" s="14" t="s">
         <v>214</v>
-      </c>
-      <c r="D6" s="14" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
+        <v>215</v>
+      </c>
+      <c r="B7" s="14" t="s">
         <v>216</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="C7" s="14" t="s">
         <v>217</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="D7" s="14" t="s">
         <v>218</v>
-      </c>
-      <c r="D7" s="14" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
+        <v>219</v>
+      </c>
+      <c r="B8" s="14" t="s">
         <v>220</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="C8" s="14" t="s">
         <v>221</v>
       </c>
-      <c r="C8" s="14" t="s">
+      <c r="D8" s="14" t="s">
         <v>222</v>
-      </c>
-      <c r="D8" s="14" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
+        <v>223</v>
+      </c>
+      <c r="B9" s="14" t="s">
         <v>224</v>
       </c>
-      <c r="B9" s="14" t="s">
+      <c r="C9" s="14" t="s">
         <v>225</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="D9" s="14" t="s">
         <v>226</v>
-      </c>
-      <c r="D9" s="14" t="s">
-        <v>227</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
+        <v>227</v>
+      </c>
+      <c r="B10" s="14" t="s">
         <v>228</v>
       </c>
-      <c r="B10" s="14" t="s">
+      <c r="C10" s="14" t="s">
         <v>229</v>
       </c>
-      <c r="C10" s="14" t="s">
+      <c r="D10" s="14" t="s">
         <v>230</v>
-      </c>
-      <c r="D10" s="14" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
+        <v>231</v>
+      </c>
+      <c r="B11" s="14" t="s">
         <v>232</v>
       </c>
-      <c r="B11" s="14" t="s">
+      <c r="C11" s="14" t="s">
         <v>233</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="D11" s="14" t="s">
         <v>234</v>
-      </c>
-      <c r="D11" s="14" t="s">
-        <v>235</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
+        <v>235</v>
+      </c>
+      <c r="B12" s="14" t="s">
         <v>236</v>
       </c>
-      <c r="B12" s="14" t="s">
+      <c r="C12" s="14" t="s">
         <v>237</v>
       </c>
-      <c r="C12" s="14" t="s">
+      <c r="D12" s="14" t="s">
         <v>238</v>
-      </c>
-      <c r="D12" s="14" t="s">
-        <v>239</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
+        <v>239</v>
+      </c>
+      <c r="B13" s="14" t="s">
         <v>240</v>
       </c>
-      <c r="B13" s="14" t="s">
+      <c r="C13" s="14" t="s">
         <v>241</v>
       </c>
-      <c r="C13" s="14" t="s">
+      <c r="D13" s="14" t="s">
         <v>242</v>
-      </c>
-      <c r="D13" s="14" t="s">
-        <v>243</v>
       </c>
     </row>
   </sheetData>
@@ -5478,202 +5509,202 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
+        <v>243</v>
+      </c>
+      <c r="B1" s="10" t="s">
         <v>244</v>
-      </c>
-      <c r="B1" s="10" t="s">
-        <v>245</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
+        <v>245</v>
+      </c>
+      <c r="B2" s="14" t="s">
         <v>246</v>
-      </c>
-      <c r="B2" s="14" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
+        <v>255</v>
+      </c>
+      <c r="B11" s="14" t="s">
         <v>256</v>
-      </c>
-      <c r="B11" s="14" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
+        <v>263</v>
+      </c>
+      <c r="B18" s="14" t="s">
         <v>264</v>
-      </c>
-      <c r="B18" s="14" t="s">
-        <v>265</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="14" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="14" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="14" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="14" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="14" t="s">
+        <v>269</v>
+      </c>
+      <c r="B23" s="14" t="s">
         <v>270</v>
-      </c>
-      <c r="B23" s="14" t="s">
-        <v>271</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="14" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="14" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B25" s="14" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
   </sheetData>
@@ -5704,221 +5735,221 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
+        <v>274</v>
+      </c>
+      <c r="B3" s="10" t="s">
         <v>275</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="C3" s="10" t="s">
         <v>276</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="D3" s="10" t="s">
         <v>277</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="E3" s="10" t="s">
         <v>278</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>279</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
+        <v>279</v>
+      </c>
+      <c r="B4" s="14" t="s">
         <v>280</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="C4" s="14" t="s">
         <v>281</v>
-      </c>
-      <c r="C4" s="14" t="s">
-        <v>282</v>
       </c>
       <c r="D4" s="14"/>
       <c r="E4" s="23"/>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
+        <v>282</v>
+      </c>
+      <c r="B5" s="14" t="s">
         <v>283</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="C5" s="14" t="s">
+        <v>281</v>
+      </c>
+      <c r="D5" s="14" t="s">
         <v>284</v>
-      </c>
-      <c r="C5" s="14" t="s">
-        <v>282</v>
-      </c>
-      <c r="D5" s="14" t="s">
-        <v>285</v>
       </c>
       <c r="E5" s="23"/>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
+        <v>285</v>
+      </c>
+      <c r="B6" s="14" t="s">
         <v>286</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="C6" s="14" t="s">
+        <v>281</v>
+      </c>
+      <c r="D6" s="14" t="s">
         <v>287</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>282</v>
-      </c>
-      <c r="D6" s="14" t="s">
-        <v>288</v>
       </c>
       <c r="E6" s="23"/>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
+        <v>288</v>
+      </c>
+      <c r="B7" s="14" t="s">
         <v>289</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="C7" s="14" t="s">
         <v>290</v>
-      </c>
-      <c r="C7" s="14" t="s">
-        <v>291</v>
       </c>
       <c r="D7" s="14"/>
       <c r="E7" s="23"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
+        <v>291</v>
+      </c>
+      <c r="B8" s="14" t="s">
         <v>292</v>
       </c>
-      <c r="B8" s="14" t="s">
-        <v>293</v>
-      </c>
       <c r="C8" s="14" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="D8" s="14"/>
       <c r="E8" s="23"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="D9" s="14"/>
       <c r="E9" s="23"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
+        <v>294</v>
+      </c>
+      <c r="B10" s="14" t="s">
         <v>295</v>
       </c>
-      <c r="B10" s="14" t="s">
+      <c r="C10" s="14" t="s">
         <v>296</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>297</v>
       </c>
       <c r="D10" s="14"/>
       <c r="E10" s="23"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="D11" s="14"/>
       <c r="E11" s="23"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
+        <v>298</v>
+      </c>
+      <c r="B12" s="14" t="s">
         <v>299</v>
       </c>
-      <c r="B12" s="14" t="s">
-        <v>300</v>
-      </c>
       <c r="C12" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="D12" s="14"/>
       <c r="E12" s="23"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
+        <v>300</v>
+      </c>
+      <c r="B13" s="14" t="s">
         <v>301</v>
       </c>
-      <c r="B13" s="14" t="s">
+      <c r="C13" s="14" t="s">
         <v>302</v>
-      </c>
-      <c r="C13" s="14" t="s">
-        <v>303</v>
       </c>
       <c r="D13" s="14"/>
       <c r="E13" s="23"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="D14" s="14"/>
       <c r="E14" s="23"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
+        <v>304</v>
+      </c>
+      <c r="B15" s="14" t="s">
         <v>305</v>
       </c>
-      <c r="B15" s="14" t="s">
-        <v>306</v>
-      </c>
       <c r="C15" s="14" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="D15" s="14"/>
       <c r="E15" s="23"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
+        <v>306</v>
+      </c>
+      <c r="B16" s="14" t="s">
         <v>307</v>
       </c>
-      <c r="B16" s="14" t="s">
-        <v>308</v>
-      </c>
       <c r="C16" s="14" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="D16" s="14"/>
       <c r="E16" s="23"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
+        <v>308</v>
+      </c>
+      <c r="B17" s="14" t="s">
         <v>309</v>
       </c>
-      <c r="B17" s="14" t="s">
-        <v>310</v>
-      </c>
       <c r="C17" s="14" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="D17" s="14"/>
       <c r="E17" s="23"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
+        <v>310</v>
+      </c>
+      <c r="B18" s="14" t="s">
         <v>311</v>
       </c>
-      <c r="B18" s="14" t="s">
-        <v>312</v>
-      </c>
       <c r="C18" s="14" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="D18" s="14"/>
       <c r="E18" s="23"/>
@@ -5948,146 +5979,146 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
+        <v>312</v>
+      </c>
+      <c r="B1" s="10" t="s">
         <v>313</v>
-      </c>
-      <c r="B1" s="10" t="s">
-        <v>314</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
+        <v>314</v>
+      </c>
+      <c r="B2" s="14" t="s">
         <v>315</v>
-      </c>
-      <c r="B2" s="14" t="s">
-        <v>316</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
+        <v>322</v>
+      </c>
+      <c r="B9" s="14" t="s">
         <v>323</v>
-      </c>
-      <c r="B9" s="14" t="s">
-        <v>324</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
+        <v>329</v>
+      </c>
+      <c r="B15" s="14" t="s">
         <v>330</v>
-      </c>
-      <c r="B15" s="14" t="s">
-        <v>331</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
+        <v>331</v>
+      </c>
+      <c r="B16" s="14" t="s">
         <v>332</v>
-      </c>
-      <c r="B16" s="14" t="s">
-        <v>333</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
+        <v>333</v>
+      </c>
+      <c r="B17" s="14" t="s">
         <v>334</v>
-      </c>
-      <c r="B17" s="14" t="s">
-        <v>335</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
+        <v>335</v>
+      </c>
+      <c r="B18" s="14" t="s">
         <v>336</v>
-      </c>
-      <c r="B18" s="14" t="s">
-        <v>337</v>
       </c>
     </row>
   </sheetData>
@@ -6115,34 +6146,34 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
+        <v>337</v>
+      </c>
+      <c r="B1" s="10" t="s">
         <v>338</v>
-      </c>
-      <c r="B1" s="10" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
+        <v>339</v>
+      </c>
+      <c r="B2" s="14" t="s">
         <v>340</v>
-      </c>
-      <c r="B2" s="14" t="s">
-        <v>341</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
+        <v>341</v>
+      </c>
+      <c r="B3" s="14" t="s">
         <v>342</v>
-      </c>
-      <c r="B3" s="14" t="s">
-        <v>343</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
+        <v>343</v>
+      </c>
+      <c r="B4" s="14" t="s">
         <v>344</v>
-      </c>
-      <c r="B4" s="14" t="s">
-        <v>345</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6150,55 +6181,55 @@
         <v>83</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
+        <v>346</v>
+      </c>
+      <c r="B6" s="14" t="s">
         <v>347</v>
-      </c>
-      <c r="B6" s="14" t="s">
-        <v>348</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
+        <v>348</v>
+      </c>
+      <c r="B7" s="14" t="s">
         <v>349</v>
-      </c>
-      <c r="B7" s="14" t="s">
-        <v>350</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
+        <v>350</v>
+      </c>
+      <c r="B8" s="14" t="s">
         <v>351</v>
-      </c>
-      <c r="B8" s="14" t="s">
-        <v>352</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
+        <v>352</v>
+      </c>
+      <c r="B9" s="14" t="s">
         <v>353</v>
-      </c>
-      <c r="B9" s="14" t="s">
-        <v>354</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
+        <v>354</v>
+      </c>
+      <c r="B10" s="14" t="s">
         <v>355</v>
-      </c>
-      <c r="B10" s="14" t="s">
-        <v>356</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
+        <v>356</v>
+      </c>
+      <c r="B11" s="14" t="s">
         <v>357</v>
-      </c>
-      <c r="B11" s="14" t="s">
-        <v>358</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add flight info to both packages and re-plan Day 4 and Day 8
3N/4D: arrive Jammu before 14:00 on 13 Mar, depart Jammu after 14:00 on
16 Mar; Day 4 adds Kol Kandoli Mata (Nagrota) and an early lunch near
the airport (146 km).
7N/8D: Jammu-Srinagar flight 11:00-12:00 on 16 Mar; Shankaracharya and
Jyeshta Devi move to the Day 4 afternoon; Day 8 goes Pahalgam - Pampore
- Srinagar Airport for flights after 14:00 on 20 Mar (643 km).
Workbooks and brochures updated; 8-day meal plan gets its own page.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A4yYiJq592wzPacq5vAVkN
</commit_message>
<xml_diff>
--- a/docs/itineraries/vaishno-devi-helicopter-4d-plan.xlsx
+++ b/docs/itineraries/vaishno-devi-helicopter-4d-plan.xlsx
@@ -23,7 +23,7 @@
     <sheet name="Open Points" sheetId="13" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Minute-by-Minute'!$A$4:$K$61</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Minute-by-Minute'!$A$4:$K$65</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="707" uniqueCount="452">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="731" uniqueCount="463">
   <si>
     <t xml:space="preserve">Vaishno Devi Helicopter Yatra – Overview</t>
   </si>
@@ -100,15 +100,24 @@
     <t xml:space="preserve">Katra</t>
   </si>
   <si>
-    <t xml:space="preserve">Katra → Jammu departure</t>
+    <t xml:space="preserve">Katra → Kol Kandoli (Nagrota) → Jammu departure</t>
   </si>
   <si>
     <t xml:space="preserve">—</t>
   </si>
   <si>
+    <t xml:space="preserve">Flight info</t>
+  </si>
+  <si>
     <t xml:space="preserve">Total</t>
   </si>
   <si>
+    <t xml:space="preserve">Arrival at Jammu Airport on 13 March 2027 before 14:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Departure from Jammu Airport on 16 March 2027 after 14:00</t>
+  </si>
+  <si>
     <t xml:space="preserve">Other transport: 2 helicopter flights (5–8 min each), Bhairon ropeway, ~5.5 km on the mountain track (2.5 km Day 2, ~3 km Day 3).</t>
   </si>
   <si>
@@ -439,19 +448,37 @@
     <t xml:space="preserve">Dinner – at the hotel, pre-ordered pure-veg menu; group pays; Day 4 briefing</t>
   </si>
   <si>
-    <t xml:space="preserve">Check-out, load luggage; collect packed lunch for the journey</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Drive to Jammu (Jammu Tawi station ~48 km; SMVD Katra station only 2 km)</t>
+    <t xml:space="preserve">Kol Kandoli Mata Temple, Nagrota</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drive towards Jammu on the Katra–Jammu highway</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Darshan of Mata in her child form – traditionally the first stop of the Vaishno Devi yatra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nagrota</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pure-veg restaurant near Jammu Airport</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drive into Jammu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Early lunch – pre-booked pure-veg restaurant; group pays</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Restaurant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Short drive to the terminal</t>
   </si>
   <si>
     <t xml:space="preserve">Departure</t>
   </si>
   <si>
-    <t xml:space="preserve">Jammu Airport / Jammu Tawi Rly Stn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Drop-off, farewell, Jai Mata Di! (book return flights / trains after 12:30)</t>
+    <t xml:space="preserve">Drop-off, farewell, Jai Mata Di! (return flights depart after 14:00)</t>
   </si>
   <si>
     <t xml:space="preserve">Legend: yellow rows = meals, blue rows = helicopter / ropeway.</t>
@@ -538,7 +565,10 @@
     <t xml:space="preserve">20:00–21:00</t>
   </si>
   <si>
-    <t xml:space="preserve">Packed from Katra hotel for onward travel after 12:30</t>
+    <t xml:space="preserve">11:15–12:15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Restaurant, pre-booked</t>
   </si>
   <si>
     <t xml:space="preserve">Aspect</t>
@@ -595,7 +625,7 @@
     <t xml:space="preserve">Overall pace</t>
   </si>
   <si>
-    <t xml:space="preserve">3 nights only; little road travel (143 km)</t>
+    <t xml:space="preserve">3 nights only; little road travel (146 km)</t>
   </si>
   <si>
     <t xml:space="preserve">Early starts on Days 2 and 3 (04:30 wake-up at Bhawan)</t>
@@ -922,7 +952,7 @@
     <t xml:space="preserve">T−45 days</t>
   </si>
   <si>
-    <t xml:space="preserve">Book flights / trains: arrival by 14:00 on Day 1; departure after 12:30 Day 4</t>
+    <t xml:space="preserve">Book flights / trains: arrival before 14:00 on 13 Mar; departure after 14:00 on 16 Mar</t>
   </si>
   <si>
     <t xml:space="preserve">Travel desk</t>
@@ -1318,7 +1348,7 @@
     <t xml:space="preserve">Atka Aarti passes</t>
   </si>
   <si>
-    <t xml:space="preserve">Vehicles, 4 days (143 km + waiting)</t>
+    <t xml:space="preserve">Vehicles, 4 days (146 km + waiting)</t>
   </si>
   <si>
     <t xml:space="preserve">Per vehicle, split by seats</t>
@@ -1328,6 +1358,9 @@
   </si>
   <si>
     <t xml:space="preserve">Per plate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lunch Day 4 (restaurant)</t>
   </si>
   <si>
     <t xml:space="preserve">Dinners Day 1 and Day 3 (hotels)</t>
@@ -2053,18 +2086,18 @@
         <v>13</v>
       </c>
       <c r="D5" s="7" t="n">
-        <f aca="false">SUMIF('Minute-by-Minute'!$A$5:$A$61,A5,'Minute-by-Minute'!$I$5:$I$61)</f>
+        <f aca="false">SUMIF('Minute-by-Minute'!$A$5:$A$65,A5,'Minute-by-Minute'!$I$5:$I$65)</f>
         <v>32</v>
       </c>
       <c r="E5" s="7" t="s">
         <v>14</v>
       </c>
       <c r="F5" s="9" t="n">
-        <f aca="false">_xlfn.MINIFS('Minute-by-Minute'!$C$5:$C$61,'Minute-by-Minute'!$A$5:$A$61,A5)</f>
+        <f aca="false">_xlfn.MINIFS('Minute-by-Minute'!$C$5:$C$65,'Minute-by-Minute'!$A$5:$A$65,A5)</f>
         <v>0.333333333333333</v>
       </c>
       <c r="G5" s="9" t="n">
-        <f aca="false">_xlfn.MAXIFS('Minute-by-Minute'!$D$5:$D$61,'Minute-by-Minute'!$A$5:$A$61,A5)</f>
+        <f aca="false">_xlfn.MAXIFS('Minute-by-Minute'!$D$5:$D$65,'Minute-by-Minute'!$A$5:$A$65,A5)</f>
         <v>0.885416666666667</v>
       </c>
       <c r="I5" s="7" t="s">
@@ -2086,18 +2119,18 @@
         <v>16</v>
       </c>
       <c r="D6" s="7" t="n">
-        <f aca="false">SUMIF('Minute-by-Minute'!$A$5:$A$61,A6,'Minute-by-Minute'!$I$5:$I$61)</f>
+        <f aca="false">SUMIF('Minute-by-Minute'!$A$5:$A$65,A6,'Minute-by-Minute'!$I$5:$I$65)</f>
         <v>52</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>17</v>
       </c>
       <c r="F6" s="9" t="n">
-        <f aca="false">_xlfn.MINIFS('Minute-by-Minute'!$C$5:$C$61,'Minute-by-Minute'!$A$5:$A$61,A6)</f>
+        <f aca="false">_xlfn.MINIFS('Minute-by-Minute'!$C$5:$C$65,'Minute-by-Minute'!$A$5:$A$65,A6)</f>
         <v>0.3125</v>
       </c>
       <c r="G6" s="9" t="n">
-        <f aca="false">_xlfn.MAXIFS('Minute-by-Minute'!$D$5:$D$61,'Minute-by-Minute'!$A$5:$A$61,A6)</f>
+        <f aca="false">_xlfn.MAXIFS('Minute-by-Minute'!$D$5:$D$65,'Minute-by-Minute'!$A$5:$A$65,A6)</f>
         <v>0.854166666666667</v>
       </c>
       <c r="I6" s="7" t="s">
@@ -2119,18 +2152,18 @@
         <v>19</v>
       </c>
       <c r="D7" s="7" t="n">
-        <f aca="false">SUMIF('Minute-by-Minute'!$A$5:$A$61,A7,'Minute-by-Minute'!$I$5:$I$61)</f>
+        <f aca="false">SUMIF('Minute-by-Minute'!$A$5:$A$65,A7,'Minute-by-Minute'!$I$5:$I$65)</f>
         <v>9</v>
       </c>
       <c r="E7" s="7" t="s">
         <v>20</v>
       </c>
       <c r="F7" s="9" t="n">
-        <f aca="false">_xlfn.MINIFS('Minute-by-Minute'!$C$5:$C$61,'Minute-by-Minute'!$A$5:$A$61,A7)</f>
+        <f aca="false">_xlfn.MINIFS('Minute-by-Minute'!$C$5:$C$65,'Minute-by-Minute'!$A$5:$A$65,A7)</f>
         <v>0.1875</v>
       </c>
       <c r="G7" s="9" t="n">
-        <f aca="false">_xlfn.MAXIFS('Minute-by-Minute'!$D$5:$D$61,'Minute-by-Minute'!$A$5:$A$61,A7)</f>
+        <f aca="false">_xlfn.MAXIFS('Minute-by-Minute'!$D$5:$D$65,'Minute-by-Minute'!$A$5:$A$65,A7)</f>
         <v>0.875</v>
       </c>
     </row>
@@ -2146,38 +2179,49 @@
         <v>21</v>
       </c>
       <c r="D8" s="7" t="n">
-        <f aca="false">SUMIF('Minute-by-Minute'!$A$5:$A$61,A8,'Minute-by-Minute'!$I$5:$I$61)</f>
-        <v>50</v>
+        <f aca="false">SUMIF('Minute-by-Minute'!$A$5:$A$65,A8,'Minute-by-Minute'!$I$5:$I$65)</f>
+        <v>53</v>
       </c>
       <c r="E8" s="7" t="s">
         <v>22</v>
       </c>
       <c r="F8" s="9" t="n">
-        <f aca="false">_xlfn.MINIFS('Minute-by-Minute'!$C$5:$C$61,'Minute-by-Minute'!$A$5:$A$61,A8)</f>
+        <f aca="false">_xlfn.MINIFS('Minute-by-Minute'!$C$5:$C$65,'Minute-by-Minute'!$A$5:$A$65,A8)</f>
         <v>0.3125</v>
       </c>
       <c r="G8" s="9" t="n">
-        <f aca="false">_xlfn.MAXIFS('Minute-by-Minute'!$D$5:$D$61,'Minute-by-Minute'!$A$5:$A$61,A8)</f>
-        <v>0.458333333333333</v>
+        <f aca="false">_xlfn.MAXIFS('Minute-by-Minute'!$D$5:$D$65,'Minute-by-Minute'!$A$5:$A$65,A8)</f>
+        <v>0.541666666666667</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D9" s="3" t="n">
         <f aca="false">SUM(D5:D8)</f>
-        <v>143</v>
+        <v>146</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I10" s="2" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -2208,121 +2252,121 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>358</v>
+        <v>368</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>359</v>
+        <v>369</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>360</v>
+        <v>370</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>362</v>
+        <v>372</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>363</v>
+        <v>373</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>364</v>
+        <v>374</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>365</v>
+        <v>375</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>169</v>
+        <v>179</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>366</v>
+        <v>376</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>367</v>
+        <v>377</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>368</v>
+        <v>378</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>369</v>
+        <v>379</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>169</v>
+        <v>179</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>370</v>
+        <v>380</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>371</v>
+        <v>381</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>372</v>
+        <v>382</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>373</v>
+        <v>383</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>374</v>
+        <v>384</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>375</v>
+        <v>385</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>376</v>
+        <v>386</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>377</v>
+        <v>387</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>378</v>
+        <v>388</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>379</v>
+        <v>389</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>380</v>
+        <v>390</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>335</v>
+        <v>345</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>381</v>
+        <v>391</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>382</v>
+        <v>392</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>169</v>
+        <v>179</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>366</v>
+        <v>376</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>329</v>
+        <v>339</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>383</v>
+        <v>393</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>384</v>
+        <v>394</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>385</v>
+        <v>395</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>386</v>
+        <v>396</v>
       </c>
     </row>
   </sheetData>
@@ -2352,81 +2396,81 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>387</v>
+        <v>397</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>388</v>
+        <v>398</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>389</v>
+        <v>399</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>390</v>
+        <v>400</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>302</v>
+        <v>312</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>391</v>
+        <v>401</v>
       </c>
       <c r="C2" s="23"/>
       <c r="D2" s="23"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>392</v>
+        <v>402</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>393</v>
+        <v>403</v>
       </c>
       <c r="C3" s="23"/>
       <c r="D3" s="23"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>394</v>
+        <v>404</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>395</v>
+        <v>405</v>
       </c>
       <c r="C4" s="23"/>
       <c r="D4" s="23"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>396</v>
+        <v>406</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>397</v>
+        <v>407</v>
       </c>
       <c r="C5" s="23"/>
       <c r="D5" s="23"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>398</v>
+        <v>408</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>399</v>
+        <v>409</v>
       </c>
       <c r="C6" s="23"/>
       <c r="D6" s="23"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>400</v>
+        <v>410</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>401</v>
+        <v>411</v>
       </c>
       <c r="C7" s="23"/>
       <c r="D7" s="23"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B8" s="14"/>
       <c r="C8" s="23"/>
@@ -2434,7 +2478,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="B9" s="14"/>
       <c r="C9" s="23"/>
@@ -2442,7 +2486,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>402</v>
+        <v>412</v>
       </c>
       <c r="B10" s="14"/>
       <c r="C10" s="23"/>
@@ -2450,7 +2494,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>403</v>
+        <v>413</v>
       </c>
       <c r="B11" s="14"/>
       <c r="C11" s="23"/>
@@ -2458,7 +2502,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>404</v>
+        <v>414</v>
       </c>
       <c r="B12" s="14"/>
       <c r="C12" s="23"/>
@@ -2466,14 +2510,14 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>405</v>
+        <v>415</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>406</v>
+        <v>416</v>
       </c>
       <c r="C13" s="14"/>
       <c r="D13" s="14" t="s">
-        <v>407</v>
+        <v>417</v>
       </c>
     </row>
   </sheetData>
@@ -2492,7 +2536,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
@@ -2503,216 +2547,228 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>408</v>
+        <v>418</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>409</v>
+        <v>419</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>410</v>
+        <v>420</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>411</v>
+        <v>421</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>412</v>
+        <v>422</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>413</v>
+        <v>423</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>414</v>
+        <v>424</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>415</v>
+        <v>425</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>416</v>
+        <v>426</v>
       </c>
       <c r="D5" s="24"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>417</v>
+        <v>427</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>418</v>
+        <v>428</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>419</v>
+        <v>429</v>
       </c>
       <c r="D6" s="24"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>420</v>
+        <v>430</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>421</v>
+        <v>431</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>419</v>
+        <v>429</v>
       </c>
       <c r="D7" s="24"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>422</v>
+        <v>432</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>418</v>
+        <v>428</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>419</v>
+        <v>429</v>
       </c>
       <c r="D8" s="24"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>423</v>
+        <v>433</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>424</v>
+        <v>434</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>419</v>
+        <v>429</v>
       </c>
       <c r="D9" s="24"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
+        <v>435</v>
+      </c>
+      <c r="B10" s="7" t="s">
         <v>425</v>
       </c>
-      <c r="B10" s="7" t="s">
-        <v>415</v>
-      </c>
       <c r="C10" s="7" t="s">
-        <v>419</v>
+        <v>429</v>
       </c>
       <c r="D10" s="24"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>426</v>
+        <v>436</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>415</v>
+        <v>425</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>419</v>
+        <v>429</v>
       </c>
       <c r="D11" s="24"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>427</v>
+        <v>437</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>428</v>
+        <v>438</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>419</v>
+        <v>429</v>
       </c>
       <c r="D12" s="24"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
+        <v>439</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>440</v>
+      </c>
+      <c r="C13" s="7" t="s">
         <v>429</v>
-      </c>
-      <c r="B13" s="7" t="s">
-        <v>430</v>
-      </c>
-      <c r="C13" s="7" t="s">
-        <v>419</v>
       </c>
       <c r="D13" s="24"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>431</v>
+        <v>441</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>430</v>
+        <v>440</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>419</v>
+        <v>429</v>
       </c>
       <c r="D14" s="24"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>432</v>
+        <v>442</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>430</v>
+        <v>440</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>419</v>
+        <v>429</v>
       </c>
       <c r="D15" s="24"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>433</v>
+        <v>443</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>415</v>
+        <v>440</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>419</v>
+        <v>429</v>
       </c>
       <c r="D16" s="24"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>434</v>
+        <v>444</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>435</v>
+        <v>425</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>419</v>
+        <v>429</v>
       </c>
       <c r="D17" s="24"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="s">
-        <v>436</v>
-      </c>
-      <c r="D18" s="25" t="n">
-        <f aca="false">SUMIF(C5:C17,"Yes",D5:D17)</f>
+      <c r="A18" s="7" t="s">
+        <v>445</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>446</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>429</v>
+      </c>
+      <c r="D18" s="24"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="3" t="s">
+        <v>447</v>
+      </c>
+      <c r="D19" s="25" t="n">
+        <f aca="false">SUMIF(C5:C18,"Yes",D5:D18)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2" t="s">
-        <v>437</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>438</v>
-      </c>
-      <c r="D19" s="26" t="n">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="D20" s="26" t="n">
         <v>0.05</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="s">
-        <v>439</v>
-      </c>
-      <c r="D20" s="25" t="n">
-        <f aca="false">D18*(1+D19)</f>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="3" t="s">
+        <v>450</v>
+      </c>
+      <c r="D21" s="25" t="n">
+        <f aca="false">D19*(1+D20)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2" t="s">
-        <v>440</v>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="2" t="s">
+        <v>451</v>
       </c>
     </row>
   </sheetData>
@@ -2740,69 +2796,69 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>441</v>
+        <v>452</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>278</v>
+        <v>288</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>442</v>
+        <v>453</v>
       </c>
       <c r="B2" s="14"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>443</v>
+        <v>454</v>
       </c>
       <c r="B3" s="14"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>444</v>
+        <v>455</v>
       </c>
       <c r="B4" s="14"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>445</v>
+        <v>456</v>
       </c>
       <c r="B5" s="14"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>446</v>
+        <v>457</v>
       </c>
       <c r="B6" s="14"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>447</v>
+        <v>458</v>
       </c>
       <c r="B7" s="14"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>448</v>
+        <v>459</v>
       </c>
       <c r="B8" s="14"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>449</v>
+        <v>460</v>
       </c>
       <c r="B9" s="14"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>450</v>
+        <v>461</v>
       </c>
       <c r="B10" s="14"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>451</v>
+        <v>462</v>
       </c>
       <c r="B11" s="14"/>
     </row>
@@ -2822,7 +2878,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K63"/>
+  <dimension ref="A1:K67"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -2839,12 +2895,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2855,31 +2911,31 @@
         <v>6</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="I4" s="10" t="s">
         <v>8</v>
       </c>
       <c r="J4" s="10" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="K4" s="10" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2901,15 +2957,15 @@
         <v>30</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="G5" s="11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="H5" s="11"/>
       <c r="I5" s="11"/>
       <c r="J5" s="11" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="K5" s="11"/>
     </row>
@@ -2932,18 +2988,18 @@
         <v>30</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="G6" s="14" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="H6" s="14"/>
       <c r="I6" s="14"/>
       <c r="J6" s="14" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="K6" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2965,22 +3021,22 @@
         <v>20</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="H7" s="14" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="I7" s="14" t="n">
         <v>7</v>
       </c>
       <c r="J7" s="14" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="K7" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3002,18 +3058,18 @@
         <v>25</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="G8" s="14" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="H8" s="14"/>
       <c r="I8" s="14"/>
       <c r="J8" s="14" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="K8" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3035,18 +3091,18 @@
         <v>35</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="G9" s="11" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="H9" s="11"/>
       <c r="I9" s="11"/>
       <c r="J9" s="11" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="K9" s="18" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3068,22 +3124,22 @@
         <v>15</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="G10" s="14" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="H10" s="14" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="I10" s="14" t="n">
         <v>5</v>
       </c>
       <c r="J10" s="14" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="K10" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3105,18 +3161,18 @@
         <v>40</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G11" s="14" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="H11" s="14"/>
       <c r="I11" s="14"/>
       <c r="J11" s="14" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="K11" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3138,22 +3194,22 @@
         <v>10</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="G12" s="14" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="H12" s="14" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="I12" s="14" t="n">
         <v>1</v>
       </c>
       <c r="J12" s="14" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="K12" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3175,18 +3231,18 @@
         <v>25</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G13" s="14" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="H13" s="14"/>
       <c r="I13" s="14"/>
       <c r="J13" s="14" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="K13" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3208,22 +3264,22 @@
         <v>20</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="G14" s="14" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="H14" s="14" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="I14" s="14" t="n">
         <v>6</v>
       </c>
       <c r="J14" s="14" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="K14" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3245,18 +3301,18 @@
         <v>50</v>
       </c>
       <c r="F15" s="14" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G15" s="14" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H15" s="14"/>
       <c r="I15" s="14"/>
       <c r="J15" s="14" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="K15" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3278,22 +3334,22 @@
         <v>25</v>
       </c>
       <c r="F16" s="14" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="G16" s="14" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="H16" s="14" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="I16" s="14" t="n">
         <v>7</v>
       </c>
       <c r="J16" s="14" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="K16" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3315,18 +3371,18 @@
         <v>35</v>
       </c>
       <c r="F17" s="14" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G17" s="14" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="H17" s="14"/>
       <c r="I17" s="14"/>
       <c r="J17" s="14" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="K17" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3348,22 +3404,22 @@
         <v>20</v>
       </c>
       <c r="F18" s="14" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="G18" s="14" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="H18" s="14" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="I18" s="14" t="n">
         <v>6</v>
       </c>
       <c r="J18" s="14" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="K18" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3385,18 +3441,18 @@
         <v>25</v>
       </c>
       <c r="F19" s="14" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="G19" s="14" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="H19" s="14"/>
       <c r="I19" s="14"/>
       <c r="J19" s="14" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="K19" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3418,18 +3474,18 @@
         <v>60</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="G20" s="11" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="H20" s="11"/>
       <c r="I20" s="11"/>
       <c r="J20" s="11" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="K20" s="18" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3451,18 +3507,18 @@
         <v>60</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="G21" s="11" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="H21" s="11"/>
       <c r="I21" s="11"/>
       <c r="J21" s="11" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K21" s="18" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3484,18 +3540,18 @@
         <v>30</v>
       </c>
       <c r="F22" s="14" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="G22" s="14" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="H22" s="14"/>
       <c r="I22" s="14"/>
       <c r="J22" s="14" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="K22" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3517,10 +3573,10 @@
         <v>90</v>
       </c>
       <c r="F23" s="14" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="G23" s="14" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="H23" s="14" t="s">
         <v>20</v>
@@ -3529,10 +3585,10 @@
         <v>50</v>
       </c>
       <c r="J23" s="14" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="K23" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3554,18 +3610,18 @@
         <v>30</v>
       </c>
       <c r="F24" s="14" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="G24" s="14" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="H24" s="14"/>
       <c r="I24" s="14"/>
       <c r="J24" s="14" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="K24" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3587,22 +3643,22 @@
         <v>10</v>
       </c>
       <c r="F25" s="14" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="G25" s="14" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="H25" s="14" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="I25" s="14" t="n">
         <v>2</v>
       </c>
       <c r="J25" s="14" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="K25" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3624,18 +3680,18 @@
         <v>65</v>
       </c>
       <c r="F26" s="14" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="G26" s="14" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="H26" s="14"/>
       <c r="I26" s="14"/>
       <c r="J26" s="14" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="K26" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3657,20 +3713,20 @@
         <v>10</v>
       </c>
       <c r="F27" s="19" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="G27" s="19" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="H27" s="19" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="I27" s="19"/>
       <c r="J27" s="19" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="K27" s="22" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3692,20 +3748,20 @@
         <v>65</v>
       </c>
       <c r="F28" s="14" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="G28" s="14" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="H28" s="14" t="s">
         <v>17</v>
       </c>
       <c r="I28" s="14"/>
       <c r="J28" s="14" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="K28" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3727,7 +3783,7 @@
         <v>30</v>
       </c>
       <c r="F29" s="14" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="G29" s="14" t="s">
         <v>17</v>
@@ -3735,10 +3791,10 @@
       <c r="H29" s="14"/>
       <c r="I29" s="14"/>
       <c r="J29" s="14" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="K29" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3760,18 +3816,18 @@
         <v>45</v>
       </c>
       <c r="F30" s="11" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="G30" s="11" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="H30" s="11"/>
       <c r="I30" s="11"/>
       <c r="J30" s="11" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="K30" s="18" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3793,7 +3849,7 @@
         <v>105</v>
       </c>
       <c r="F31" s="14" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="G31" s="14" t="s">
         <v>17</v>
@@ -3801,10 +3857,10 @@
       <c r="H31" s="14"/>
       <c r="I31" s="14"/>
       <c r="J31" s="14" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="K31" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3826,18 +3882,18 @@
         <v>90</v>
       </c>
       <c r="F32" s="14" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G32" s="14" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="H32" s="14"/>
       <c r="I32" s="14"/>
       <c r="J32" s="14" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="K32" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3859,7 +3915,7 @@
         <v>90</v>
       </c>
       <c r="F33" s="14" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="G33" s="14" t="s">
         <v>17</v>
@@ -3867,10 +3923,10 @@
       <c r="H33" s="14"/>
       <c r="I33" s="14"/>
       <c r="J33" s="14" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="K33" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3892,18 +3948,18 @@
         <v>60</v>
       </c>
       <c r="F34" s="11" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="G34" s="11" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="H34" s="11"/>
       <c r="I34" s="11"/>
       <c r="J34" s="11" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="K34" s="18" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3925,7 +3981,7 @@
         <v>60</v>
       </c>
       <c r="F35" s="14" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="G35" s="14" t="s">
         <v>17</v>
@@ -3933,10 +3989,10 @@
       <c r="H35" s="14"/>
       <c r="I35" s="14"/>
       <c r="J35" s="14" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="K35" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3958,7 +4014,7 @@
         <v>90</v>
       </c>
       <c r="F36" s="14" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="G36" s="14" t="s">
         <v>17</v>
@@ -3966,10 +4022,10 @@
       <c r="H36" s="14"/>
       <c r="I36" s="14"/>
       <c r="J36" s="14" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="K36" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3991,7 +4047,7 @@
         <v>30</v>
       </c>
       <c r="F37" s="14" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="G37" s="14" t="s">
         <v>17</v>
@@ -3999,10 +4055,10 @@
       <c r="H37" s="14"/>
       <c r="I37" s="14"/>
       <c r="J37" s="14" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="K37" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4024,18 +4080,18 @@
         <v>60</v>
       </c>
       <c r="F38" s="11" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="G38" s="11" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="H38" s="11"/>
       <c r="I38" s="11"/>
       <c r="J38" s="11" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="K38" s="18" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4057,7 +4113,7 @@
         <v>30</v>
       </c>
       <c r="F39" s="14" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="G39" s="14" t="s">
         <v>17</v>
@@ -4065,10 +4121,10 @@
       <c r="H39" s="14"/>
       <c r="I39" s="14"/>
       <c r="J39" s="14" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="K39" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4090,20 +4146,20 @@
         <v>15</v>
       </c>
       <c r="F40" s="14" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="G40" s="14" t="s">
         <v>17</v>
       </c>
       <c r="H40" s="14" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="I40" s="14"/>
       <c r="J40" s="14" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="K40" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4125,20 +4181,20 @@
         <v>20</v>
       </c>
       <c r="F41" s="19" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="G41" s="19" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="H41" s="19" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="I41" s="19"/>
       <c r="J41" s="19" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="K41" s="22" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4160,18 +4216,18 @@
         <v>40</v>
       </c>
       <c r="F42" s="14" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G42" s="14" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="H42" s="14"/>
       <c r="I42" s="14"/>
       <c r="J42" s="14" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="K42" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4193,20 +4249,20 @@
         <v>60</v>
       </c>
       <c r="F43" s="14" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="G43" s="14" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="H43" s="14" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="I43" s="14"/>
       <c r="J43" s="14" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="K43" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4228,18 +4284,18 @@
         <v>60</v>
       </c>
       <c r="F44" s="14" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="G44" s="14" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="H44" s="14"/>
       <c r="I44" s="14"/>
       <c r="J44" s="14" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="K44" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4261,20 +4317,20 @@
         <v>10</v>
       </c>
       <c r="F45" s="19" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="G45" s="19" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="H45" s="19" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="I45" s="19"/>
       <c r="J45" s="19" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="K45" s="22" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4296,22 +4352,22 @@
         <v>15</v>
       </c>
       <c r="F46" s="14" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="G46" s="14" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="H46" s="14" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="I46" s="14" t="n">
         <v>2</v>
       </c>
       <c r="J46" s="14" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="K46" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4333,18 +4389,18 @@
         <v>35</v>
       </c>
       <c r="F47" s="14" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="G47" s="14" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="H47" s="14"/>
       <c r="I47" s="14"/>
       <c r="J47" s="14" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="K47" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4366,18 +4422,18 @@
         <v>45</v>
       </c>
       <c r="F48" s="11" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="G48" s="11" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="H48" s="11"/>
       <c r="I48" s="11"/>
       <c r="J48" s="11" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="K48" s="18" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4399,18 +4455,18 @@
         <v>120</v>
       </c>
       <c r="F49" s="14" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="G49" s="14" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="H49" s="14"/>
       <c r="I49" s="14"/>
       <c r="J49" s="14" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="K49" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4432,22 +4488,22 @@
         <v>15</v>
       </c>
       <c r="F50" s="14" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="G50" s="14" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="H50" s="14" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="I50" s="14" t="n">
         <v>3</v>
       </c>
       <c r="J50" s="14" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="K50" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4469,18 +4525,18 @@
         <v>45</v>
       </c>
       <c r="F51" s="14" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G51" s="14" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="H51" s="14"/>
       <c r="I51" s="14"/>
       <c r="J51" s="14" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="K51" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4502,22 +4558,22 @@
         <v>10</v>
       </c>
       <c r="F52" s="14" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="G52" s="14" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="H52" s="14" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="I52" s="14" t="n">
         <v>1</v>
       </c>
       <c r="J52" s="14" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="K52" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4539,18 +4595,18 @@
         <v>30</v>
       </c>
       <c r="F53" s="14" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G53" s="14" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="H53" s="14"/>
       <c r="I53" s="14"/>
       <c r="J53" s="14" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="K53" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4572,22 +4628,22 @@
         <v>15</v>
       </c>
       <c r="F54" s="14" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="G54" s="14" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="H54" s="14" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="I54" s="14" t="n">
         <v>2</v>
       </c>
       <c r="J54" s="14" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="K54" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4609,18 +4665,18 @@
         <v>95</v>
       </c>
       <c r="F55" s="14" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="G55" s="14" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="H55" s="14"/>
       <c r="I55" s="14"/>
       <c r="J55" s="14" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="K55" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4642,22 +4698,22 @@
         <v>15</v>
       </c>
       <c r="F56" s="14" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="G56" s="14" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="H56" s="14" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="I56" s="14" t="n">
         <v>1</v>
       </c>
       <c r="J56" s="14" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="K56" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4679,18 +4735,18 @@
         <v>60</v>
       </c>
       <c r="F57" s="11" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="G57" s="11" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="H57" s="11"/>
       <c r="I57" s="11"/>
       <c r="J57" s="11" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="K57" s="18" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4712,18 +4768,18 @@
         <v>60</v>
       </c>
       <c r="F58" s="11" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="G58" s="11" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="H58" s="11"/>
       <c r="I58" s="11"/>
       <c r="J58" s="11" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K58" s="18" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4745,18 +4801,18 @@
         <v>30</v>
       </c>
       <c r="F59" s="14" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="G59" s="14" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="H59" s="14"/>
       <c r="I59" s="14"/>
       <c r="J59" s="14" t="s">
-        <v>134</v>
+        <v>76</v>
       </c>
       <c r="K59" s="17" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4771,32 +4827,32 @@
         <v>0.375</v>
       </c>
       <c r="D60" s="16" t="n">
-        <v>0.4375</v>
+        <v>0.416666666666667</v>
       </c>
       <c r="E60" s="14" t="n">
         <f aca="false">ROUND((D60-C60)*1440,0)</f>
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="F60" s="14" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="G60" s="14" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="H60" s="14" t="s">
-        <v>44</v>
+        <v>137</v>
       </c>
       <c r="I60" s="14" t="n">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="J60" s="14" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="K60" s="17" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="14" t="n">
         <v>4</v>
       </c>
@@ -4805,17 +4861,17 @@
         <v>46462</v>
       </c>
       <c r="C61" s="16" t="n">
-        <v>0.4375</v>
+        <v>0.416666666666667</v>
       </c>
       <c r="D61" s="16" t="n">
-        <v>0.458333333333333</v>
+        <v>0.447916666666667</v>
       </c>
       <c r="E61" s="14" t="n">
         <f aca="false">ROUND((D61-C61)*1440,0)</f>
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="F61" s="14" t="s">
-        <v>136</v>
+        <v>58</v>
       </c>
       <c r="G61" s="14" t="s">
         <v>137</v>
@@ -4823,19 +4879,159 @@
       <c r="H61" s="14"/>
       <c r="I61" s="14"/>
       <c r="J61" s="14" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="K61" s="17" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="5" t="s">
-        <v>139</v>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="B62" s="15" t="n">
+        <f aca="false">Overview!$B$3+A62-1</f>
+        <v>46462</v>
+      </c>
+      <c r="C62" s="16" t="n">
+        <v>0.447916666666667</v>
+      </c>
+      <c r="D62" s="16" t="n">
+        <v>0.46875</v>
+      </c>
+      <c r="E62" s="14" t="n">
+        <f aca="false">ROUND((D62-C62)*1440,0)</f>
+        <v>30</v>
+      </c>
+      <c r="F62" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="G62" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="H62" s="14" t="s">
+        <v>141</v>
+      </c>
+      <c r="I62" s="14" t="n">
+        <v>14</v>
+      </c>
+      <c r="J62" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="K62" s="17" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="B63" s="12" t="n">
+        <f aca="false">Overview!$B$3+A63-1</f>
+        <v>46462</v>
+      </c>
+      <c r="C63" s="13" t="n">
+        <v>0.46875</v>
+      </c>
+      <c r="D63" s="13" t="n">
+        <v>0.510416666666667</v>
+      </c>
+      <c r="E63" s="11" t="n">
+        <f aca="false">ROUND((D63-C63)*1440,0)</f>
+        <v>60</v>
+      </c>
+      <c r="F63" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="G63" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="H63" s="11"/>
+      <c r="I63" s="11"/>
+      <c r="J63" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="K63" s="18" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="B64" s="15" t="n">
+        <f aca="false">Overview!$B$3+A64-1</f>
+        <v>46462</v>
+      </c>
+      <c r="C64" s="16" t="n">
+        <v>0.510416666666667</v>
+      </c>
+      <c r="D64" s="16" t="n">
+        <v>0.520833333333333</v>
+      </c>
+      <c r="E64" s="14" t="n">
+        <f aca="false">ROUND((D64-C64)*1440,0)</f>
+        <v>15</v>
+      </c>
+      <c r="F64" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="G64" s="14" t="s">
+        <v>144</v>
+      </c>
+      <c r="H64" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="I64" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J64" s="14" t="s">
+        <v>145</v>
+      </c>
+      <c r="K64" s="17" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="B65" s="15" t="n">
+        <f aca="false">Overview!$B$3+A65-1</f>
+        <v>46462</v>
+      </c>
+      <c r="C65" s="16" t="n">
+        <v>0.520833333333333</v>
+      </c>
+      <c r="D65" s="16" t="n">
+        <v>0.541666666666667</v>
+      </c>
+      <c r="E65" s="14" t="n">
+        <f aca="false">ROUND((D65-C65)*1440,0)</f>
+        <v>30</v>
+      </c>
+      <c r="F65" s="14" t="s">
+        <v>146</v>
+      </c>
+      <c r="G65" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="H65" s="14"/>
+      <c r="I65" s="14"/>
+      <c r="J65" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="K65" s="17" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="5" t="s">
+        <v>148</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:K61"/>
+  <autoFilter ref="A4:K65"/>
   <hyperlinks>
     <hyperlink ref="K6" r:id="rId1" display="Open map"/>
     <hyperlink ref="K7" r:id="rId2" display="Open map"/>
@@ -4893,6 +5089,10 @@
     <hyperlink ref="K59" r:id="rId54" display="Open map"/>
     <hyperlink ref="K60" r:id="rId55" display="Open map"/>
     <hyperlink ref="K61" r:id="rId56" display="Open map"/>
+    <hyperlink ref="K62" r:id="rId57" display="Open map"/>
+    <hyperlink ref="K63" r:id="rId58" display="Open map"/>
+    <hyperlink ref="K64" r:id="rId59" display="Open map"/>
+    <hyperlink ref="K65" r:id="rId60" display="Open map"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -4901,7 +5101,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId57"/>
+  <drawing r:id="rId61"/>
 </worksheet>
 </file>
 
@@ -4923,7 +5123,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4931,19 +5131,19 @@
         <v>5</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>143</v>
+        <v>152</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>145</v>
+        <v>154</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4951,19 +5151,19 @@
         <v>1</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>146</v>
+        <v>155</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>147</v>
+        <v>156</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>149</v>
+        <v>158</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4971,19 +5171,19 @@
         <v>1</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>150</v>
+        <v>159</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>151</v>
+        <v>160</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>152</v>
+        <v>161</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4991,19 +5191,19 @@
         <v>1</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>152</v>
+        <v>161</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5011,19 +5211,19 @@
         <v>2</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>156</v>
+        <v>165</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5031,19 +5231,19 @@
         <v>2</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>158</v>
+        <v>167</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>159</v>
+        <v>168</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>160</v>
+        <v>169</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>161</v>
+        <v>170</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5051,19 +5251,19 @@
         <v>2</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>162</v>
+        <v>171</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>159</v>
+        <v>168</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>160</v>
+        <v>169</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>161</v>
+        <v>170</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5071,19 +5271,19 @@
         <v>3</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>159</v>
+        <v>168</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>160</v>
+        <v>169</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>161</v>
+        <v>170</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5091,19 +5291,19 @@
         <v>3</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>163</v>
+        <v>172</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>164</v>
+        <v>173</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>152</v>
+        <v>161</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5111,19 +5311,19 @@
         <v>3</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>152</v>
+        <v>161</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5131,19 +5331,19 @@
         <v>4</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>156</v>
+        <v>165</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5151,19 +5351,19 @@
         <v>4</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>22</v>
+        <v>176</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>167</v>
+        <v>141</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>156</v>
+        <v>177</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>152</v>
+        <v>161</v>
       </c>
     </row>
   </sheetData>
@@ -5191,90 +5391,90 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>169</v>
+        <v>179</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>170</v>
+        <v>180</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>171</v>
+        <v>181</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>172</v>
+        <v>182</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>173</v>
+        <v>183</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>174</v>
+        <v>184</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>175</v>
+        <v>185</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>176</v>
+        <v>186</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>177</v>
+        <v>187</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>178</v>
+        <v>188</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>180</v>
+        <v>190</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>181</v>
+        <v>191</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>182</v>
+        <v>192</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>183</v>
+        <v>193</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>184</v>
+        <v>194</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>185</v>
+        <v>195</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>186</v>
+        <v>196</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>187</v>
+        <v>197</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>188</v>
+        <v>198</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>189</v>
+        <v>199</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>190</v>
+        <v>200</v>
       </c>
     </row>
   </sheetData>
@@ -5304,184 +5504,184 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>191</v>
+        <v>201</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>194</v>
+        <v>204</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>196</v>
+        <v>206</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>197</v>
+        <v>207</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>198</v>
+        <v>208</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>199</v>
+        <v>209</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>201</v>
+        <v>211</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>202</v>
+        <v>212</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>203</v>
+        <v>213</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>204</v>
+        <v>214</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>205</v>
+        <v>215</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>206</v>
+        <v>216</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>207</v>
+        <v>217</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>208</v>
+        <v>218</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>209</v>
+        <v>219</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>210</v>
+        <v>220</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>211</v>
+        <v>221</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>212</v>
+        <v>222</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>213</v>
+        <v>223</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>214</v>
+        <v>224</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>215</v>
+        <v>225</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>216</v>
+        <v>226</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>217</v>
+        <v>227</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>218</v>
+        <v>228</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>219</v>
+        <v>229</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>220</v>
+        <v>230</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>221</v>
+        <v>231</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>222</v>
+        <v>232</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>223</v>
+        <v>233</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>224</v>
+        <v>234</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>225</v>
+        <v>235</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>226</v>
+        <v>236</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>227</v>
+        <v>237</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>228</v>
+        <v>238</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>229</v>
+        <v>239</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>230</v>
+        <v>240</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>231</v>
+        <v>241</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>232</v>
+        <v>242</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>233</v>
+        <v>243</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>234</v>
+        <v>244</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>238</v>
+        <v>248</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>239</v>
+        <v>249</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>240</v>
+        <v>250</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>241</v>
+        <v>251</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>242</v>
+        <v>252</v>
       </c>
     </row>
   </sheetData>
@@ -5509,202 +5709,202 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>243</v>
+        <v>253</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>244</v>
+        <v>254</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>245</v>
+        <v>255</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>246</v>
+        <v>256</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>245</v>
+        <v>255</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>247</v>
+        <v>257</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>245</v>
+        <v>255</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>248</v>
+        <v>258</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>245</v>
+        <v>255</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>249</v>
+        <v>259</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>245</v>
+        <v>255</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>250</v>
+        <v>260</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>245</v>
+        <v>255</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>251</v>
+        <v>261</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>245</v>
+        <v>255</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>252</v>
+        <v>262</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>245</v>
+        <v>255</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>253</v>
+        <v>263</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>245</v>
+        <v>255</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>254</v>
+        <v>264</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>255</v>
+        <v>265</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>256</v>
+        <v>266</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>255</v>
+        <v>265</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>257</v>
+        <v>267</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>255</v>
+        <v>265</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>258</v>
+        <v>268</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>255</v>
+        <v>265</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>259</v>
+        <v>269</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
-        <v>255</v>
+        <v>265</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>260</v>
+        <v>270</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>255</v>
+        <v>265</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>261</v>
+        <v>271</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
-        <v>255</v>
+        <v>265</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>262</v>
+        <v>272</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>263</v>
+        <v>273</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>264</v>
+        <v>274</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="14" t="s">
-        <v>263</v>
+        <v>273</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>265</v>
+        <v>275</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="14" t="s">
-        <v>263</v>
+        <v>273</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>266</v>
+        <v>276</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="14" t="s">
-        <v>263</v>
+        <v>273</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>267</v>
+        <v>277</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="14" t="s">
-        <v>263</v>
+        <v>273</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>268</v>
+        <v>278</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="14" t="s">
-        <v>269</v>
+        <v>279</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>270</v>
+        <v>280</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="14" t="s">
-        <v>269</v>
+        <v>279</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>271</v>
+        <v>281</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="14" t="s">
-        <v>269</v>
+        <v>279</v>
       </c>
       <c r="B25" s="14" t="s">
-        <v>272</v>
+        <v>282</v>
       </c>
     </row>
   </sheetData>
@@ -5735,221 +5935,221 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>273</v>
+        <v>283</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>274</v>
+        <v>284</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>275</v>
+        <v>285</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>276</v>
+        <v>286</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>277</v>
+        <v>287</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>278</v>
+        <v>288</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>279</v>
+        <v>289</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>280</v>
+        <v>290</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>281</v>
+        <v>291</v>
       </c>
       <c r="D4" s="14"/>
       <c r="E4" s="23"/>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>282</v>
+        <v>292</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>283</v>
+        <v>293</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>281</v>
+        <v>291</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>284</v>
+        <v>294</v>
       </c>
       <c r="E5" s="23"/>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>285</v>
+        <v>295</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>286</v>
+        <v>296</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>281</v>
+        <v>291</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>287</v>
+        <v>297</v>
       </c>
       <c r="E6" s="23"/>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>288</v>
+        <v>298</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>289</v>
+        <v>299</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="D7" s="14"/>
       <c r="E7" s="23"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
+        <v>301</v>
+      </c>
+      <c r="B8" s="14" t="s">
+        <v>302</v>
+      </c>
+      <c r="C8" s="14" t="s">
         <v>291</v>
-      </c>
-      <c r="B8" s="14" t="s">
-        <v>292</v>
-      </c>
-      <c r="C8" s="14" t="s">
-        <v>281</v>
       </c>
       <c r="D8" s="14"/>
       <c r="E8" s="23"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
+        <v>301</v>
+      </c>
+      <c r="B9" s="14" t="s">
+        <v>303</v>
+      </c>
+      <c r="C9" s="14" t="s">
         <v>291</v>
-      </c>
-      <c r="B9" s="14" t="s">
-        <v>293</v>
-      </c>
-      <c r="C9" s="14" t="s">
-        <v>281</v>
       </c>
       <c r="D9" s="14"/>
       <c r="E9" s="23"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>294</v>
+        <v>304</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>295</v>
+        <v>305</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>296</v>
+        <v>306</v>
       </c>
       <c r="D10" s="14"/>
       <c r="E10" s="23"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>294</v>
+        <v>304</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>297</v>
+        <v>307</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>296</v>
+        <v>306</v>
       </c>
       <c r="D11" s="14"/>
       <c r="E11" s="23"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>298</v>
+        <v>308</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>299</v>
+        <v>309</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>296</v>
+        <v>306</v>
       </c>
       <c r="D12" s="14"/>
       <c r="E12" s="23"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>300</v>
+        <v>310</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>301</v>
+        <v>311</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>302</v>
+        <v>312</v>
       </c>
       <c r="D13" s="14"/>
       <c r="E13" s="23"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>300</v>
+        <v>310</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>303</v>
+        <v>313</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>296</v>
+        <v>306</v>
       </c>
       <c r="D14" s="14"/>
       <c r="E14" s="23"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
-        <v>304</v>
+        <v>314</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>305</v>
+        <v>315</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>302</v>
+        <v>312</v>
       </c>
       <c r="D15" s="14"/>
       <c r="E15" s="23"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>306</v>
+        <v>316</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>307</v>
+        <v>317</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>302</v>
+        <v>312</v>
       </c>
       <c r="D16" s="14"/>
       <c r="E16" s="23"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
-        <v>308</v>
+        <v>318</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>309</v>
+        <v>319</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>302</v>
+        <v>312</v>
       </c>
       <c r="D17" s="14"/>
       <c r="E17" s="23"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>310</v>
+        <v>320</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>311</v>
+        <v>321</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>302</v>
+        <v>312</v>
       </c>
       <c r="D18" s="14"/>
       <c r="E18" s="23"/>
@@ -5979,146 +6179,146 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>312</v>
+        <v>322</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>313</v>
+        <v>323</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>314</v>
+        <v>324</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>315</v>
+        <v>325</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>314</v>
+        <v>324</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>316</v>
+        <v>326</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>314</v>
+        <v>324</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>317</v>
+        <v>327</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>314</v>
+        <v>324</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>318</v>
+        <v>328</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>314</v>
+        <v>324</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>319</v>
+        <v>329</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>314</v>
+        <v>324</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>320</v>
+        <v>330</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>314</v>
+        <v>324</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>321</v>
+        <v>331</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>322</v>
+        <v>332</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>323</v>
+        <v>333</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>322</v>
+        <v>332</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>324</v>
+        <v>334</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>322</v>
+        <v>332</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>325</v>
+        <v>335</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>322</v>
+        <v>332</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>326</v>
+        <v>336</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>322</v>
+        <v>332</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>327</v>
+        <v>337</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>322</v>
+        <v>332</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>328</v>
+        <v>338</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
-        <v>329</v>
+        <v>339</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>330</v>
+        <v>340</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>331</v>
+        <v>341</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>332</v>
+        <v>342</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
-        <v>333</v>
+        <v>343</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>334</v>
+        <v>344</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>335</v>
+        <v>345</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>336</v>
+        <v>346</v>
       </c>
     </row>
   </sheetData>
@@ -6146,90 +6346,90 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>337</v>
+        <v>347</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>338</v>
+        <v>348</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>339</v>
+        <v>349</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>340</v>
+        <v>350</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>341</v>
+        <v>351</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>342</v>
+        <v>352</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>343</v>
+        <v>353</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>344</v>
+        <v>354</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>345</v>
+        <v>355</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>346</v>
+        <v>356</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>347</v>
+        <v>357</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>348</v>
+        <v>358</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>349</v>
+        <v>359</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>350</v>
+        <v>360</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>351</v>
+        <v>361</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>352</v>
+        <v>362</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>353</v>
+        <v>363</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>354</v>
+        <v>364</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>355</v>
+        <v>365</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>356</v>
+        <v>366</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>357</v>
+        <v>367</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Trim Day 1 to Raghunath and Ranbireshwar; base all Kashmir nights in Srinagar; Day 7 without Pahalgam
Day 1 drops Bawe Wali Mata, Bahu Fort and Peer Kho and adds Raghunath Bazaar.
8-day: Gulmarg and Sonamarg become day trips from one Srinagar hotel (4 nights);
Day 7 is Avantipur, Martand, Pampore and an afternoon of Srinagar shopping.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A4yYiJq592wzPacq5vAVkN
</commit_message>
<xml_diff>
--- a/docs/itineraries/vaishno-devi-helicopter-4d-plan.xlsx
+++ b/docs/itineraries/vaishno-devi-helicopter-4d-plan.xlsx
@@ -23,7 +23,7 @@
     <sheet name="Open Points" sheetId="13" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Minute-by-Minute'!$A$4:$K$60</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Minute-by-Minute'!$A$4:$K$58</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="678" uniqueCount="429">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="669" uniqueCount="425">
   <si>
     <t xml:space="preserve">Vaishno Devi Helicopter Yatra – Overview</t>
   </si>
@@ -217,34 +217,28 @@
     <t xml:space="preserve">Darshan of the 7.5 ft Shiva lingam and crystal lingams</t>
   </si>
   <si>
-    <t xml:space="preserve">Bahu Fort (Bawe Wali Mata)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cross the Tawi to Bahu Fort</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bawe Wali Mata Temple &amp; Bahu Fort</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Darshan of Mahakali (Bawe Wali Mata); fort ramparts and Bagh-e-Bahu gardens at sunset</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bahu Fort</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Peer Kho Cave Temple</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Drive along Circular Road</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cave shrine of the self-manifest Shiva lingam; evening aarti</t>
+    <t xml:space="preserve">Raghunath Bazaar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Short hop to the old-city market</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shopping</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Raghunath Bazaar, Jammu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dry fruits, Kalari cheese, Dogra handicrafts</t>
   </si>
   <si>
     <t xml:space="preserve">Return to the hotel</t>
   </si>
   <si>
-    <t xml:space="preserve">Freshen up; Day 2 briefing (photo ID, small bag for Bhawan; main luggage stays at this hotel)</t>
+    <t xml:space="preserve">Rest</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rest, kirtan; Day 2 briefing (photo ID, small bag for Bhawan; main luggage stays at this hotel)</t>
   </si>
   <si>
     <t xml:space="preserve">Dinner</t>
@@ -307,9 +301,6 @@
     <t xml:space="preserve">Restaurant, Bhawan</t>
   </si>
   <si>
-    <t xml:space="preserve">Rest</t>
-  </si>
-  <si>
     <t xml:space="preserve">Rest, japa, group kirtan</t>
   </si>
   <si>
@@ -400,9 +391,6 @@
     <t xml:space="preserve">Drive to the market</t>
   </si>
   <si>
-    <t xml:space="preserve">Shopping</t>
-  </si>
-  <si>
     <t xml:space="preserve">Prasad, chunri, dry fruits, walnut and handicrafts</t>
   </si>
   <si>
@@ -499,7 +487,7 @@
     <t xml:space="preserve">Jammu sightseeing on Day 1</t>
   </si>
   <si>
-    <t xml:space="preserve">Uses arrival day well; four temples in 32 km</t>
+    <t xml:space="preserve">Uses arrival day well; Raghunath and Ranbireshwar temples and Raghunath Bazaar, only 19 km</t>
   </si>
   <si>
     <t xml:space="preserve">Afternoon-only window after a 14:00 arrival; little slack if flights are late</t>
@@ -691,7 +679,7 @@
     <t xml:space="preserve">Choose flights landing well before 14:00</t>
   </si>
   <si>
-    <t xml:space="preserve">Drop Peer Kho on Day 1</t>
+    <t xml:space="preserve">Shorten Raghunath Bazaar shopping on Day 1</t>
   </si>
   <si>
     <t xml:space="preserve">Lost yatri in crowd</t>
@@ -2008,18 +1996,18 @@
         <v>13</v>
       </c>
       <c r="D5" s="7" t="n">
-        <f aca="false">SUMIF('Minute-by-Minute'!$A$5:$A$60,A5,'Minute-by-Minute'!$I$5:$I$60)</f>
-        <v>32</v>
+        <f aca="false">SUMIF('Minute-by-Minute'!$A$5:$A$58,A5,'Minute-by-Minute'!$I$5:$I$58)</f>
+        <v>19</v>
       </c>
       <c r="E5" s="7" t="s">
         <v>14</v>
       </c>
       <c r="F5" s="9" t="n">
-        <f aca="false">_xlfn.MINIFS('Minute-by-Minute'!$C$5:$C$60,'Minute-by-Minute'!$A$5:$A$60,A5)</f>
+        <f aca="false">_xlfn.MINIFS('Minute-by-Minute'!$C$5:$C$58,'Minute-by-Minute'!$A$5:$A$58,A5)</f>
         <v>0.583333333333333</v>
       </c>
       <c r="G5" s="9" t="n">
-        <f aca="false">_xlfn.MAXIFS('Minute-by-Minute'!$D$5:$D$60,'Minute-by-Minute'!$A$5:$A$60,A5)</f>
+        <f aca="false">_xlfn.MAXIFS('Minute-by-Minute'!$D$5:$D$58,'Minute-by-Minute'!$A$5:$A$58,A5)</f>
         <v>0.885416666666667</v>
       </c>
       <c r="I5" s="7" t="s">
@@ -2041,18 +2029,18 @@
         <v>16</v>
       </c>
       <c r="D6" s="7" t="n">
-        <f aca="false">SUMIF('Minute-by-Minute'!$A$5:$A$60,A6,'Minute-by-Minute'!$I$5:$I$60)</f>
+        <f aca="false">SUMIF('Minute-by-Minute'!$A$5:$A$58,A6,'Minute-by-Minute'!$I$5:$I$58)</f>
         <v>52</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>17</v>
       </c>
       <c r="F6" s="9" t="n">
-        <f aca="false">_xlfn.MINIFS('Minute-by-Minute'!$C$5:$C$60,'Minute-by-Minute'!$A$5:$A$60,A6)</f>
+        <f aca="false">_xlfn.MINIFS('Minute-by-Minute'!$C$5:$C$58,'Minute-by-Minute'!$A$5:$A$58,A6)</f>
         <v>0.3125</v>
       </c>
       <c r="G6" s="9" t="n">
-        <f aca="false">_xlfn.MAXIFS('Minute-by-Minute'!$D$5:$D$60,'Minute-by-Minute'!$A$5:$A$60,A6)</f>
+        <f aca="false">_xlfn.MAXIFS('Minute-by-Minute'!$D$5:$D$58,'Minute-by-Minute'!$A$5:$A$58,A6)</f>
         <v>0.854166666666667</v>
       </c>
       <c r="I6" s="7" t="s">
@@ -2074,18 +2062,18 @@
         <v>19</v>
       </c>
       <c r="D7" s="7" t="n">
-        <f aca="false">SUMIF('Minute-by-Minute'!$A$5:$A$60,A7,'Minute-by-Minute'!$I$5:$I$60)</f>
+        <f aca="false">SUMIF('Minute-by-Minute'!$A$5:$A$58,A7,'Minute-by-Minute'!$I$5:$I$58)</f>
         <v>58</v>
       </c>
       <c r="E7" s="7" t="s">
         <v>14</v>
       </c>
       <c r="F7" s="9" t="n">
-        <f aca="false">_xlfn.MINIFS('Minute-by-Minute'!$C$5:$C$60,'Minute-by-Minute'!$A$5:$A$60,A7)</f>
+        <f aca="false">_xlfn.MINIFS('Minute-by-Minute'!$C$5:$C$58,'Minute-by-Minute'!$A$5:$A$58,A7)</f>
         <v>0.1875</v>
       </c>
       <c r="G7" s="9" t="n">
-        <f aca="false">_xlfn.MAXIFS('Minute-by-Minute'!$D$5:$D$60,'Minute-by-Minute'!$A$5:$A$60,A7)</f>
+        <f aca="false">_xlfn.MAXIFS('Minute-by-Minute'!$D$5:$D$58,'Minute-by-Minute'!$A$5:$A$58,A7)</f>
         <v>0.875</v>
       </c>
     </row>
@@ -2101,18 +2089,18 @@
         <v>20</v>
       </c>
       <c r="D8" s="7" t="n">
-        <f aca="false">SUMIF('Minute-by-Minute'!$A$5:$A$60,A8,'Minute-by-Minute'!$I$5:$I$60)</f>
+        <f aca="false">SUMIF('Minute-by-Minute'!$A$5:$A$58,A8,'Minute-by-Minute'!$I$5:$I$58)</f>
         <v>7</v>
       </c>
       <c r="E8" s="7" t="s">
         <v>21</v>
       </c>
       <c r="F8" s="9" t="n">
-        <f aca="false">_xlfn.MINIFS('Minute-by-Minute'!$C$5:$C$60,'Minute-by-Minute'!$A$5:$A$60,A8)</f>
+        <f aca="false">_xlfn.MINIFS('Minute-by-Minute'!$C$5:$C$58,'Minute-by-Minute'!$A$5:$A$58,A8)</f>
         <v>0.3125</v>
       </c>
       <c r="G8" s="9" t="n">
-        <f aca="false">_xlfn.MAXIFS('Minute-by-Minute'!$D$5:$D$60,'Minute-by-Minute'!$A$5:$A$60,A8)</f>
+        <f aca="false">_xlfn.MAXIFS('Minute-by-Minute'!$D$5:$D$58,'Minute-by-Minute'!$A$5:$A$58,A8)</f>
         <v>0.40625</v>
       </c>
       <c r="I8" s="3" t="s">
@@ -2125,7 +2113,7 @@
       </c>
       <c r="D9" s="3" t="n">
         <f aca="false">SUM(D5:D8)</f>
-        <v>149</v>
+        <v>136</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>24</v>
@@ -2185,121 +2173,121 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
+        <v>333</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>334</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>335</v>
+      </c>
+      <c r="D1" s="11" t="s">
+        <v>336</v>
+      </c>
+      <c r="E1" s="11" t="s">
         <v>337</v>
-      </c>
-      <c r="B1" s="11" t="s">
-        <v>338</v>
-      </c>
-      <c r="C1" s="11" t="s">
-        <v>339</v>
-      </c>
-      <c r="D1" s="11" t="s">
-        <v>340</v>
-      </c>
-      <c r="E1" s="11" t="s">
-        <v>341</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="12" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>343</v>
+        <v>339</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="D2" s="12" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>346</v>
+        <v>342</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>347</v>
+        <v>343</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>348</v>
+        <v>344</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>349</v>
+        <v>345</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
+        <v>346</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>347</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>348</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>349</v>
+      </c>
+      <c r="E4" s="12" t="s">
         <v>350</v>
-      </c>
-      <c r="B4" s="12" t="s">
-        <v>351</v>
-      </c>
-      <c r="C4" s="12" t="s">
-        <v>352</v>
-      </c>
-      <c r="D4" s="12" t="s">
-        <v>353</v>
-      </c>
-      <c r="E4" s="12" t="s">
-        <v>354</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>352</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>353</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>354</v>
+      </c>
+      <c r="E5" s="12" t="s">
         <v>355</v>
-      </c>
-      <c r="B5" s="12" t="s">
-        <v>356</v>
-      </c>
-      <c r="C5" s="12" t="s">
-        <v>357</v>
-      </c>
-      <c r="D5" s="12" t="s">
-        <v>358</v>
-      </c>
-      <c r="E5" s="12" t="s">
-        <v>359</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>360</v>
+        <v>356</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>361</v>
+        <v>357</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>362</v>
+        <v>358</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>363</v>
+        <v>359</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>364</v>
+        <v>360</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>365</v>
+        <v>361</v>
       </c>
     </row>
   </sheetData>
@@ -2329,81 +2317,81 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>366</v>
+        <v>362</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>368</v>
+        <v>364</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>369</v>
+        <v>365</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="12" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="C2" s="24"/>
       <c r="D2" s="24"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>371</v>
+        <v>367</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>372</v>
+        <v>368</v>
       </c>
       <c r="C3" s="24"/>
       <c r="D3" s="24"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>373</v>
+        <v>369</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>374</v>
+        <v>370</v>
       </c>
       <c r="C4" s="24"/>
       <c r="D4" s="24"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
-        <v>375</v>
+        <v>371</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>376</v>
+        <v>372</v>
       </c>
       <c r="C5" s="24"/>
       <c r="D5" s="24"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="C6" s="24"/>
       <c r="D6" s="24"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>379</v>
+        <v>375</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>380</v>
+        <v>376</v>
       </c>
       <c r="C7" s="24"/>
       <c r="D7" s="24"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
       <c r="B8" s="12"/>
       <c r="C8" s="24"/>
@@ -2411,7 +2399,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="24"/>
@@ -2419,7 +2407,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
       <c r="B10" s="12"/>
       <c r="C10" s="24"/>
@@ -2427,7 +2415,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>384</v>
+        <v>380</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="24"/>
@@ -2435,14 +2423,14 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="12" t="s">
-        <v>385</v>
+        <v>381</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>386</v>
+        <v>382</v>
       </c>
       <c r="C12" s="12"/>
       <c r="D12" s="12" t="s">
-        <v>387</v>
+        <v>383</v>
       </c>
     </row>
   </sheetData>
@@ -2472,168 +2460,168 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>388</v>
+        <v>384</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>389</v>
+        <v>385</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="25" t="s">
-        <v>390</v>
+        <v>386</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>391</v>
+        <v>387</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>392</v>
+        <v>388</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>395</v>
+        <v>391</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>396</v>
+        <v>392</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>397</v>
+        <v>393</v>
       </c>
       <c r="D5" s="26"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>398</v>
+        <v>394</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>399</v>
+        <v>395</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>400</v>
+        <v>396</v>
       </c>
       <c r="D6" s="26"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>401</v>
+        <v>397</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>402</v>
+        <v>398</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>400</v>
+        <v>396</v>
       </c>
       <c r="D7" s="26"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>403</v>
+        <v>399</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>404</v>
+        <v>400</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>400</v>
+        <v>396</v>
       </c>
       <c r="D8" s="26"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="B9" s="7" t="s">
+        <v>392</v>
+      </c>
+      <c r="C9" s="7" t="s">
         <v>396</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>400</v>
       </c>
       <c r="D9" s="26"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>405</v>
+        <v>401</v>
       </c>
       <c r="B10" s="7" t="s">
+        <v>392</v>
+      </c>
+      <c r="C10" s="7" t="s">
         <v>396</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>400</v>
       </c>
       <c r="D10" s="26"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>406</v>
+        <v>402</v>
       </c>
       <c r="B11" s="7" t="s">
+        <v>392</v>
+      </c>
+      <c r="C11" s="7" t="s">
         <v>396</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>400</v>
       </c>
       <c r="D11" s="26"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>407</v>
+        <v>403</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>408</v>
+        <v>404</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>400</v>
+        <v>396</v>
       </c>
       <c r="D12" s="26"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>409</v>
+        <v>405</v>
       </c>
       <c r="B13" s="7" t="s">
+        <v>392</v>
+      </c>
+      <c r="C13" s="7" t="s">
         <v>396</v>
-      </c>
-      <c r="C13" s="7" t="s">
-        <v>400</v>
       </c>
       <c r="D13" s="26"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>410</v>
+        <v>406</v>
       </c>
       <c r="B14" s="7" t="s">
+        <v>392</v>
+      </c>
+      <c r="C14" s="7" t="s">
         <v>396</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>400</v>
       </c>
       <c r="D14" s="26"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>411</v>
+        <v>407</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>412</v>
+        <v>408</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>400</v>
+        <v>396</v>
       </c>
       <c r="D15" s="26"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>413</v>
+        <v>409</v>
       </c>
       <c r="D16" s="27" t="n">
         <f aca="false">SUMIF(C5:C15,"Yes",D5:D15)</f>
@@ -2642,10 +2630,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>414</v>
+        <v>410</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>415</v>
+        <v>411</v>
       </c>
       <c r="D17" s="28" t="n">
         <v>0.05</v>
@@ -2653,7 +2641,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>416</v>
+        <v>412</v>
       </c>
       <c r="D18" s="27" t="n">
         <f aca="false">D16*(1+D17)</f>
@@ -2662,7 +2650,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>417</v>
+        <v>413</v>
       </c>
     </row>
   </sheetData>
@@ -2690,69 +2678,69 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>418</v>
+        <v>414</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="12" t="s">
-        <v>419</v>
+        <v>415</v>
       </c>
       <c r="B2" s="24"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>420</v>
+        <v>416</v>
       </c>
       <c r="B3" s="24"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>421</v>
+        <v>417</v>
       </c>
       <c r="B4" s="24"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
-        <v>422</v>
+        <v>418</v>
       </c>
       <c r="B5" s="24"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>423</v>
+        <v>419</v>
       </c>
       <c r="B6" s="24"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>424</v>
+        <v>420</v>
       </c>
       <c r="B7" s="24"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
-        <v>425</v>
+        <v>421</v>
       </c>
       <c r="B8" s="24"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>426</v>
+        <v>422</v>
       </c>
       <c r="B9" s="24"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>427</v>
+        <v>423</v>
       </c>
       <c r="B10" s="24"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>428</v>
+        <v>424</v>
       </c>
       <c r="B11" s="24"/>
     </row>
@@ -2772,7 +2760,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K62"/>
+  <dimension ref="A1:K60"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -3087,11 +3075,11 @@
         <v>0.704861111111111</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>0.722222222222222</v>
+        <v>0.729166666666667</v>
       </c>
       <c r="E12" s="12" t="n">
         <f aca="false">ROUND((D12-C12)*1440,0)</f>
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="F12" s="12" t="s">
         <v>55</v>
@@ -3117,14 +3105,14 @@
         <v>46459</v>
       </c>
       <c r="C13" s="14" t="n">
-        <v>0.722222222222222</v>
+        <v>0.729166666666667</v>
       </c>
       <c r="D13" s="14" t="n">
         <v>0.736111111111111</v>
       </c>
       <c r="E13" s="12" t="n">
         <f aca="false">ROUND((D13-C13)*1440,0)</f>
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F13" s="12" t="s">
         <v>45</v>
@@ -3136,7 +3124,7 @@
         <v>60</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J13" s="12" t="s">
         <v>61</v>
@@ -3145,7 +3133,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="12" t="n">
         <v>1</v>
       </c>
@@ -3157,22 +3145,22 @@
         <v>0.736111111111111</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>0.770833333333333</v>
+        <v>0.777777777777778</v>
       </c>
       <c r="E14" s="12" t="n">
         <f aca="false">ROUND((D14-C14)*1440,0)</f>
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="F14" s="12" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="G14" s="12" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H14" s="12"/>
       <c r="I14" s="12"/>
       <c r="J14" s="12" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="K14" s="15" t="s">
         <v>44</v>
@@ -3187,35 +3175,35 @@
         <v>46459</v>
       </c>
       <c r="C15" s="14" t="n">
-        <v>0.770833333333333</v>
+        <v>0.777777777777778</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>0.788194444444444</v>
+        <v>0.791666666666667</v>
       </c>
       <c r="E15" s="12" t="n">
         <f aca="false">ROUND((D15-C15)*1440,0)</f>
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F15" s="12" t="s">
         <v>45</v>
       </c>
       <c r="G15" s="12" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="H15" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="I15" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="J15" s="12" t="s">
         <v>65</v>
-      </c>
-      <c r="I15" s="12" t="n">
-        <v>7</v>
-      </c>
-      <c r="J15" s="12" t="s">
-        <v>66</v>
       </c>
       <c r="K15" s="15" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="12" t="n">
         <v>1</v>
       </c>
@@ -3224,20 +3212,20 @@
         <v>46459</v>
       </c>
       <c r="C16" s="14" t="n">
-        <v>0.788194444444444</v>
+        <v>0.791666666666667</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>0.8125</v>
+        <v>0.84375</v>
       </c>
       <c r="E16" s="12" t="n">
         <f aca="false">ROUND((D16-C16)*1440,0)</f>
-        <v>35</v>
+        <v>75</v>
       </c>
       <c r="F16" s="12" t="s">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="G16" s="12" t="s">
-        <v>65</v>
+        <v>47</v>
       </c>
       <c r="H16" s="12"/>
       <c r="I16" s="12"/>
@@ -3249,142 +3237,142 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="12" t="n">
+      <c r="A17" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="B17" s="13" t="n">
+      <c r="B17" s="17" t="n">
         <f aca="false">Overview!$B$3+A17-1</f>
         <v>46459</v>
       </c>
-      <c r="C17" s="14" t="n">
-        <v>0.8125</v>
-      </c>
-      <c r="D17" s="14" t="n">
-        <v>0.826388888888889</v>
-      </c>
-      <c r="E17" s="12" t="n">
+      <c r="C17" s="18" t="n">
+        <v>0.84375</v>
+      </c>
+      <c r="D17" s="18" t="n">
+        <v>0.885416666666667</v>
+      </c>
+      <c r="E17" s="16" t="n">
         <f aca="false">ROUND((D17-C17)*1440,0)</f>
-        <v>20</v>
-      </c>
-      <c r="F17" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="G17" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="H17" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="F17" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="G17" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="H17" s="16"/>
+      <c r="I17" s="16"/>
+      <c r="J17" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="K17" s="19" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="B18" s="17" t="n">
+        <f aca="false">Overview!$B$3+A18-1</f>
+        <v>46460</v>
+      </c>
+      <c r="C18" s="18" t="n">
+        <v>0.3125</v>
+      </c>
+      <c r="D18" s="18" t="n">
+        <v>0.354166666666667</v>
+      </c>
+      <c r="E18" s="16" t="n">
+        <f aca="false">ROUND((D18-C18)*1440,0)</f>
+        <v>60</v>
+      </c>
+      <c r="F18" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="G18" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="H18" s="16"/>
+      <c r="I18" s="16"/>
+      <c r="J18" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="K18" s="19" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B19" s="13" t="n">
+        <f aca="false">Overview!$B$3+A19-1</f>
+        <v>46460</v>
+      </c>
+      <c r="C19" s="14" t="n">
+        <v>0.354166666666667</v>
+      </c>
+      <c r="D19" s="14" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="E19" s="12" t="n">
+        <f aca="false">ROUND((D19-C19)*1440,0)</f>
+        <v>30</v>
+      </c>
+      <c r="F19" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="G19" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="I17" s="12" t="n">
-        <v>6</v>
-      </c>
-      <c r="J17" s="12" t="s">
-        <v>68</v>
-      </c>
-      <c r="K17" s="15" t="s">
+      <c r="H19" s="12"/>
+      <c r="I19" s="12"/>
+      <c r="J19" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="K19" s="15" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="B18" s="13" t="n">
-        <f aca="false">Overview!$B$3+A18-1</f>
-        <v>46459</v>
-      </c>
-      <c r="C18" s="14" t="n">
-        <v>0.826388888888889</v>
-      </c>
-      <c r="D18" s="14" t="n">
-        <v>0.84375</v>
-      </c>
-      <c r="E18" s="12" t="n">
-        <f aca="false">ROUND((D18-C18)*1440,0)</f>
-        <v>25</v>
-      </c>
-      <c r="F18" s="12" t="s">
-        <v>49</v>
-      </c>
-      <c r="G18" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="H18" s="12"/>
-      <c r="I18" s="12"/>
-      <c r="J18" s="12" t="s">
-        <v>69</v>
-      </c>
-      <c r="K18" s="15" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="B19" s="17" t="n">
-        <f aca="false">Overview!$B$3+A19-1</f>
-        <v>46459</v>
-      </c>
-      <c r="C19" s="18" t="n">
-        <v>0.84375</v>
-      </c>
-      <c r="D19" s="18" t="n">
-        <v>0.885416666666667</v>
-      </c>
-      <c r="E19" s="16" t="n">
-        <f aca="false">ROUND((D19-C19)*1440,0)</f>
-        <v>60</v>
-      </c>
-      <c r="F19" s="16" t="s">
-        <v>70</v>
-      </c>
-      <c r="G19" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="H19" s="16"/>
-      <c r="I19" s="16"/>
-      <c r="J19" s="16" t="s">
-        <v>70</v>
-      </c>
-      <c r="K19" s="19" t="s">
-        <v>44</v>
-      </c>
-    </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="16" t="n">
+      <c r="A20" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="B20" s="17" t="n">
+      <c r="B20" s="13" t="n">
         <f aca="false">Overview!$B$3+A20-1</f>
         <v>46460</v>
       </c>
-      <c r="C20" s="18" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="D20" s="18" t="n">
-        <v>0.354166666666667</v>
-      </c>
-      <c r="E20" s="16" t="n">
+      <c r="C20" s="14" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="D20" s="14" t="n">
+        <v>0.4375</v>
+      </c>
+      <c r="E20" s="12" t="n">
         <f aca="false">ROUND((D20-C20)*1440,0)</f>
-        <v>60</v>
-      </c>
-      <c r="F20" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="F20" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="G20" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="H20" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="G20" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="H20" s="16"/>
-      <c r="I20" s="16"/>
-      <c r="J20" s="16" t="s">
-        <v>71</v>
-      </c>
-      <c r="K20" s="19" t="s">
+      <c r="I20" s="12" t="n">
+        <v>50</v>
+      </c>
+      <c r="J20" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="K20" s="15" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="12" t="n">
         <v>2</v>
       </c>
@@ -3393,25 +3381,25 @@
         <v>46460</v>
       </c>
       <c r="C21" s="14" t="n">
-        <v>0.354166666666667</v>
+        <v>0.4375</v>
       </c>
       <c r="D21" s="14" t="n">
-        <v>0.375</v>
+        <v>0.458333333333333</v>
       </c>
       <c r="E21" s="12" t="n">
         <f aca="false">ROUND((D21-C21)*1440,0)</f>
         <v>30</v>
       </c>
       <c r="F21" s="12" t="s">
-        <v>49</v>
+        <v>73</v>
       </c>
       <c r="G21" s="12" t="s">
-        <v>47</v>
+        <v>74</v>
       </c>
       <c r="H21" s="12"/>
       <c r="I21" s="12"/>
       <c r="J21" s="12" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K21" s="15" t="s">
         <v>44</v>
@@ -3426,35 +3414,35 @@
         <v>46460</v>
       </c>
       <c r="C22" s="14" t="n">
-        <v>0.375</v>
+        <v>0.458333333333333</v>
       </c>
       <c r="D22" s="14" t="n">
-        <v>0.4375</v>
+        <v>0.465277777777778</v>
       </c>
       <c r="E22" s="12" t="n">
         <f aca="false">ROUND((D22-C22)*1440,0)</f>
-        <v>90</v>
+        <v>10</v>
       </c>
       <c r="F22" s="12" t="s">
         <v>45</v>
       </c>
       <c r="G22" s="12" t="s">
-        <v>47</v>
+        <v>76</v>
       </c>
       <c r="H22" s="12" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>50</v>
+        <v>2</v>
       </c>
       <c r="J22" s="12" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="K22" s="15" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="n">
         <v>2</v>
       </c>
@@ -3463,167 +3451,163 @@
         <v>46460</v>
       </c>
       <c r="C23" s="14" t="n">
-        <v>0.4375</v>
+        <v>0.465277777777778</v>
       </c>
       <c r="D23" s="14" t="n">
-        <v>0.458333333333333</v>
+        <v>0.510416666666667</v>
       </c>
       <c r="E23" s="12" t="n">
         <f aca="false">ROUND((D23-C23)*1440,0)</f>
-        <v>30</v>
+        <v>65</v>
       </c>
       <c r="F23" s="12" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="G23" s="12" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H23" s="12"/>
       <c r="I23" s="12"/>
       <c r="J23" s="12" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="K23" s="15" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="12" t="n">
+      <c r="A24" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="B24" s="13" t="n">
+      <c r="B24" s="21" t="n">
         <f aca="false">Overview!$B$3+A24-1</f>
         <v>46460</v>
       </c>
-      <c r="C24" s="14" t="n">
-        <v>0.458333333333333</v>
-      </c>
-      <c r="D24" s="14" t="n">
-        <v>0.465277777777778</v>
-      </c>
-      <c r="E24" s="12" t="n">
+      <c r="C24" s="22" t="n">
+        <v>0.510416666666667</v>
+      </c>
+      <c r="D24" s="22" t="n">
+        <v>0.517361111111111</v>
+      </c>
+      <c r="E24" s="20" t="n">
         <f aca="false">ROUND((D24-C24)*1440,0)</f>
         <v>10</v>
       </c>
-      <c r="F24" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="G24" s="12" t="s">
-        <v>78</v>
-      </c>
-      <c r="H24" s="12" t="s">
-        <v>79</v>
-      </c>
-      <c r="I24" s="12" t="n">
+      <c r="F24" s="20" t="s">
+        <v>81</v>
+      </c>
+      <c r="G24" s="20" t="s">
+        <v>77</v>
+      </c>
+      <c r="H24" s="20" t="s">
+        <v>82</v>
+      </c>
+      <c r="I24" s="20"/>
+      <c r="J24" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="K24" s="23" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="J24" s="12" t="s">
-        <v>80</v>
-      </c>
-      <c r="K24" s="15" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="B25" s="13" t="n">
+      <c r="B25" s="21" t="n">
         <f aca="false">Overview!$B$3+A25-1</f>
         <v>46460</v>
       </c>
-      <c r="C25" s="14" t="n">
-        <v>0.465277777777778</v>
-      </c>
-      <c r="D25" s="14" t="n">
-        <v>0.510416666666667</v>
-      </c>
-      <c r="E25" s="12" t="n">
+      <c r="C25" s="22" t="n">
+        <v>0.517361111111111</v>
+      </c>
+      <c r="D25" s="22" t="n">
+        <v>0.541666666666667</v>
+      </c>
+      <c r="E25" s="20" t="n">
         <f aca="false">ROUND((D25-C25)*1440,0)</f>
-        <v>65</v>
-      </c>
-      <c r="F25" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="G25" s="12" t="s">
-        <v>79</v>
-      </c>
-      <c r="H25" s="12"/>
-      <c r="I25" s="12"/>
-      <c r="J25" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="F25" s="20" t="s">
+        <v>84</v>
+      </c>
+      <c r="G25" s="20" t="s">
         <v>82</v>
       </c>
-      <c r="K25" s="15" t="s">
+      <c r="H25" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="I25" s="20"/>
+      <c r="J25" s="20" t="s">
+        <v>85</v>
+      </c>
+      <c r="K25" s="23" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="20" t="n">
+      <c r="A26" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="B26" s="21" t="n">
+      <c r="B26" s="13" t="n">
         <f aca="false">Overview!$B$3+A26-1</f>
         <v>46460</v>
       </c>
-      <c r="C26" s="22" t="n">
-        <v>0.510416666666667</v>
-      </c>
-      <c r="D26" s="22" t="n">
-        <v>0.517361111111111</v>
-      </c>
-      <c r="E26" s="20" t="n">
+      <c r="C26" s="14" t="n">
+        <v>0.541666666666667</v>
+      </c>
+      <c r="D26" s="14" t="n">
+        <v>0.5625</v>
+      </c>
+      <c r="E26" s="12" t="n">
         <f aca="false">ROUND((D26-C26)*1440,0)</f>
-        <v>10</v>
-      </c>
-      <c r="F26" s="20" t="s">
-        <v>83</v>
-      </c>
-      <c r="G26" s="20" t="s">
-        <v>79</v>
-      </c>
-      <c r="H26" s="20" t="s">
-        <v>84</v>
-      </c>
-      <c r="I26" s="20"/>
-      <c r="J26" s="20" t="s">
-        <v>85</v>
-      </c>
-      <c r="K26" s="23" t="s">
+        <v>30</v>
+      </c>
+      <c r="F26" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="G26" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="H26" s="12"/>
+      <c r="I26" s="12"/>
+      <c r="J26" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="K26" s="15" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="20" t="n">
+      <c r="A27" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="B27" s="21" t="n">
+      <c r="B27" s="17" t="n">
         <f aca="false">Overview!$B$3+A27-1</f>
         <v>46460</v>
       </c>
-      <c r="C27" s="22" t="n">
-        <v>0.517361111111111</v>
-      </c>
-      <c r="D27" s="22" t="n">
-        <v>0.541666666666667</v>
-      </c>
-      <c r="E27" s="20" t="n">
+      <c r="C27" s="18" t="n">
+        <v>0.5625</v>
+      </c>
+      <c r="D27" s="18" t="n">
+        <v>0.59375</v>
+      </c>
+      <c r="E27" s="16" t="n">
         <f aca="false">ROUND((D27-C27)*1440,0)</f>
-        <v>35</v>
-      </c>
-      <c r="F27" s="20" t="s">
-        <v>86</v>
-      </c>
-      <c r="G27" s="20" t="s">
-        <v>84</v>
-      </c>
-      <c r="H27" s="20" t="s">
-        <v>17</v>
-      </c>
-      <c r="I27" s="20"/>
-      <c r="J27" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="F27" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="G27" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="K27" s="23" t="s">
+      <c r="H27" s="16"/>
+      <c r="I27" s="16"/>
+      <c r="J27" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="K27" s="19" t="s">
         <v>44</v>
       </c>
     </row>
@@ -3636,17 +3620,17 @@
         <v>46460</v>
       </c>
       <c r="C28" s="14" t="n">
-        <v>0.541666666666667</v>
+        <v>0.59375</v>
       </c>
       <c r="D28" s="14" t="n">
-        <v>0.5625</v>
+        <v>0.6875</v>
       </c>
       <c r="E28" s="12" t="n">
         <f aca="false">ROUND((D28-C28)*1440,0)</f>
-        <v>30</v>
+        <v>135</v>
       </c>
       <c r="F28" s="12" t="s">
-        <v>49</v>
+        <v>66</v>
       </c>
       <c r="G28" s="12" t="s">
         <v>17</v>
@@ -3661,35 +3645,35 @@
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="16" t="n">
+      <c r="A29" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="B29" s="17" t="n">
+      <c r="B29" s="13" t="n">
         <f aca="false">Overview!$B$3+A29-1</f>
         <v>46460</v>
       </c>
-      <c r="C29" s="18" t="n">
-        <v>0.5625</v>
-      </c>
-      <c r="D29" s="18" t="n">
-        <v>0.59375</v>
-      </c>
-      <c r="E29" s="16" t="n">
+      <c r="C29" s="14" t="n">
+        <v>0.6875</v>
+      </c>
+      <c r="D29" s="14" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E29" s="12" t="n">
         <f aca="false">ROUND((D29-C29)*1440,0)</f>
-        <v>45</v>
-      </c>
-      <c r="F29" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="G29" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="F29" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="G29" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="H29" s="16"/>
-      <c r="I29" s="16"/>
-      <c r="J29" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="K29" s="19" t="s">
+      <c r="H29" s="12"/>
+      <c r="I29" s="12"/>
+      <c r="J29" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="K29" s="15" t="s">
         <v>44</v>
       </c>
     </row>
@@ -3702,17 +3686,17 @@
         <v>46460</v>
       </c>
       <c r="C30" s="14" t="n">
-        <v>0.59375</v>
+        <v>0.75</v>
       </c>
       <c r="D30" s="14" t="n">
-        <v>0.6875</v>
+        <v>0.8125</v>
       </c>
       <c r="E30" s="12" t="n">
         <f aca="false">ROUND((D30-C30)*1440,0)</f>
-        <v>135</v>
+        <v>90</v>
       </c>
       <c r="F30" s="12" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G30" s="12" t="s">
         <v>17</v>
@@ -3720,65 +3704,65 @@
       <c r="H30" s="12"/>
       <c r="I30" s="12"/>
       <c r="J30" s="12" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K30" s="15" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="12" t="n">
+      <c r="A31" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="B31" s="13" t="n">
+      <c r="B31" s="17" t="n">
         <f aca="false">Overview!$B$3+A31-1</f>
         <v>46460</v>
       </c>
-      <c r="C31" s="14" t="n">
-        <v>0.6875</v>
-      </c>
-      <c r="D31" s="14" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="E31" s="12" t="n">
+      <c r="C31" s="18" t="n">
+        <v>0.8125</v>
+      </c>
+      <c r="D31" s="18" t="n">
+        <v>0.854166666666667</v>
+      </c>
+      <c r="E31" s="16" t="n">
         <f aca="false">ROUND((D31-C31)*1440,0)</f>
-        <v>90</v>
-      </c>
-      <c r="F31" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="G31" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="H31" s="12"/>
-      <c r="I31" s="12"/>
-      <c r="J31" s="12" t="s">
-        <v>93</v>
-      </c>
-      <c r="K31" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="F31" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="G31" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="H31" s="16"/>
+      <c r="I31" s="16"/>
+      <c r="J31" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="K31" s="19" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B32" s="13" t="n">
         <f aca="false">Overview!$B$3+A32-1</f>
-        <v>46460</v>
+        <v>46461</v>
       </c>
       <c r="C32" s="14" t="n">
-        <v>0.75</v>
+        <v>0.1875</v>
       </c>
       <c r="D32" s="14" t="n">
-        <v>0.8125</v>
+        <v>0.229166666666667</v>
       </c>
       <c r="E32" s="12" t="n">
         <f aca="false">ROUND((D32-C32)*1440,0)</f>
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="F32" s="12" t="s">
-        <v>94</v>
+        <v>49</v>
       </c>
       <c r="G32" s="12" t="s">
         <v>17</v>
@@ -3786,42 +3770,42 @@
       <c r="H32" s="12"/>
       <c r="I32" s="12"/>
       <c r="J32" s="12" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="K32" s="15" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="16" t="n">
-        <v>2</v>
-      </c>
-      <c r="B33" s="17" t="n">
+      <c r="A33" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="B33" s="13" t="n">
         <f aca="false">Overview!$B$3+A33-1</f>
-        <v>46460</v>
-      </c>
-      <c r="C33" s="18" t="n">
-        <v>0.8125</v>
-      </c>
-      <c r="D33" s="18" t="n">
-        <v>0.854166666666667</v>
-      </c>
-      <c r="E33" s="16" t="n">
+        <v>46461</v>
+      </c>
+      <c r="C33" s="14" t="n">
+        <v>0.229166666666667</v>
+      </c>
+      <c r="D33" s="14" t="n">
+        <v>0.291666666666667</v>
+      </c>
+      <c r="E33" s="12" t="n">
         <f aca="false">ROUND((D33-C33)*1440,0)</f>
-        <v>60</v>
-      </c>
-      <c r="F33" s="16" t="s">
-        <v>70</v>
-      </c>
-      <c r="G33" s="16" t="s">
-        <v>89</v>
-      </c>
-      <c r="H33" s="16"/>
-      <c r="I33" s="16"/>
-      <c r="J33" s="16" t="s">
-        <v>70</v>
-      </c>
-      <c r="K33" s="19" t="s">
+        <v>90</v>
+      </c>
+      <c r="F33" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="G33" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="H33" s="12"/>
+      <c r="I33" s="12"/>
+      <c r="J33" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="K33" s="15" t="s">
         <v>44</v>
       </c>
     </row>
@@ -3834,17 +3818,17 @@
         <v>46461</v>
       </c>
       <c r="C34" s="14" t="n">
-        <v>0.1875</v>
+        <v>0.291666666666667</v>
       </c>
       <c r="D34" s="14" t="n">
-        <v>0.229166666666667</v>
+        <v>0.3125</v>
       </c>
       <c r="E34" s="12" t="n">
         <f aca="false">ROUND((D34-C34)*1440,0)</f>
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="F34" s="12" t="s">
-        <v>49</v>
+        <v>66</v>
       </c>
       <c r="G34" s="12" t="s">
         <v>17</v>
@@ -3852,42 +3836,42 @@
       <c r="H34" s="12"/>
       <c r="I34" s="12"/>
       <c r="J34" s="12" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="K34" s="15" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="12" t="n">
+      <c r="A35" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="B35" s="13" t="n">
+      <c r="B35" s="17" t="n">
         <f aca="false">Overview!$B$3+A35-1</f>
         <v>46461</v>
       </c>
-      <c r="C35" s="14" t="n">
-        <v>0.229166666666667</v>
-      </c>
-      <c r="D35" s="14" t="n">
-        <v>0.291666666666667</v>
-      </c>
-      <c r="E35" s="12" t="n">
+      <c r="C35" s="18" t="n">
+        <v>0.3125</v>
+      </c>
+      <c r="D35" s="18" t="n">
+        <v>0.354166666666667</v>
+      </c>
+      <c r="E35" s="16" t="n">
         <f aca="false">ROUND((D35-C35)*1440,0)</f>
-        <v>90</v>
-      </c>
-      <c r="F35" s="12" t="s">
-        <v>94</v>
-      </c>
-      <c r="G35" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="H35" s="12"/>
-      <c r="I35" s="12"/>
-      <c r="J35" s="12" t="s">
-        <v>97</v>
-      </c>
-      <c r="K35" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="F35" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="G35" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="H35" s="16"/>
+      <c r="I35" s="16"/>
+      <c r="J35" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="K35" s="19" t="s">
         <v>44</v>
       </c>
     </row>
@@ -3900,17 +3884,17 @@
         <v>46461</v>
       </c>
       <c r="C36" s="14" t="n">
-        <v>0.291666666666667</v>
+        <v>0.354166666666667</v>
       </c>
       <c r="D36" s="14" t="n">
-        <v>0.3125</v>
+        <v>0.375</v>
       </c>
       <c r="E36" s="12" t="n">
         <f aca="false">ROUND((D36-C36)*1440,0)</f>
         <v>30</v>
       </c>
       <c r="F36" s="12" t="s">
-        <v>90</v>
+        <v>49</v>
       </c>
       <c r="G36" s="12" t="s">
         <v>17</v>
@@ -3918,75 +3902,79 @@
       <c r="H36" s="12"/>
       <c r="I36" s="12"/>
       <c r="J36" s="12" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="K36" s="15" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="16" t="n">
+      <c r="A37" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="B37" s="17" t="n">
+      <c r="B37" s="13" t="n">
         <f aca="false">Overview!$B$3+A37-1</f>
         <v>46461</v>
       </c>
-      <c r="C37" s="18" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="D37" s="18" t="n">
-        <v>0.354166666666667</v>
-      </c>
-      <c r="E37" s="16" t="n">
+      <c r="C37" s="14" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="D37" s="14" t="n">
+        <v>0.385416666666667</v>
+      </c>
+      <c r="E37" s="12" t="n">
         <f aca="false">ROUND((D37-C37)*1440,0)</f>
-        <v>60</v>
-      </c>
-      <c r="F37" s="16" t="s">
-        <v>71</v>
-      </c>
-      <c r="G37" s="16" t="s">
-        <v>89</v>
-      </c>
-      <c r="H37" s="16"/>
-      <c r="I37" s="16"/>
-      <c r="J37" s="16" t="s">
-        <v>71</v>
-      </c>
-      <c r="K37" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="F37" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="G37" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="H37" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="I37" s="12"/>
+      <c r="J37" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="K37" s="15" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="12" t="n">
+      <c r="A38" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="B38" s="13" t="n">
+      <c r="B38" s="21" t="n">
         <f aca="false">Overview!$B$3+A38-1</f>
         <v>46461</v>
       </c>
-      <c r="C38" s="14" t="n">
-        <v>0.354166666666667</v>
-      </c>
-      <c r="D38" s="14" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="E38" s="12" t="n">
+      <c r="C38" s="22" t="n">
+        <v>0.385416666666667</v>
+      </c>
+      <c r="D38" s="22" t="n">
+        <v>0.399305555555556</v>
+      </c>
+      <c r="E38" s="20" t="n">
         <f aca="false">ROUND((D38-C38)*1440,0)</f>
-        <v>30</v>
-      </c>
-      <c r="F38" s="12" t="s">
-        <v>49</v>
-      </c>
-      <c r="G38" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="H38" s="12"/>
-      <c r="I38" s="12"/>
-      <c r="J38" s="12" t="s">
-        <v>99</v>
-      </c>
-      <c r="K38" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="F38" s="20" t="s">
+        <v>100</v>
+      </c>
+      <c r="G38" s="20" t="s">
+        <v>98</v>
+      </c>
+      <c r="H38" s="20" t="s">
+        <v>101</v>
+      </c>
+      <c r="I38" s="20"/>
+      <c r="J38" s="20" t="s">
+        <v>102</v>
+      </c>
+      <c r="K38" s="23" t="s">
         <v>44</v>
       </c>
     </row>
@@ -3999,64 +3987,62 @@
         <v>46461</v>
       </c>
       <c r="C39" s="14" t="n">
-        <v>0.375</v>
+        <v>0.399305555555556</v>
       </c>
       <c r="D39" s="14" t="n">
-        <v>0.385416666666667</v>
+        <v>0.427083333333333</v>
       </c>
       <c r="E39" s="12" t="n">
         <f aca="false">ROUND((D39-C39)*1440,0)</f>
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="F39" s="12" t="s">
-        <v>100</v>
+        <v>55</v>
       </c>
       <c r="G39" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="H39" s="12" t="s">
-        <v>101</v>
-      </c>
+        <v>103</v>
+      </c>
+      <c r="H39" s="12"/>
       <c r="I39" s="12"/>
       <c r="J39" s="12" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="K39" s="15" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="20" t="n">
+      <c r="A40" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="B40" s="21" t="n">
+      <c r="B40" s="13" t="n">
         <f aca="false">Overview!$B$3+A40-1</f>
         <v>46461</v>
       </c>
-      <c r="C40" s="22" t="n">
-        <v>0.385416666666667</v>
-      </c>
-      <c r="D40" s="22" t="n">
-        <v>0.399305555555556</v>
-      </c>
-      <c r="E40" s="20" t="n">
+      <c r="C40" s="14" t="n">
+        <v>0.427083333333333</v>
+      </c>
+      <c r="D40" s="14" t="n">
+        <v>0.46875</v>
+      </c>
+      <c r="E40" s="12" t="n">
         <f aca="false">ROUND((D40-C40)*1440,0)</f>
-        <v>20</v>
-      </c>
-      <c r="F40" s="20" t="s">
-        <v>103</v>
-      </c>
-      <c r="G40" s="20" t="s">
-        <v>101</v>
-      </c>
-      <c r="H40" s="20" t="s">
-        <v>104</v>
-      </c>
-      <c r="I40" s="20"/>
-      <c r="J40" s="20" t="s">
+        <v>60</v>
+      </c>
+      <c r="F40" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="G40" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="K40" s="23" t="s">
+      <c r="H40" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="I40" s="12"/>
+      <c r="J40" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="K40" s="15" t="s">
         <v>44</v>
       </c>
     </row>
@@ -4069,20 +4055,20 @@
         <v>46461</v>
       </c>
       <c r="C41" s="14" t="n">
-        <v>0.399305555555556</v>
+        <v>0.46875</v>
       </c>
       <c r="D41" s="14" t="n">
-        <v>0.427083333333333</v>
+        <v>0.510416666666667</v>
       </c>
       <c r="E41" s="12" t="n">
         <f aca="false">ROUND((D41-C41)*1440,0)</f>
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="F41" s="12" t="s">
-        <v>55</v>
+        <v>79</v>
       </c>
       <c r="G41" s="12" t="s">
-        <v>106</v>
+        <v>82</v>
       </c>
       <c r="H41" s="12"/>
       <c r="I41" s="12"/>
@@ -4094,37 +4080,37 @@
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="12" t="n">
+      <c r="A42" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="B42" s="13" t="n">
+      <c r="B42" s="21" t="n">
         <f aca="false">Overview!$B$3+A42-1</f>
         <v>46461</v>
       </c>
-      <c r="C42" s="14" t="n">
-        <v>0.427083333333333</v>
-      </c>
-      <c r="D42" s="14" t="n">
-        <v>0.46875</v>
-      </c>
-      <c r="E42" s="12" t="n">
+      <c r="C42" s="22" t="n">
+        <v>0.510416666666667</v>
+      </c>
+      <c r="D42" s="22" t="n">
+        <v>0.517361111111111</v>
+      </c>
+      <c r="E42" s="20" t="n">
         <f aca="false">ROUND((D42-C42)*1440,0)</f>
-        <v>60</v>
-      </c>
-      <c r="F42" s="12" t="s">
-        <v>100</v>
-      </c>
-      <c r="G42" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="F42" s="20" t="s">
+        <v>81</v>
+      </c>
+      <c r="G42" s="20" t="s">
+        <v>82</v>
+      </c>
+      <c r="H42" s="20" t="s">
+        <v>77</v>
+      </c>
+      <c r="I42" s="20"/>
+      <c r="J42" s="20" t="s">
         <v>108</v>
       </c>
-      <c r="H42" s="12" t="s">
-        <v>84</v>
-      </c>
-      <c r="I42" s="12"/>
-      <c r="J42" s="12" t="s">
-        <v>109</v>
-      </c>
-      <c r="K42" s="15" t="s">
+      <c r="K42" s="23" t="s">
         <v>44</v>
       </c>
     </row>
@@ -4137,23 +4123,27 @@
         <v>46461</v>
       </c>
       <c r="C43" s="14" t="n">
-        <v>0.46875</v>
+        <v>0.517361111111111</v>
       </c>
       <c r="D43" s="14" t="n">
-        <v>0.510416666666667</v>
+        <v>0.527777777777778</v>
       </c>
       <c r="E43" s="12" t="n">
         <f aca="false">ROUND((D43-C43)*1440,0)</f>
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="F43" s="12" t="s">
-        <v>81</v>
+        <v>45</v>
       </c>
       <c r="G43" s="12" t="s">
-        <v>84</v>
-      </c>
-      <c r="H43" s="12"/>
-      <c r="I43" s="12"/>
+        <v>77</v>
+      </c>
+      <c r="H43" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="I43" s="12" t="n">
+        <v>2</v>
+      </c>
       <c r="J43" s="12" t="s">
         <v>110</v>
       </c>
@@ -4162,37 +4152,35 @@
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="20" t="n">
+      <c r="A44" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="B44" s="21" t="n">
+      <c r="B44" s="17" t="n">
         <f aca="false">Overview!$B$3+A44-1</f>
         <v>46461</v>
       </c>
-      <c r="C44" s="22" t="n">
-        <v>0.510416666666667</v>
-      </c>
-      <c r="D44" s="22" t="n">
-        <v>0.517361111111111</v>
-      </c>
-      <c r="E44" s="20" t="n">
+      <c r="C44" s="18" t="n">
+        <v>0.527777777777778</v>
+      </c>
+      <c r="D44" s="18" t="n">
+        <v>0.5625</v>
+      </c>
+      <c r="E44" s="16" t="n">
         <f aca="false">ROUND((D44-C44)*1440,0)</f>
-        <v>10</v>
-      </c>
-      <c r="F44" s="20" t="s">
-        <v>83</v>
-      </c>
-      <c r="G44" s="20" t="s">
-        <v>84</v>
-      </c>
-      <c r="H44" s="20" t="s">
-        <v>79</v>
-      </c>
-      <c r="I44" s="20"/>
-      <c r="J44" s="20" t="s">
-        <v>111</v>
-      </c>
-      <c r="K44" s="23" t="s">
+        <v>50</v>
+      </c>
+      <c r="F44" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="G44" s="16" t="s">
+        <v>109</v>
+      </c>
+      <c r="H44" s="16"/>
+      <c r="I44" s="16"/>
+      <c r="J44" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="K44" s="19" t="s">
         <v>44</v>
       </c>
     </row>
@@ -4205,10 +4193,10 @@
         <v>46461</v>
       </c>
       <c r="C45" s="14" t="n">
-        <v>0.517361111111111</v>
+        <v>0.5625</v>
       </c>
       <c r="D45" s="14" t="n">
-        <v>0.527777777777778</v>
+        <v>0.572916666666667</v>
       </c>
       <c r="E45" s="12" t="n">
         <f aca="false">ROUND((D45-C45)*1440,0)</f>
@@ -4218,51 +4206,51 @@
         <v>45</v>
       </c>
       <c r="G45" s="12" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="H45" s="12" t="s">
+        <v>111</v>
+      </c>
+      <c r="I45" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="J45" s="12" t="s">
         <v>112</v>
-      </c>
-      <c r="I45" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="J45" s="12" t="s">
-        <v>113</v>
       </c>
       <c r="K45" s="15" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="16" t="n">
+    <row r="46" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="B46" s="17" t="n">
+      <c r="B46" s="13" t="n">
         <f aca="false">Overview!$B$3+A46-1</f>
         <v>46461</v>
       </c>
-      <c r="C46" s="18" t="n">
-        <v>0.527777777777778</v>
-      </c>
-      <c r="D46" s="18" t="n">
-        <v>0.5625</v>
-      </c>
-      <c r="E46" s="16" t="n">
+      <c r="C46" s="14" t="n">
+        <v>0.572916666666667</v>
+      </c>
+      <c r="D46" s="14" t="n">
+        <v>0.604166666666667</v>
+      </c>
+      <c r="E46" s="12" t="n">
         <f aca="false">ROUND((D46-C46)*1440,0)</f>
-        <v>50</v>
-      </c>
-      <c r="F46" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="G46" s="16" t="s">
-        <v>112</v>
-      </c>
-      <c r="H46" s="16"/>
-      <c r="I46" s="16"/>
-      <c r="J46" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="K46" s="19" t="s">
+        <v>45</v>
+      </c>
+      <c r="F46" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="G46" s="12" t="s">
+        <v>111</v>
+      </c>
+      <c r="H46" s="12"/>
+      <c r="I46" s="12"/>
+      <c r="J46" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="K46" s="15" t="s">
         <v>44</v>
       </c>
     </row>
@@ -4275,35 +4263,35 @@
         <v>46461</v>
       </c>
       <c r="C47" s="14" t="n">
-        <v>0.5625</v>
+        <v>0.604166666666667</v>
       </c>
       <c r="D47" s="14" t="n">
-        <v>0.572916666666667</v>
+        <v>0.611111111111111</v>
       </c>
       <c r="E47" s="12" t="n">
         <f aca="false">ROUND((D47-C47)*1440,0)</f>
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F47" s="12" t="s">
         <v>45</v>
       </c>
       <c r="G47" s="12" t="s">
-        <v>73</v>
+        <v>111</v>
       </c>
       <c r="H47" s="12" t="s">
         <v>114</v>
       </c>
       <c r="I47" s="12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J47" s="12" t="s">
-        <v>115</v>
+        <v>58</v>
       </c>
       <c r="K47" s="15" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="12" t="n">
         <v>3</v>
       </c>
@@ -4312,14 +4300,14 @@
         <v>46461</v>
       </c>
       <c r="C48" s="14" t="n">
-        <v>0.572916666666667</v>
+        <v>0.611111111111111</v>
       </c>
       <c r="D48" s="14" t="n">
-        <v>0.604166666666667</v>
+        <v>0.631944444444444</v>
       </c>
       <c r="E48" s="12" t="n">
         <f aca="false">ROUND((D48-C48)*1440,0)</f>
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="F48" s="12" t="s">
         <v>55</v>
@@ -4330,7 +4318,7 @@
       <c r="H48" s="12"/>
       <c r="I48" s="12"/>
       <c r="J48" s="12" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="K48" s="15" t="s">
         <v>44</v>
@@ -4345,14 +4333,14 @@
         <v>46461</v>
       </c>
       <c r="C49" s="14" t="n">
-        <v>0.604166666666667</v>
+        <v>0.631944444444444</v>
       </c>
       <c r="D49" s="14" t="n">
-        <v>0.611111111111111</v>
+        <v>0.642361111111111</v>
       </c>
       <c r="E49" s="12" t="n">
         <f aca="false">ROUND((D49-C49)*1440,0)</f>
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F49" s="12" t="s">
         <v>45</v>
@@ -4361,13 +4349,13 @@
         <v>114</v>
       </c>
       <c r="H49" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="I49" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="J49" s="12" t="s">
         <v>117</v>
-      </c>
-      <c r="I49" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="J49" s="12" t="s">
-        <v>58</v>
       </c>
       <c r="K49" s="15" t="s">
         <v>44</v>
@@ -4382,20 +4370,20 @@
         <v>46461</v>
       </c>
       <c r="C50" s="14" t="n">
-        <v>0.611111111111111</v>
+        <v>0.642361111111111</v>
       </c>
       <c r="D50" s="14" t="n">
-        <v>0.631944444444444</v>
+        <v>0.6875</v>
       </c>
       <c r="E50" s="12" t="n">
         <f aca="false">ROUND((D50-C50)*1440,0)</f>
-        <v>30</v>
+        <v>65</v>
       </c>
       <c r="F50" s="12" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="G50" s="12" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H50" s="12"/>
       <c r="I50" s="12"/>
@@ -4415,29 +4403,29 @@
         <v>46461</v>
       </c>
       <c r="C51" s="14" t="n">
-        <v>0.631944444444444</v>
+        <v>0.6875</v>
       </c>
       <c r="D51" s="14" t="n">
-        <v>0.642361111111111</v>
+        <v>0.75</v>
       </c>
       <c r="E51" s="12" t="n">
         <f aca="false">ROUND((D51-C51)*1440,0)</f>
-        <v>15</v>
+        <v>90</v>
       </c>
       <c r="F51" s="12" t="s">
         <v>45</v>
       </c>
       <c r="G51" s="12" t="s">
-        <v>117</v>
+        <v>71</v>
       </c>
       <c r="H51" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="I51" s="12" t="n">
+        <v>50</v>
+      </c>
+      <c r="J51" s="12" t="s">
         <v>119</v>
-      </c>
-      <c r="I51" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="J51" s="12" t="s">
-        <v>120</v>
       </c>
       <c r="K51" s="15" t="s">
         <v>44</v>
@@ -4452,25 +4440,25 @@
         <v>46461</v>
       </c>
       <c r="C52" s="14" t="n">
-        <v>0.642361111111111</v>
+        <v>0.75</v>
       </c>
       <c r="D52" s="14" t="n">
-        <v>0.6875</v>
+        <v>0.770833333333333</v>
       </c>
       <c r="E52" s="12" t="n">
         <f aca="false">ROUND((D52-C52)*1440,0)</f>
-        <v>65</v>
+        <v>30</v>
       </c>
       <c r="F52" s="12" t="s">
-        <v>121</v>
+        <v>49</v>
       </c>
       <c r="G52" s="12" t="s">
-        <v>119</v>
+        <v>47</v>
       </c>
       <c r="H52" s="12"/>
       <c r="I52" s="12"/>
       <c r="J52" s="12" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="K52" s="15" t="s">
         <v>44</v>
@@ -4485,163 +4473,163 @@
         <v>46461</v>
       </c>
       <c r="C53" s="14" t="n">
-        <v>0.6875</v>
+        <v>0.770833333333333</v>
       </c>
       <c r="D53" s="14" t="n">
-        <v>0.75</v>
+        <v>0.833333333333333</v>
       </c>
       <c r="E53" s="12" t="n">
         <f aca="false">ROUND((D53-C53)*1440,0)</f>
         <v>90</v>
       </c>
       <c r="F53" s="12" t="s">
-        <v>45</v>
+        <v>66</v>
       </c>
       <c r="G53" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="H53" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="I53" s="12" t="n">
-        <v>50</v>
-      </c>
+      <c r="H53" s="12"/>
+      <c r="I53" s="12"/>
       <c r="J53" s="12" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="K53" s="15" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="12" t="n">
+      <c r="A54" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="B54" s="13" t="n">
+      <c r="B54" s="17" t="n">
         <f aca="false">Overview!$B$3+A54-1</f>
         <v>46461</v>
       </c>
-      <c r="C54" s="14" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="D54" s="14" t="n">
-        <v>0.770833333333333</v>
-      </c>
-      <c r="E54" s="12" t="n">
+      <c r="C54" s="18" t="n">
+        <v>0.833333333333333</v>
+      </c>
+      <c r="D54" s="18" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="E54" s="16" t="n">
         <f aca="false">ROUND((D54-C54)*1440,0)</f>
+        <v>60</v>
+      </c>
+      <c r="F54" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="G54" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="H54" s="16"/>
+      <c r="I54" s="16"/>
+      <c r="J54" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="K54" s="19" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="B55" s="17" t="n">
+        <f aca="false">Overview!$B$3+A55-1</f>
+        <v>46462</v>
+      </c>
+      <c r="C55" s="18" t="n">
+        <v>0.3125</v>
+      </c>
+      <c r="D55" s="18" t="n">
+        <v>0.354166666666667</v>
+      </c>
+      <c r="E55" s="16" t="n">
+        <f aca="false">ROUND((D55-C55)*1440,0)</f>
+        <v>60</v>
+      </c>
+      <c r="F55" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="G55" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="H55" s="16"/>
+      <c r="I55" s="16"/>
+      <c r="J55" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="K55" s="19" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B56" s="13" t="n">
+        <f aca="false">Overview!$B$3+A56-1</f>
+        <v>46462</v>
+      </c>
+      <c r="C56" s="14" t="n">
+        <v>0.354166666666667</v>
+      </c>
+      <c r="D56" s="14" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="E56" s="12" t="n">
+        <f aca="false">ROUND((D56-C56)*1440,0)</f>
         <v>30</v>
       </c>
-      <c r="F54" s="12" t="s">
+      <c r="F56" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="G54" s="12" t="s">
+      <c r="G56" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="H54" s="12"/>
-      <c r="I54" s="12"/>
-      <c r="J54" s="12" t="s">
-        <v>124</v>
-      </c>
-      <c r="K54" s="15" t="s">
+      <c r="H56" s="12"/>
+      <c r="I56" s="12"/>
+      <c r="J56" s="12" t="s">
+        <v>122</v>
+      </c>
+      <c r="K56" s="15" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="B55" s="13" t="n">
-        <f aca="false">Overview!$B$3+A55-1</f>
-        <v>46461</v>
-      </c>
-      <c r="C55" s="14" t="n">
-        <v>0.770833333333333</v>
-      </c>
-      <c r="D55" s="14" t="n">
-        <v>0.833333333333333</v>
-      </c>
-      <c r="E55" s="12" t="n">
-        <f aca="false">ROUND((D55-C55)*1440,0)</f>
-        <v>90</v>
-      </c>
-      <c r="F55" s="12" t="s">
-        <v>90</v>
-      </c>
-      <c r="G55" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="H55" s="12"/>
-      <c r="I55" s="12"/>
-      <c r="J55" s="12" t="s">
-        <v>125</v>
-      </c>
-      <c r="K55" s="15" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="16" t="n">
-        <v>3</v>
-      </c>
-      <c r="B56" s="17" t="n">
-        <f aca="false">Overview!$B$3+A56-1</f>
-        <v>46461</v>
-      </c>
-      <c r="C56" s="18" t="n">
-        <v>0.833333333333333</v>
-      </c>
-      <c r="D56" s="18" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="E56" s="16" t="n">
-        <f aca="false">ROUND((D56-C56)*1440,0)</f>
-        <v>60</v>
-      </c>
-      <c r="F56" s="16" t="s">
-        <v>70</v>
-      </c>
-      <c r="G56" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="H56" s="16"/>
-      <c r="I56" s="16"/>
-      <c r="J56" s="16" t="s">
-        <v>70</v>
-      </c>
-      <c r="K56" s="19" t="s">
-        <v>44</v>
-      </c>
-    </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="16" t="n">
+      <c r="A57" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="B57" s="17" t="n">
+      <c r="B57" s="13" t="n">
         <f aca="false">Overview!$B$3+A57-1</f>
         <v>46462</v>
       </c>
-      <c r="C57" s="18" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="D57" s="18" t="n">
-        <v>0.354166666666667</v>
-      </c>
-      <c r="E57" s="16" t="n">
+      <c r="C57" s="14" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="D57" s="14" t="n">
+        <v>0.388888888888889</v>
+      </c>
+      <c r="E57" s="12" t="n">
         <f aca="false">ROUND((D57-C57)*1440,0)</f>
-        <v>60</v>
-      </c>
-      <c r="F57" s="16" t="s">
-        <v>71</v>
-      </c>
-      <c r="G57" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="H57" s="16"/>
-      <c r="I57" s="16"/>
-      <c r="J57" s="16" t="s">
-        <v>71</v>
-      </c>
-      <c r="K57" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="F57" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="G57" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="H57" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="I57" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="J57" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="K57" s="15" t="s">
         <v>44</v>
       </c>
     </row>
@@ -4654,107 +4642,37 @@
         <v>46462</v>
       </c>
       <c r="C58" s="14" t="n">
-        <v>0.354166666666667</v>
+        <v>0.388888888888889</v>
       </c>
       <c r="D58" s="14" t="n">
-        <v>0.375</v>
+        <v>0.40625</v>
       </c>
       <c r="E58" s="12" t="n">
         <f aca="false">ROUND((D58-C58)*1440,0)</f>
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F58" s="12" t="s">
-        <v>49</v>
+        <v>124</v>
       </c>
       <c r="G58" s="12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H58" s="12"/>
       <c r="I58" s="12"/>
       <c r="J58" s="12" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="K58" s="15" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="B59" s="13" t="n">
-        <f aca="false">Overview!$B$3+A59-1</f>
-        <v>46462</v>
-      </c>
-      <c r="C59" s="14" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="D59" s="14" t="n">
-        <v>0.388888888888889</v>
-      </c>
-      <c r="E59" s="12" t="n">
-        <f aca="false">ROUND((D59-C59)*1440,0)</f>
-        <v>20</v>
-      </c>
-      <c r="F59" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="G59" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="H59" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="I59" s="12" t="n">
-        <v>7</v>
-      </c>
-      <c r="J59" s="12" t="s">
-        <v>127</v>
-      </c>
-      <c r="K59" s="15" t="s">
-        <v>44</v>
-      </c>
-    </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="B60" s="13" t="n">
-        <f aca="false">Overview!$B$3+A60-1</f>
-        <v>46462</v>
-      </c>
-      <c r="C60" s="14" t="n">
-        <v>0.388888888888889</v>
-      </c>
-      <c r="D60" s="14" t="n">
-        <v>0.40625</v>
-      </c>
-      <c r="E60" s="12" t="n">
-        <f aca="false">ROUND((D60-C60)*1440,0)</f>
-        <v>25</v>
-      </c>
-      <c r="F60" s="12" t="s">
-        <v>128</v>
-      </c>
-      <c r="G60" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="H60" s="12"/>
-      <c r="I60" s="12"/>
-      <c r="J60" s="12" t="s">
-        <v>129</v>
-      </c>
-      <c r="K60" s="15" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="5" t="s">
-        <v>130</v>
+      <c r="A60" s="5" t="s">
+        <v>126</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:K60"/>
+  <autoFilter ref="A4:K58"/>
   <hyperlinks>
     <hyperlink ref="K5" r:id="rId1" display="Open map"/>
     <hyperlink ref="K6" r:id="rId2" display="Open map"/>
@@ -4810,8 +4728,6 @@
     <hyperlink ref="K56" r:id="rId52" display="Open map"/>
     <hyperlink ref="K57" r:id="rId53" display="Open map"/>
     <hyperlink ref="K58" r:id="rId54" display="Open map"/>
-    <hyperlink ref="K59" r:id="rId55" display="Open map"/>
-    <hyperlink ref="K60" r:id="rId56" display="Open map"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -4820,7 +4736,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId57"/>
+  <drawing r:id="rId55"/>
 </worksheet>
 </file>
 
@@ -4840,7 +4756,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4848,13 +4764,13 @@
         <v>5</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4865,7 +4781,7 @@
         <v>51</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="D4" s="12" t="s">
         <v>52</v>
@@ -4876,10 +4792,10 @@
         <v>1</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D5" s="12" t="s">
         <v>52</v>
@@ -4890,10 +4806,10 @@
         <v>2</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="D6" s="12" t="s">
         <v>52</v>
@@ -4907,10 +4823,10 @@
         <v>51</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4918,13 +4834,13 @@
         <v>2</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4932,13 +4848,13 @@
         <v>3</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4949,10 +4865,10 @@
         <v>51</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4960,10 +4876,10 @@
         <v>3</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="D11" s="12" t="s">
         <v>52</v>
@@ -4974,10 +4890,10 @@
         <v>4</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="D12" s="12" t="s">
         <v>52</v>
@@ -5008,112 +4924,112 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="12" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
     </row>
   </sheetData>
@@ -5143,184 +5059,184 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="12" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D2" s="12" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="12" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
     </row>
   </sheetData>
@@ -5348,194 +5264,194 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="12" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
+        <v>221</v>
+      </c>
+      <c r="B5" s="12" t="s">
         <v>225</v>
-      </c>
-      <c r="B5" s="12" t="s">
-        <v>229</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="12" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="12" t="s">
+        <v>231</v>
+      </c>
+      <c r="B14" s="12" t="s">
         <v>235</v>
-      </c>
-      <c r="B14" s="12" t="s">
-        <v>239</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="12" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="12" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="12" t="s">
+        <v>238</v>
+      </c>
+      <c r="B20" s="12" t="s">
         <v>242</v>
-      </c>
-      <c r="B20" s="12" t="s">
-        <v>246</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="12" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="12" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="12" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
     </row>
   </sheetData>
@@ -5566,221 +5482,221 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="11" t="s">
+        <v>249</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>250</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>251</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>252</v>
+      </c>
+      <c r="E3" s="11" t="s">
         <v>253</v>
-      </c>
-      <c r="B3" s="11" t="s">
-        <v>254</v>
-      </c>
-      <c r="C3" s="11" t="s">
-        <v>255</v>
-      </c>
-      <c r="D3" s="11" t="s">
-        <v>256</v>
-      </c>
-      <c r="E3" s="11" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="D4" s="12"/>
       <c r="E4" s="24"/>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="E5" s="24"/>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="E6" s="24"/>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="D7" s="12"/>
       <c r="E7" s="24"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="D8" s="12"/>
       <c r="E8" s="24"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="D9" s="12"/>
       <c r="E9" s="24"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="D10" s="12"/>
       <c r="E10" s="24"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="D11" s="12"/>
       <c r="E11" s="24"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="12" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="D12" s="12"/>
       <c r="E12" s="24"/>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="D13" s="12"/>
       <c r="E13" s="24"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="12" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="D14" s="12"/>
       <c r="E14" s="24"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="12" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="D15" s="12"/>
       <c r="E15" s="24"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="12" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="D16" s="12"/>
       <c r="E16" s="24"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="D17" s="12"/>
       <c r="E17" s="24"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="D18" s="12"/>
       <c r="E18" s="24"/>
@@ -5810,146 +5726,146 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="12" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
+        <v>289</v>
+      </c>
+      <c r="B5" s="12" t="s">
         <v>293</v>
-      </c>
-      <c r="B5" s="12" t="s">
-        <v>297</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="12" t="s">
+        <v>297</v>
+      </c>
+      <c r="B12" s="12" t="s">
         <v>301</v>
-      </c>
-      <c r="B12" s="12" t="s">
-        <v>305</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="12" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="12" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="12" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
     </row>
   </sheetData>
@@ -5977,90 +5893,90 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="12" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Aarti at the Holy Cave arranged once (Day 2 evening or Day 3 morning, as allotted)
Updates brochures, posters, yatri itineraries, Excel plans and SQL content.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A4yYiJq592wzPacq5vAVkN
</commit_message>
<xml_diff>
--- a/docs/itineraries/vaishno-devi-helicopter-4d-plan.xlsx
+++ b/docs/itineraries/vaishno-devi-helicopter-4d-plan.xlsx
@@ -127,7 +127,7 @@
     <t xml:space="preserve">Price</t>
   </si>
   <si>
-    <t xml:space="preserve">Highlights: Evening &amp; Morning Atka Aarti at the Holy Cave (main temple), arranged for the group so yatris spend more time before Mata Rani; Banganga darshan on Day 3.</t>
+    <t xml:space="preserve">Highlights: Atka Aarti at the Holy Cave, arranged once for the group (evening or morning, as allotted by the Shrine Board), so yatris spend more time before Mata Rani; Banganga darshan on Day 3.</t>
   </si>
   <si>
     <t xml:space="preserve">3N/4D: ₹50,000 per person + 5% GST, excluding flight charges</t>
@@ -316,13 +316,13 @@
     <t xml:space="preserve">Aarti</t>
   </si>
   <si>
-    <t xml:space="preserve">Evening Atka Aarti at the Holy Cave (main temple) – Aarti passes arranged by the organisers so yatris sit before Mata Rani for the full Aarti</t>
+    <t xml:space="preserve">Atka Aarti at the Holy Cave (main temple), arranged once for the group – this evening or tomorrow morning, as allotted by the Shrine Board; otherwise kirtan and japa</t>
   </si>
   <si>
     <t xml:space="preserve">Wake-up, bath, get ready</t>
   </si>
   <si>
-    <t xml:space="preserve">Morning Atka Aarti at the Holy Cave (main temple) – arranged by the organisers; more time before Mata Rani</t>
+    <t xml:space="preserve">Morning Atka Aarti at the Holy Cave if this is our allotted slot; otherwise japa and early darshan</t>
   </si>
   <si>
     <t xml:space="preserve">Rest, pack small bag</t>
@@ -421,7 +421,7 @@
     <t xml:space="preserve">Farewell – Jai Mata Di! (return flights after 14:00)</t>
   </si>
   <si>
-    <t xml:space="preserve">Legend: yellow rows = meals; peach rows = highlights (Evening &amp; Morning Atka Aarti, Banganga darshan); blue rows = helicopter / battery car / ropeway.</t>
+    <t xml:space="preserve">Legend: yellow rows = meals; peach rows = highlights (both possible Atka Aarti slots – the group gets one, as allotted by the Shrine Board; Banganga darshan); blue rows = helicopter / battery car / ropeway.</t>
   </si>
   <si>
     <t xml:space="preserve">Meal plan (all pure-veg)</t>
@@ -496,7 +496,7 @@
     <t xml:space="preserve">Night at Bhawan</t>
   </si>
   <si>
-    <t xml:space="preserve">Both Evening and Morning Aarti; unhurried darshan</t>
+    <t xml:space="preserve">Atka Aarti at the Holy Cave, arranged once for the group (evening or morning, as allotted by the Shrine Board); unhurried darshan</t>
   </si>
   <si>
     <t xml:space="preserve">Shared, basic rooms; limited supply</t>
@@ -613,7 +613,7 @@
     <t xml:space="preserve">Book on SMVDSB portal as soon as dates are fixed</t>
   </si>
   <si>
-    <t xml:space="preserve">Darshan Day 2 evening, return to Jammu same night; Morning Aarti dropped</t>
+    <t xml:space="preserve">Darshan Day 2 evening, return to Jammu same night; Atka Aarti only if the evening slot is allotted</t>
   </si>
   <si>
     <t xml:space="preserve">Long darshan queues</t>
@@ -859,7 +859,7 @@
     <t xml:space="preserve">Book Bhawan accommodation Day 2 night</t>
   </si>
   <si>
-    <t xml:space="preserve">Book Atka Aarti passes for the Evening &amp; Morning Atka Aarti at the Holy Cave (main temple)</t>
+    <t xml:space="preserve">Book Atka Aarti passes: Atka Aarti at the Holy Cave, arranged once for the group (evening or morning, as allotted by the Shrine Board)</t>
   </si>
   <si>
     <t xml:space="preserve">Arranged for the group so yatris spend more time before Mata Rani</t>
@@ -1267,7 +1267,7 @@
     <t xml:space="preserve">Bhairon ropeway</t>
   </si>
   <si>
-    <t xml:space="preserve">Atka Aarti passes – Evening &amp; Morning Atka Aarti at the Holy Cave, arranged for the group</t>
+    <t xml:space="preserve">Atka Aarti passes – Atka Aarti at the Holy Cave, arranged once for the group (evening or morning, as allotted by the Shrine Board)</t>
   </si>
   <si>
     <t xml:space="preserve">Vehicles, 4 days (149 km + waiting)</t>
@@ -1318,7 +1318,7 @@
     <t xml:space="preserve">Bhawan accommodation booked for Day 2 night</t>
   </si>
   <si>
-    <t xml:space="preserve">Atka Aarti passes – availability and booking window</t>
+    <t xml:space="preserve">Atka Aarti passes – booking window, and which slot (Day 2 evening or Day 3 morning) the Shrine Board allots</t>
   </si>
   <si>
     <t xml:space="preserve">Bhairon ropeway tickets; Sanjichhat → Bhawan battery car</t>
@@ -2765,7 +2765,7 @@
       </c>
       <c r="B5" s="28"/>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
         <v>427</v>
       </c>
@@ -3734,7 +3734,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="24" t="n">
         <v>2</v>
       </c>
@@ -5080,7 +5080,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
         <v>152</v>
       </c>

</xml_diff>